<commit_message>
SCRUM-101: кейси TC-009–TC-014 (КТ) у статусі draft — F-140, GUI-90, GUI-50, F-100, GUI-70
</commit_message>
<xml_diff>
--- a/docs/sprint3/test-cases.xlsx
+++ b/docs/sprint3/test-cases.xlsx
@@ -675,99 +675,419 @@
       <c r="N9" s="2" t="n"/>
     </row>
     <row r="10">
-      <c r="A10" s="2" t="n"/>
-      <c r="B10" s="2" t="n"/>
-      <c r="C10" s="2" t="n"/>
-      <c r="D10" s="2" t="n"/>
-      <c r="E10" s="2" t="n"/>
-      <c r="F10" s="2" t="n"/>
-      <c r="G10" s="2" t="n"/>
-      <c r="H10" s="2" t="n"/>
-      <c r="I10" s="2" t="n"/>
-      <c r="J10" s="2" t="n"/>
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TC-009</t>
+        </is>
+      </c>
+      <c r="B10" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">F-140, GUI-50</t>
+        </is>
+      </c>
+      <c r="C10" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Контактна форма: повідомлення з 49 символів (нижче межі) не надсилається</t>
+        </is>
+      </c>
+      <c r="D10" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Chrome 120 або новіший, вікно 1280×800; demo доступне (збірка 2026-10-11); обліковий запис не потрібен (звернення від анонімного відвідувача); дані лише вигадані.</t>
+        </is>
+      </c>
+      <c r="E10" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1. Відкрити https://practicesoftwaretesting.com/contact у Chrome (нова сесія).
+2. У поле «Your first name» ввести: Test
+3. У поле «Your last name» ввести: Tester
+4. У поле «Your email» ввести: tester.tc009@example.com
+5. У списку «Select a subject» вибрати: Customer service
+6. У поле «Message» ввести 49 символів: abcdefghijabcdefghijabcdefghijabcdefghijabcdefghi
+7. Натиснути «Send».
+8. Закрити вкладку.</t>
+        </is>
+      </c>
+      <c r="F10" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Після кроку 1: відкрито сторінку «Contact», усі поля порожні.
+Після кроку 6: у полі «Message» 49 символів.
+Після кроку 7: форму не надіслано, сторінка «Contact» залишається відкритою; під полем «Message» текстове повідомлення про помилку: довжина повідомлення має бути не менше 50 символів (F-140, GUI-50); під іншими полями повідомлень про помилки немає; повідомлення про прийняття звернення над формою відсутнє.</t>
+        </is>
+      </c>
+      <c r="G10" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">High</t>
+        </is>
+      </c>
+      <c r="H10" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">негативний</t>
+        </is>
+      </c>
+      <c r="I10" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Допустима довжина повідомлення 50–250 (F-140). 49 — на 1 менше за нижню межу, клас недопустимих значень. Решта полів валідні, тому відхилення можливе лише через довжину.</t>
+        </is>
+      </c>
+      <c r="J10" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Горбонос Олександра</t>
+        </is>
+      </c>
       <c r="K10" s="2" t="n"/>
       <c r="L10" s="2" t="n"/>
-      <c r="M10" s="2" t="n"/>
+      <c r="M10" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">draft</t>
+        </is>
+      </c>
       <c r="N10" s="2" t="n"/>
     </row>
     <row r="11">
-      <c r="A11" s="2" t="n"/>
-      <c r="B11" s="2" t="n"/>
-      <c r="C11" s="2" t="n"/>
-      <c r="D11" s="2" t="n"/>
-      <c r="E11" s="2" t="n"/>
-      <c r="F11" s="2" t="n"/>
-      <c r="G11" s="2" t="n"/>
-      <c r="H11" s="2" t="n"/>
-      <c r="I11" s="2" t="n"/>
-      <c r="J11" s="2" t="n"/>
+      <c r="A11" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TC-010</t>
+        </is>
+      </c>
+      <c r="B11" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">F-140, GUI-90</t>
+        </is>
+      </c>
+      <c r="C11" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Контактна форма: повідомлення з 50 символів (нижня межа) приймається, показано підтвердження</t>
+        </is>
+      </c>
+      <c r="D11" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Chrome 120 або новіший, вікно 1280×800; demo доступне (збірка 2026-10-11); обліковий запис не потрібен (звернення від анонімного відвідувача); дані лише вигадані.</t>
+        </is>
+      </c>
+      <c r="E11" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1. Відкрити https://practicesoftwaretesting.com/contact у Chrome (нова сесія).
+2. У поле «Your first name» ввести: Test
+3. У поле «Your last name» ввести: Tester
+4. У поле «Your email» ввести: tester.tc010@example.com
+5. У списку «Select a subject» вибрати: Customer service
+6. У поле «Message» ввести 50 символів: abcdefghijabcdefghijabcdefghijabcdefghijabcdefghij
+7. Натиснути «Send».
+8. Закрити вкладку.</t>
+        </is>
+      </c>
+      <c r="F11" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Після кроку 1: відкрито сторінку «Contact»; є поля імені, прізвища й адреси електронної пошти, розкривний список теми, багаторядкове поле «Message», елемент вибору файла «Attachment» і кнопка «Send» (GUI-90).
+Після кроку 6: у полі «Message» 50 символів.
+Після кроку 7: звернення прийнято; над формою виводиться повідомлення про прийняття звернення (F-140, GUI-90); повідомлень про помилки під полями немає.</t>
+        </is>
+      </c>
+      <c r="G11" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Medium</t>
+        </is>
+      </c>
+      <c r="H11" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">позитивний</t>
+        </is>
+      </c>
+      <c r="I11" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">50 — нижня межа допустимого діапазону 50–250 (перше допустиме значення). Вкладення не додається, щоб один кейс відповідав одному набору даних.</t>
+        </is>
+      </c>
+      <c r="J11" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Горбонос Олександра</t>
+        </is>
+      </c>
       <c r="K11" s="2" t="n"/>
       <c r="L11" s="2" t="n"/>
-      <c r="M11" s="2" t="n"/>
+      <c r="M11" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">draft</t>
+        </is>
+      </c>
       <c r="N11" s="2" t="n"/>
     </row>
     <row r="12">
-      <c r="A12" s="2" t="n"/>
-      <c r="B12" s="2" t="n"/>
-      <c r="C12" s="2" t="n"/>
-      <c r="D12" s="2" t="n"/>
-      <c r="E12" s="2" t="n"/>
-      <c r="F12" s="2" t="n"/>
-      <c r="G12" s="2" t="n"/>
-      <c r="H12" s="2" t="n"/>
-      <c r="I12" s="2" t="n"/>
-      <c r="J12" s="2" t="n"/>
+      <c r="A12" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TC-011</t>
+        </is>
+      </c>
+      <c r="B12" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">F-140</t>
+        </is>
+      </c>
+      <c r="C12" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Контактна форма: повідомлення з 250 символів (верхня межа) приймається</t>
+        </is>
+      </c>
+      <c r="D12" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Chrome 120 або новіший, вікно 1280×800; demo доступне (збірка 2026-10-11); обліковий запис не потрібен (звернення від анонімного відвідувача); дані лише вигадані.</t>
+        </is>
+      </c>
+      <c r="E12" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1. Відкрити https://practicesoftwaretesting.com/contact у Chrome (нова сесія).
+2. У поле «Your first name» ввести: Test
+3. У поле «Your last name» ввести: Tester
+4. У поле «Your email» ввести: tester.tc011@example.com
+5. У списку «Select a subject» вибрати: Customer service
+6. У поле «Message» ввести 250 символів: abcdefghijabcdefghijabcdefghijabcdefghijabcdefghijabcdefghijabcdefghijabcdefghijabcdefghijabcdefghijabcdefghijabcdefghijabcdefghijabcdefghijabcdefghijabcdefghijabcdefghijabcdefghijabcdefghijabcdefghijabcdefghijabcdefghijabcdefghijabcdefghijabcdefghij
+7. Натиснути «Send».
+8. Закрити вкладку.</t>
+        </is>
+      </c>
+      <c r="F12" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Після кроку 1: відкрито сторінку «Contact», усі поля порожні.
+Після кроку 6: у полі «Message» 250 символів.
+Після кроку 7: звернення прийнято; над формою виводиться повідомлення про прийняття звернення (F-140); повідомлень про помилки під полями немає.</t>
+        </is>
+      </c>
+      <c r="G12" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Medium</t>
+        </is>
+      </c>
+      <c r="H12" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">позитивний</t>
+        </is>
+      </c>
+      <c r="I12" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">250 — верхня межа допустимого діапазону 50–250 (останнє допустиме значення).</t>
+        </is>
+      </c>
+      <c r="J12" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Горбонос Олександра</t>
+        </is>
+      </c>
       <c r="K12" s="2" t="n"/>
       <c r="L12" s="2" t="n"/>
-      <c r="M12" s="2" t="n"/>
+      <c r="M12" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">draft</t>
+        </is>
+      </c>
       <c r="N12" s="2" t="n"/>
     </row>
     <row r="13">
-      <c r="A13" s="2" t="n"/>
-      <c r="B13" s="2" t="n"/>
-      <c r="C13" s="2" t="n"/>
-      <c r="D13" s="2" t="n"/>
-      <c r="E13" s="2" t="n"/>
-      <c r="F13" s="2" t="n"/>
-      <c r="G13" s="2" t="n"/>
-      <c r="H13" s="2" t="n"/>
-      <c r="I13" s="2" t="n"/>
-      <c r="J13" s="2" t="n"/>
+      <c r="A13" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TC-012</t>
+        </is>
+      </c>
+      <c r="B13" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">F-140, GUI-50</t>
+        </is>
+      </c>
+      <c r="C13" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Контактна форма: повідомлення з 251 символу (вище межі) не надсилається</t>
+        </is>
+      </c>
+      <c r="D13" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Chrome 120 або новіший, вікно 1280×800; demo доступне (збірка 2026-10-11); обліковий запис не потрібен (звернення від анонімного відвідувача); дані лише вигадані.</t>
+        </is>
+      </c>
+      <c r="E13" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1. Відкрити https://practicesoftwaretesting.com/contact у Chrome (нова сесія).
+2. У поле «Your first name» ввести: Test
+3. У поле «Your last name» ввести: Tester
+4. У поле «Your email» ввести: tester.tc012@example.com
+5. У списку «Select a subject» вибрати: Customer service
+6. У поле «Message» ввести 251 символ: abcdefghijabcdefghijabcdefghijabcdefghijabcdefghijabcdefghijabcdefghijabcdefghijabcdefghijabcdefghijabcdefghijabcdefghijabcdefghijabcdefghijabcdefghijabcdefghijabcdefghijabcdefghijabcdefghijabcdefghijabcdefghijabcdefghijabcdefghijabcdefghijabcdefghija
+7. Натиснути «Send».
+8. Закрити вкладку.</t>
+        </is>
+      </c>
+      <c r="F13" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Після кроку 1: відкрито сторінку «Contact», усі поля порожні.
+Після кроку 6: у полі «Message» 251 символ.
+Після кроку 7: форму не надіслано, сторінка «Contact» залишається відкритою; під полем «Message» текстове повідомлення про помилку: довжина повідомлення має бути не більше 250 символів (F-140, GUI-50); під іншими полями повідомлень про помилки немає; повідомлення про прийняття звернення над формою відсутнє.</t>
+        </is>
+      </c>
+      <c r="G13" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">High</t>
+        </is>
+      </c>
+      <c r="H13" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">негативний</t>
+        </is>
+      </c>
+      <c r="I13" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">251 — на 1 більше за верхню межу діапазону 50–250, клас недопустимих значень. Решта полів валідні.</t>
+        </is>
+      </c>
+      <c r="J13" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Горбонос Олександра</t>
+        </is>
+      </c>
       <c r="K13" s="2" t="n"/>
       <c r="L13" s="2" t="n"/>
-      <c r="M13" s="2" t="n"/>
+      <c r="M13" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">draft</t>
+        </is>
+      </c>
       <c r="N13" s="2" t="n"/>
     </row>
     <row r="14">
-      <c r="A14" s="2" t="n"/>
-      <c r="B14" s="2" t="n"/>
-      <c r="C14" s="2" t="n"/>
-      <c r="D14" s="2" t="n"/>
-      <c r="E14" s="2" t="n"/>
-      <c r="F14" s="2" t="n"/>
-      <c r="G14" s="2" t="n"/>
-      <c r="H14" s="2" t="n"/>
-      <c r="I14" s="2" t="n"/>
-      <c r="J14" s="2" t="n"/>
+      <c r="A14" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TC-013</t>
+        </is>
+      </c>
+      <c r="B14" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">F-140, GUI-50</t>
+        </is>
+      </c>
+      <c r="C14" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Контактна форма: вкладення недопустимого формату (.png) блокує надсилання</t>
+        </is>
+      </c>
+      <c r="D14" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Chrome 120 або новіший, вікно 1280×800; demo доступне (збірка 2026-10-11); обліковий запис не потрібен (звернення від анонімного відвідувача); дані лише вигадані. На комп'ютері є файл note.png розміром до 100 КБ з вигаданим зображенням без особистих даних.</t>
+        </is>
+      </c>
+      <c r="E14" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1. Відкрити https://practicesoftwaretesting.com/contact у Chrome (нова сесія).
+2. У поле «Your first name» ввести: Test
+3. У поле «Your last name» ввести: Tester
+4. У поле «Your email» ввести: tester.tc013@example.com
+5. У списку «Select a subject» вибрати: Customer service
+6. У поле «Message» ввести 50 символів: abcdefghijabcdefghijabcdefghijabcdefghijabcdefghij
+7. У полі «Attachment» натиснути кнопку вибору файла й обрати файл note.png.
+8. Натиснути «Send».
+9. Закрити вкладку.</t>
+        </is>
+      </c>
+      <c r="F14" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Після кроку 1: відкрито сторінку «Contact», усі поля порожні.
+Після кроку 6: у полі «Message» 50 символів (допустима довжина).
+Після кроку 7: у полі «Attachment» відображається назва файла note.png.
+Після кроку 8: форму не надіслано, сторінка «Contact» залишається відкритою; біля поля «Attachment» текстове повідомлення про помилку: файл недопустимий (F-140, GUI-50); повідомлення про прийняття звернення над формою відсутнє.</t>
+        </is>
+      </c>
+      <c r="G14" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">High</t>
+        </is>
+      </c>
+      <c r="H14" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">негативний</t>
+        </is>
+      </c>
+      <c r="I14" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Файл .png — недопустимий формат (допускається один файл .txt до 500 КБ, F-140). Довжина повідомлення 50 і решта полів валідні, тож єдина причина відхилення — вкладення.</t>
+        </is>
+      </c>
+      <c r="J14" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Горбонос Олександра</t>
+        </is>
+      </c>
       <c r="K14" s="2" t="n"/>
       <c r="L14" s="2" t="n"/>
-      <c r="M14" s="2" t="n"/>
+      <c r="M14" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">draft</t>
+        </is>
+      </c>
       <c r="N14" s="2" t="n"/>
     </row>
     <row r="15">
-      <c r="A15" s="2" t="n"/>
-      <c r="B15" s="2" t="n"/>
-      <c r="C15" s="2" t="n"/>
-      <c r="D15" s="2" t="n"/>
-      <c r="E15" s="2" t="n"/>
-      <c r="F15" s="2" t="n"/>
-      <c r="G15" s="2" t="n"/>
-      <c r="H15" s="2" t="n"/>
-      <c r="I15" s="2" t="n"/>
-      <c r="J15" s="2" t="n"/>
+      <c r="A15" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TC-014</t>
+        </is>
+      </c>
+      <c r="B15" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">F-100, GUI-70</t>
+        </is>
+      </c>
+      <c r="C15" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Крок «Cart»: зміна кількості перераховує «Total», видалення рядка показує порожній кошик</t>
+        </is>
+      </c>
+      <c r="D15" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Chrome 120 або новіший, вікно 1280×800; demo доступне (збірка 2026-10-11); кошик порожній (нова сесія); обліковий запис не потрібен; у каталозі є товар «Combination Pliers» з ціною $14.15.</t>
+        </is>
+      </c>
+      <c r="E15" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1. Відкрити https://practicesoftwaretesting.com/ у Chrome (нова сесія).
+2. У каталозі натиснути картку «Combination Pliers».
+3. На сторінці товару натиснути «Add to cart».
+4. У шапці натиснути піктограму кошика.
+5. У полі кількості рядка «Combination Pliers» замінити значення 1 на 3.
+6. Перемістити фокус з поля кількості, натиснувши Tab.
+7. Натиснути піктограму видалення в рядку «Combination Pliers».
+8. Закрити вкладку.</t>
+        </is>
+      </c>
+      <c r="F15" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Після кроку 4: відкрито крок «Cart»; таблиця має колонки «Item», «Quantity» (поле для редагування), «Price», «Total» і піктограму видалення; єдиний рядок: «Combination Pliers», кількість 1, ціна $14.15, сума рядка $14.15; під таблицею підсумок «Total» $14.15 і кнопка «Proceed to checkout» (GUI-70).
+Після кроку 6: у рядку кількість 3, сума рядка $42.45, підсумок «Total» $42.45; сторінку не перезавантажено (F-100).
+Після кроку 7: рядок «Combination Pliers» вилучено; таблиці немає; замість неї текстове повідомлення про порожній кошик (F-100, GUI-70).</t>
+        </is>
+      </c>
+      <c r="G15" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">High</t>
+        </is>
+      </c>
+      <c r="H15" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">позитивний</t>
+        </is>
+      </c>
+      <c r="I15" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Кількість 3 — типове значення допустимого класу 1–99; межі 0 / 1 / 99 / 100 перевіряють кейси TC-005–TC-008 (GUI-30). 14.15 × 3 = 42.45 — перевірка арифметики перерахунку.</t>
+        </is>
+      </c>
+      <c r="J15" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Горбонос Олександра</t>
+        </is>
+      </c>
       <c r="K15" s="2" t="n"/>
       <c r="L15" s="2" t="n"/>
-      <c r="M15" s="2" t="n"/>
+      <c r="M15" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">draft</t>
+        </is>
+      </c>
       <c r="N15" s="2" t="n"/>
     </row>
     <row r="16">

</xml_diff>

<commit_message>
SCRUM-107: зразок стилю — TC-001 (F-60), TC-002/TC-003 (GUI-30, граничні 99/100), TC-004 (F-20, негативний); статус draft, звірено з demo 25.10.2026
</commit_message>
<xml_diff>
--- a/docs/sprint3/test-cases.xlsx
+++ b/docs/sprint3/test-cases.xlsx
@@ -547,67 +547,283 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="2" t="n"/>
-      <c r="B2" s="2" t="n"/>
-      <c r="C2" s="2" t="n"/>
-      <c r="D2" s="2" t="n"/>
-      <c r="E2" s="2" t="n"/>
-      <c r="F2" s="2" t="n"/>
-      <c r="G2" s="2" t="n"/>
-      <c r="H2" s="2" t="n"/>
-      <c r="I2" s="2" t="n"/>
-      <c r="J2" s="2" t="n"/>
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>TC-001</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>F-60</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>Пошук товарів за частиною назви, введеною в нижньому регістрі, без входу</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>Chrome (поточна стабільна версія), нова сесія (вікно інкогніто), без входу. У каталозі є товари зі словом «Pliers» у назві (стан demo 25.10.2026: Combination Pliers, Pliers, Long Nose Pliers, Slip Joint Pliers).</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>1. Відкрити https://practicesoftwaretesting.com.
+2. У поле пошуку «Search» ввести pliers.
+3. Натиснути кнопку «Search».
+4. Переглянути назви всіх карток у списку результатів.
+5. Закрити вкладку.</t>
+        </is>
+      </c>
+      <c r="F2" s="2" t="inlineStr">
+        <is>
+          <t>1. Головна сторінка з каталогом карток, полем «Search» і кнопками «X» та «Search».
+2. У полі «Search» показано текст pliers.
+3. Список карток оновлено; результати під заголовком «Searched for: pliers».
+4. Кожна назва містить «pliers» без урахування регістру (наприклад, «Combination Pliers»); карток без цього слова немає.
+5. Вкладку закрито.</t>
+        </is>
+      </c>
+      <c r="G2" s="2" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="H2" s="2" t="inlineStr">
+        <is>
+          <t>позитивний</t>
+        </is>
+      </c>
+      <c r="I2" s="2" t="inlineStr">
+        <is>
+          <t>Клас «підрядок, що є в назвах товарів». Запит у нижньому регістрі, а в назвах — «Pliers» з великої літери: перевіряє умову F-60 «без урахування регістру літер».</t>
+        </is>
+      </c>
+      <c r="J2" s="2" t="inlineStr">
+        <is>
+          <t>Коротка К. (ТА)</t>
+        </is>
+      </c>
       <c r="K2" s="2" t="n"/>
       <c r="L2" s="2" t="n"/>
-      <c r="M2" s="2" t="n"/>
+      <c r="M2" s="2" t="inlineStr">
+        <is>
+          <t>draft</t>
+        </is>
+      </c>
       <c r="N2" s="2" t="n"/>
     </row>
     <row r="3">
-      <c r="A3" s="2" t="n"/>
-      <c r="B3" s="2" t="n"/>
-      <c r="C3" s="2" t="n"/>
-      <c r="D3" s="2" t="n"/>
-      <c r="E3" s="2" t="n"/>
-      <c r="F3" s="2" t="n"/>
-      <c r="G3" s="2" t="n"/>
-      <c r="H3" s="2" t="n"/>
-      <c r="I3" s="2" t="n"/>
-      <c r="J3" s="2" t="n"/>
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>TC-002</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>GUI-30</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>Додавання товару в кошик із кількістю 99 (верхня межа) без входу</t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t>Chrome (поточна стабільна версія), нова сесія (вікно інкогніто), без входу. Кошик порожній. Товар «Combination Pliers» є на першій сторінці каталогу і в наявності.</t>
+        </is>
+      </c>
+      <c r="E3" s="2" t="inlineStr">
+        <is>
+          <t>1. Відкрити https://practicesoftwaretesting.com.
+2. Натиснути на картку товару «Combination Pliers».
+3. У поле «Quantity» ввести 99 (замість значення 1).
+4. Натиснути кнопку «Add to cart».
+5. Натиснути піктограму кошика у верхньому меню.
+6. У рядку «Combination Pliers» натиснути червону кнопку видалення.
+7. Закрити вкладку.</t>
+        </is>
+      </c>
+      <c r="F3" s="2" t="inlineStr">
+        <is>
+          <t>1. Головна сторінка з каталогом; є картка «Combination Pliers».
+2. Сторінка товару «Combination Pliers»: ціна; поле «Quantity» зі значенням 1 і кнопками «−» та «+»; кнопка «Add to cart».
+3. У полі «Quantity» — 99; під полем повідомлень про помилку немає.
+4. Не пізніше ніж за 2 с — повідомлення «Product added to shopping cart.»; на піктограмі кошика в меню — 99.
+5. Крок «Cart»: один рядок «Combination Pliers», «Quantity» — 99, «Total» = 99 × ціна з кроку 2.
+6. Рядок видалено; замість таблиці — текстове повідомлення про порожній кошик (на demo 25.10.2026 — «The cart is empty. Nothing to display.»).
+7. Вкладку закрито.</t>
+        </is>
+      </c>
+      <c r="G3" s="2" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="H3" s="2" t="inlineStr">
+        <is>
+          <t>позитивний</t>
+        </is>
+      </c>
+      <c r="I3" s="2" t="inlineStr">
+        <is>
+          <t>Граничне значення: верхня межа діапазону 1–99 (GUI-30), клас «допустима кількість». Негативна пара — TC-003 (100).</t>
+        </is>
+      </c>
+      <c r="J3" s="2" t="inlineStr">
+        <is>
+          <t>Коротка К. (ТА)</t>
+        </is>
+      </c>
       <c r="K3" s="2" t="n"/>
       <c r="L3" s="2" t="n"/>
-      <c r="M3" s="2" t="n"/>
+      <c r="M3" s="2" t="inlineStr">
+        <is>
+          <t>draft</t>
+        </is>
+      </c>
       <c r="N3" s="2" t="n"/>
     </row>
     <row r="4">
-      <c r="A4" s="2" t="n"/>
-      <c r="B4" s="2" t="n"/>
-      <c r="C4" s="2" t="n"/>
-      <c r="D4" s="2" t="n"/>
-      <c r="E4" s="2" t="n"/>
-      <c r="F4" s="2" t="n"/>
-      <c r="G4" s="2" t="n"/>
-      <c r="H4" s="2" t="n"/>
-      <c r="I4" s="2" t="n"/>
-      <c r="J4" s="2" t="n"/>
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>TC-003</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>GUI-30</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>Спроба додати товар у кошик із кількістю 100 (більше верхньої межі) без входу</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>Chrome (поточна стабільна версія), нова сесія (вікно інкогніто), без входу. Кошик порожній. Товар «Combination Pliers» є на першій сторінці каталогу і в наявності.</t>
+        </is>
+      </c>
+      <c r="E4" s="2" t="inlineStr">
+        <is>
+          <t>1. Відкрити https://practicesoftwaretesting.com.
+2. Натиснути на картку товару «Combination Pliers».
+3. У поле «Quantity» ввести 100 (замість значення 1).
+4. Натиснути кнопку «Add to cart».
+5. В адресному рядку відкрити https://practicesoftwaretesting.com/checkout.
+6. Закрити вкладку.</t>
+        </is>
+      </c>
+      <c r="F4" s="2" t="inlineStr">
+        <is>
+          <t>1. Головна сторінка з каталогом; є картка «Combination Pliers».
+2. Сторінка товару «Combination Pliers»: поле «Quantity» зі значенням 1 і кнопками «−» та «+»; кнопка «Add to cart».
+3. У полі «Quantity» — 100.
+4. Товар не додано: повідомлення «Product added to shopping cart.» немає; піктограми кошика з лічильником у меню немає; під полем «Quantity» — текстове повідомлення про допустимі значення 1–99 (GUI-30, GUI-50).
+5. Крок «Cart»: текстове повідомлення про порожній кошик; рядка «Combination Pliers» немає.
+6. Вкладку закрито.</t>
+        </is>
+      </c>
+      <c r="G4" s="2" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="H4" s="2" t="inlineStr">
+        <is>
+          <t>негативний</t>
+        </is>
+      </c>
+      <c r="I4" s="2" t="inlineStr">
+        <is>
+          <t>Граничне значення: b+1 для діапазону 1–99 (GUI-30), клас «кількість більша за 99». Позитивна пара — TC-002 (99).</t>
+        </is>
+      </c>
+      <c r="J4" s="2" t="inlineStr">
+        <is>
+          <t>Коротка К. (ТА)</t>
+        </is>
+      </c>
       <c r="K4" s="2" t="n"/>
       <c r="L4" s="2" t="n"/>
-      <c r="M4" s="2" t="n"/>
+      <c r="M4" s="2" t="inlineStr">
+        <is>
+          <t>draft</t>
+        </is>
+      </c>
       <c r="N4" s="2" t="n"/>
     </row>
     <row r="5">
-      <c r="A5" s="2" t="n"/>
-      <c r="B5" s="2" t="n"/>
-      <c r="C5" s="2" t="n"/>
-      <c r="D5" s="2" t="n"/>
-      <c r="E5" s="2" t="n"/>
-      <c r="F5" s="2" t="n"/>
-      <c r="G5" s="2" t="n"/>
-      <c r="H5" s="2" t="n"/>
-      <c r="I5" s="2" t="n"/>
-      <c r="J5" s="2" t="n"/>
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>TC-004</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>F-20</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>Вхід із незареєстрованою адресою електронної пошти</t>
+        </is>
+      </c>
+      <c r="D5" s="2" t="inlineStr">
+        <is>
+          <t>Chrome (поточна стабільна версія), нова сесія (вікно інкогніто), без входу. Адреса shopline.ta.test@example.com на demo не зареєстрована.</t>
+        </is>
+      </c>
+      <c r="E5" s="2" t="inlineStr">
+        <is>
+          <t>1. Відкрити https://practicesoftwaretesting.com.
+2. Натиснути «Sign in» у верхньому меню.
+3. У поле «Email address» ввести shopline.ta.test@example.com.
+4. У поле «Password» ввести Test-pass1.
+5. Натиснути кнопку «Login».
+6. Закрити вкладку.</t>
+        </is>
+      </c>
+      <c r="F5" s="2" t="inlineStr">
+        <is>
+          <t>1. Головна сторінка з каталогом; у меню — «Sign in».
+2. Сторінка входу (адреса містить /auth/login): поля «Email address» і «Password», кнопка «Login».
+3. У полі «Email address» — shopline.ta.test@example.com.
+4. Символи пароля замасковано.
+5. Повідомлення «Invalid email or password»; адреса не змінилася (/auth/login); у меню — «Sign in» (сеанс не створено).
+6. Вкладку закрито.</t>
+        </is>
+      </c>
+      <c r="G5" s="2" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="H5" s="2" t="inlineStr">
+        <is>
+          <t>негативний</t>
+        </is>
+      </c>
+      <c r="I5" s="2" t="inlineStr">
+        <is>
+          <t>Клас «неправильна пара адреса — пароль» (F-20): вигадана незареєстрована адреса з домену example.com. Спільний обліковий запис customer@… не використано, щоб невдалі спроби входу не вплинули на інших користувачів demo (п. 5.4).</t>
+        </is>
+      </c>
+      <c r="J5" s="2" t="inlineStr">
+        <is>
+          <t>Коротка К. (ТА)</t>
+        </is>
+      </c>
       <c r="K5" s="2" t="n"/>
       <c r="L5" s="2" t="n"/>
-      <c r="M5" s="2" t="n"/>
+      <c r="M5" s="2" t="inlineStr">
+        <is>
+          <t>draft</t>
+        </is>
+      </c>
       <c r="N5" s="2" t="n"/>
     </row>
     <row r="6">

</xml_diff>

<commit_message>
SCRUM-113: кейси TC-015–TC-019 (ІТ) у статусі draft — F-20, GUI-60, GUI-10, F-110, GUI-40, F-120, F-30; звірено з demo (збірка v2.5 від 2026-10-11) 26.10.2026
</commit_message>
<xml_diff>
--- a/docs/sprint3/test-cases.xlsx
+++ b/docs/sprint3/test-cases.xlsx
@@ -771,83 +771,371 @@
       <c r="N15" s="2" t="n"/>
     </row>
     <row r="16">
-      <c r="A16" s="2" t="n"/>
-      <c r="B16" s="2" t="n"/>
-      <c r="C16" s="2" t="n"/>
-      <c r="D16" s="2" t="n"/>
-      <c r="E16" s="2" t="n"/>
-      <c r="F16" s="2" t="n"/>
-      <c r="G16" s="2" t="n"/>
-      <c r="H16" s="2" t="n"/>
-      <c r="I16" s="2" t="n"/>
-      <c r="J16" s="2" t="n"/>
+      <c r="A16" s="2" t="inlineStr">
+        <is>
+          <t>TC-015</t>
+        </is>
+      </c>
+      <c r="B16" s="2" t="inlineStr">
+        <is>
+          <t>F-20, GUI-60, GUI-10</t>
+        </is>
+      </c>
+      <c r="C16" s="2" t="inlineStr">
+        <is>
+          <t>Вхід зареєстрованого покупця з правильною парою адреса — пароль</t>
+        </is>
+      </c>
+      <c r="D16" s="2" t="inlineStr">
+        <is>
+          <t>Chrome 120 або новіший, вікно 1280×800; demo доступне (збірка v2.5 від 2026-10-11 за написом у підвалі сторінки; стан звірено 26.10.2026); нова сесія, без входу; спільний обліковий запис покупця customer@practicesoftwaretesting.com / welcome01 (SRS 1.1, розд. 2.2); пароль спільного облікового запису не змінювати (методичка, п. 5.4).</t>
+        </is>
+      </c>
+      <c r="E16" s="2" t="inlineStr">
+        <is>
+          <t>1. Відкрити https://practicesoftwaretesting.com у Chrome (нова сесія).
+2. Натиснути «Sign in» у верхньому меню.
+3. У поле «Email address» ввести: customer@practicesoftwaretesting.com
+4. У поле «Password» ввести: welcome01
+5. Натиснути кнопку «Login».
+6. Натиснути ім'я користувача у верхньому меню.
+7. У розкривному меню натиснути «Sign out».
+8. Закрити вкладку.</t>
+        </is>
+      </c>
+      <c r="F16" s="2" t="inlineStr">
+        <is>
+          <t>Після кроку 1: головна сторінка з каталогом; у шапці логотип, пункти «Home», «Categories», «Contact», «Sign in» і перемикач мови (GUI-10).
+Після кроку 2: сторінка входу (адреса містить /auth/login): заголовок «Login»; поля «Email address» і «Password» (з кнопкою показати / приховати пароль); кнопки «Login» і «Sign in with Google»; посилання «Register your account» і «Forgot your Password?» (GUI-60).
+Після кроку 3: у полі «Email address» — customer@practicesoftwaretesting.com.
+Після кроку 4: символи пароля замасковано.
+Після кроку 5: відкрито сторінку особистого кабінету, адреса містить /account (F-20); у шапці замість «Sign in» — ім'я користувача (GUI-10).
+Після кроку 6: розкривне меню з розділами кабінету і пунктом «Sign out» (GUI-10).
+Після кроку 7: сеанс завершено; у шапці знову «Sign in».
+Після кроку 8: вкладку закрито.</t>
+        </is>
+      </c>
+      <c r="G16" s="2" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="H16" s="2" t="inlineStr">
+        <is>
+          <t>позитивний</t>
+        </is>
+      </c>
+      <c r="I16" s="2" t="inlineStr">
+        <is>
+          <t>Клас «правильна пара адреса — пароль» (F-20). Дані — тестовий обліковий запис покупця з SRS 1.1 (розд. 2.2); вхід і вихід не змінюють даних облікового запису. Вихід на кроці 7 лишає demo в початковому стані для наступних кейсів. Негативні пари — TC-016 (зареєстрована адреса, неправильний пароль) і TC-004 (незареєстрована адреса).</t>
+        </is>
+      </c>
+      <c r="J16" s="2" t="inlineStr">
+        <is>
+          <t>Тимчак А. (ІТ)</t>
+        </is>
+      </c>
       <c r="K16" s="2" t="n"/>
       <c r="L16" s="2" t="n"/>
-      <c r="M16" s="2" t="n"/>
+      <c r="M16" s="2" t="inlineStr">
+        <is>
+          <t>draft</t>
+        </is>
+      </c>
       <c r="N16" s="2" t="n"/>
     </row>
     <row r="17">
-      <c r="A17" s="2" t="n"/>
-      <c r="B17" s="2" t="n"/>
-      <c r="C17" s="2" t="n"/>
-      <c r="D17" s="2" t="n"/>
-      <c r="E17" s="2" t="n"/>
-      <c r="F17" s="2" t="n"/>
-      <c r="G17" s="2" t="n"/>
-      <c r="H17" s="2" t="n"/>
-      <c r="I17" s="2" t="n"/>
-      <c r="J17" s="2" t="n"/>
+      <c r="A17" s="2" t="inlineStr">
+        <is>
+          <t>TC-016</t>
+        </is>
+      </c>
+      <c r="B17" s="2" t="inlineStr">
+        <is>
+          <t>F-20</t>
+        </is>
+      </c>
+      <c r="C17" s="2" t="inlineStr">
+        <is>
+          <t>Вхід із зареєстрованою адресою і неправильним паролем</t>
+        </is>
+      </c>
+      <c r="D17" s="2" t="inlineStr">
+        <is>
+          <t>Chrome 120 або новіший, вікно 1280×800; demo доступне (збірка v2.5 від 2026-10-11 за написом у підвалі сторінки; стан звірено 26.10.2026); нова сесія, без входу. Адреса customer@practicesoftwaretesting.com зареєстрована на demo (SRS 1.1, розд. 2.2). Лише одна спроба з неправильним паролем за виконання кейсу, щоб не заблокувати спільний обліковий запис для інших користувачів demo (методичка, п. 5.4).</t>
+        </is>
+      </c>
+      <c r="E17" s="2" t="inlineStr">
+        <is>
+          <t>1. Відкрити https://practicesoftwaretesting.com у Chrome (нова сесія).
+2. Натиснути «Sign in» у верхньому меню.
+3. У поле «Email address» ввести: customer@practicesoftwaretesting.com
+4. У поле «Password» ввести: Wrong-pass1
+5. Натиснути кнопку «Login».
+6. Закрити вкладку.</t>
+        </is>
+      </c>
+      <c r="F17" s="2" t="inlineStr">
+        <is>
+          <t>Після кроку 1: головна сторінка з каталогом; у меню — «Sign in».
+Після кроку 2: сторінка входу (адреса містить /auth/login): поля «Email address» і «Password», кнопка «Login».
+Після кроку 3: у полі «Email address» — customer@practicesoftwaretesting.com.
+Після кроку 4: символи пароля замасковано.
+Після кроку 5: повідомлення «Invalid email or password» (F-20); адреса не змінилася (/auth/login); у меню — «Sign in» (сеанс не створено).
+Після кроку 6: вкладку закрито.</t>
+        </is>
+      </c>
+      <c r="G17" s="2" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="H17" s="2" t="inlineStr">
+        <is>
+          <t>негативний</t>
+        </is>
+      </c>
+      <c r="I17" s="2" t="inlineStr">
+        <is>
+          <t>Клас «зареєстрована адреса, неправильний пароль» (F-20) — інший клас, ніж у TC-004 (незареєстрована адреса): перевіряє, що для правильної адреси система показує те саме повідомлення і не створює сеанс. Пароль Wrong-pass1 вигаданий і відрізняється від welcome01. Позитивна пара — TC-015.</t>
+        </is>
+      </c>
+      <c r="J17" s="2" t="inlineStr">
+        <is>
+          <t>Тимчак А. (ІТ)</t>
+        </is>
+      </c>
       <c r="K17" s="2" t="n"/>
       <c r="L17" s="2" t="n"/>
-      <c r="M17" s="2" t="n"/>
+      <c r="M17" s="2" t="inlineStr">
+        <is>
+          <t>draft</t>
+        </is>
+      </c>
       <c r="N17" s="2" t="n"/>
     </row>
     <row r="18">
-      <c r="A18" s="2" t="n"/>
-      <c r="B18" s="2" t="n"/>
-      <c r="C18" s="2" t="n"/>
-      <c r="D18" s="2" t="n"/>
-      <c r="E18" s="2" t="n"/>
-      <c r="F18" s="2" t="n"/>
-      <c r="G18" s="2" t="n"/>
-      <c r="H18" s="2" t="n"/>
-      <c r="I18" s="2" t="n"/>
-      <c r="J18" s="2" t="n"/>
+      <c r="A18" s="2" t="inlineStr">
+        <is>
+          <t>TC-017</t>
+        </is>
+      </c>
+      <c r="B18" s="2" t="inlineStr">
+        <is>
+          <t>F-110</t>
+        </is>
+      </c>
+      <c r="C18" s="2" t="inlineStr">
+        <is>
+          <t>Оформлення замовлення у 4 кроки з входом на кроці «Sign in» і оплатою «Cash on Delivery»</t>
+        </is>
+      </c>
+      <c r="D18" s="2" t="inlineStr">
+        <is>
+          <t>Chrome 120 або новіший, вікно 1280×800; demo доступне (збірка v2.5 від 2026-10-11 за написом у підвалі сторінки; стан звірено 26.10.2026); нова сесія, без входу, кошик порожній; спільний обліковий запис покупця customer@practicesoftwaretesting.com / welcome01 (SRS 1.1, розд. 2.2); пароль спільного облікового запису не змінювати (методичка, п. 5.4). Товар «Combination Pliers» є в каталозі і в наявності. Адреса доставки вигадана.</t>
+        </is>
+      </c>
+      <c r="E18" s="2" t="inlineStr">
+        <is>
+          <t>1. Відкрити https://practicesoftwaretesting.com у Chrome (нова сесія).
+2. Натиснути картку товару «Combination Pliers».
+3. Натиснути кнопку «Add to cart».
+4. Натиснути піктограму кошика у верхньому меню.
+5. Натиснути «Proceed to checkout».
+6. У поле «Email address» ввести: customer@practicesoftwaretesting.com
+7. У поле «Password» ввести: welcome01
+8. Натиснути кнопку «Login».
+9. У поле «Street» ввести (замість поточного значення): Testova 1
+10. У поле «City» ввести (замість поточного значення): Kyiv
+11. У поле «State» ввести (замість поточного значення): Kyiv
+12. У поле «Country» ввести (замість поточного значення): Ukraine
+13. У поле «Postal code» ввести (замість поточного значення): 01001
+14. Натиснути «Proceed to checkout».
+15. У списку способів оплати вибрати «Cash on Delivery».
+16. Натиснути «Confirm».
+17. Закрити вкладку.</t>
+        </is>
+      </c>
+      <c r="F18" s="2" t="inlineStr">
+        <is>
+          <t>Після кроку 1: головна сторінка з каталогом; є картка «Combination Pliers».
+Після кроку 2: сторінка товару «Combination Pliers» з ціною і кнопкою «Add to cart».
+Після кроку 3: не пізніше ніж за 2 с — повідомлення «Product added to shopping cart.» (F-90).
+Після кроку 4: крок «Cart» (1 з 4); над таблицею — чотири кроки «Cart», «Sign in», «Billing Address», «Payment» (F-110); один рядок «Combination Pliers», кількість 1, «Total» дорівнює ціні з кроку 2 (сума товарів, F-110).
+Після кроку 5: крок «Sign in» (2 з 4): форма входу з полями «Email address» і «Password», кнопка «Login».
+Після кроку 6: у полі «Email address» — customer@practicesoftwaretesting.com.
+Після кроку 7: символи пароля замасковано.
+Після кроку 8: вхід виконано, відкрито крок «Billing Address» (3 з 4) (F-20, F-110); є поля «Street», «City», «State», «Country», «Postal code».
+Після кроків 9–13: у полях відображено введені значення: Testova 1, Kyiv, Kyiv, Ukraine, 01001.
+Після кроку 14: крок «Payment» (4 з 4); список способів оплати містить банківський переказ, оплату при отриманні, кредитну картку, «купити зараз — заплатити пізніше» і подарункову картку (F-110).
+Після кроку 15: вибрано «Cash on Delivery»; кнопка «Confirm» доступна.
+Після кроку 16: замовлення підтверджено; показано текстове повідомлення з номером рахунку-інвойсу (F-110; SRS 1.1 точного тексту не задає).
+Після кроку 17: вкладку закрито.</t>
+        </is>
+      </c>
+      <c r="G18" s="2" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="H18" s="2" t="inlineStr">
+        <is>
+          <t>позитивний</t>
+        </is>
+      </c>
+      <c r="I18" s="2" t="inlineStr">
+        <is>
+          <t>Основний сценарій F-110: неавторизований покупець проходить усі 4 кроки і входить на кроці 2 (клас «вхід під час оформлення»). Оплата при отриманні не потребує платіжних даних; реальна оплата на demo не проводиться (SRS 1.1, розд. 2.3). Адреса вигадана, поля заповнюються явно, щоб кейс не залежав від даних профілю. Знижки і вартість доставки (BL-50 – BL-80) не перевіряються: модуль лояльності не інтегровано в demo (SRS 1.1, розд. 2.3).</t>
+        </is>
+      </c>
+      <c r="J18" s="2" t="inlineStr">
+        <is>
+          <t>Тимчак А. (ІТ)</t>
+        </is>
+      </c>
       <c r="K18" s="2" t="n"/>
       <c r="L18" s="2" t="n"/>
-      <c r="M18" s="2" t="n"/>
+      <c r="M18" s="2" t="inlineStr">
+        <is>
+          <t>draft</t>
+        </is>
+      </c>
       <c r="N18" s="2" t="n"/>
     </row>
     <row r="19">
-      <c r="A19" s="2" t="n"/>
-      <c r="B19" s="2" t="n"/>
-      <c r="C19" s="2" t="n"/>
-      <c r="D19" s="2" t="n"/>
-      <c r="E19" s="2" t="n"/>
-      <c r="F19" s="2" t="n"/>
-      <c r="G19" s="2" t="n"/>
-      <c r="H19" s="2" t="n"/>
-      <c r="I19" s="2" t="n"/>
-      <c r="J19" s="2" t="n"/>
+      <c r="A19" s="2" t="inlineStr">
+        <is>
+          <t>TC-018</t>
+        </is>
+      </c>
+      <c r="B19" s="2" t="inlineStr">
+        <is>
+          <t>GUI-40, F-120</t>
+        </is>
+      </c>
+      <c r="C19" s="2" t="inlineStr">
+        <is>
+          <t>«Add to favourites» без входу: повідомлення про відмову, товар не додано</t>
+        </is>
+      </c>
+      <c r="D19" s="2" t="inlineStr">
+        <is>
+          <t>Chrome 120 або новіший, вікно 1280×800; demo доступне (збірка v2.5 від 2026-10-11 за написом у підвалі сторінки; стан звірено 26.10.2026); нова сесія, без входу. Товар «Combination Pliers» є в каталозі.</t>
+        </is>
+      </c>
+      <c r="E19" s="2" t="inlineStr">
+        <is>
+          <t>1. Відкрити https://practicesoftwaretesting.com у Chrome (нова сесія).
+2. Натиснути картку товару «Combination Pliers».
+3. Натиснути кнопку «Add to favourites».
+4. Закрити вкладку.</t>
+        </is>
+      </c>
+      <c r="F19" s="2" t="inlineStr">
+        <is>
+          <t>Після кроку 1: головна сторінка з каталогом; у меню — «Sign in»; є картка «Combination Pliers».
+Після кроку 2: сторінка товару «Combination Pliers»; кнопка «Add to favourites» відображається (GUI-40).
+Після кроку 3: повідомлення «Unauthorized, can not add product to your favorite list» (GUI-40); відкрита та сама сторінка товару; у меню — «Sign in» (товар до обраного не додано, F-120).
+Після кроку 4: вкладку закрито.</t>
+        </is>
+      </c>
+      <c r="G19" s="2" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="H19" s="2" t="inlineStr">
+        <is>
+          <t>негативний</t>
+        </is>
+      </c>
+      <c r="I19" s="2" t="inlineStr">
+        <is>
+          <t>Клас «неавторизований покупець» для F-120 / GUI-40. Текст повідомлення — з GUI-40 SRS 1.1; на demo 26.10.2026 він виводиться з крапкою в кінці. Позитивна пара (додавання після входу, перегляд у «My favorites», видалення) — резервний кейс ІТ (TC-025+).</t>
+        </is>
+      </c>
+      <c r="J19" s="2" t="inlineStr">
+        <is>
+          <t>Тимчак А. (ІТ)</t>
+        </is>
+      </c>
       <c r="K19" s="2" t="n"/>
       <c r="L19" s="2" t="n"/>
-      <c r="M19" s="2" t="n"/>
+      <c r="M19" s="2" t="inlineStr">
+        <is>
+          <t>draft</t>
+        </is>
+      </c>
       <c r="N19" s="2" t="n"/>
     </row>
     <row r="20">
-      <c r="A20" s="2" t="n"/>
-      <c r="B20" s="2" t="n"/>
-      <c r="C20" s="2" t="n"/>
-      <c r="D20" s="2" t="n"/>
-      <c r="E20" s="2" t="n"/>
-      <c r="F20" s="2" t="n"/>
-      <c r="G20" s="2" t="n"/>
-      <c r="H20" s="2" t="n"/>
-      <c r="I20" s="2" t="n"/>
-      <c r="J20" s="2" t="n"/>
+      <c r="A20" s="2" t="inlineStr">
+        <is>
+          <t>TC-019</t>
+        </is>
+      </c>
+      <c r="B20" s="2" t="inlineStr">
+        <is>
+          <t>F-30</t>
+        </is>
+      </c>
+      <c r="C20" s="2" t="inlineStr">
+        <is>
+          <t>Форма відновлення пароля: перехід за посиланням «Forgot your Password?» і надсилання адреси</t>
+        </is>
+      </c>
+      <c r="D20" s="2" t="inlineStr">
+        <is>
+          <t>Chrome 120 або новіший, вікно 1280×800; demo доступне (збірка v2.5 від 2026-10-11 за написом у підвалі сторінки; стан звірено 26.10.2026); нова сесія, без входу. Обліковий запис shopline.it.tc019@example.com зареєстровано заздалегідь через «Register your account» з вигаданими даними. Спільні облікові записи customer@… і admin@… не використовувати: відновлення може змінити їхній пароль (методичка, п. 5.4). Доставку листа на demo не спостерігаємо: адреса вигадана.</t>
+        </is>
+      </c>
+      <c r="E20" s="2" t="inlineStr">
+        <is>
+          <t>1. Відкрити https://practicesoftwaretesting.com у Chrome (нова сесія).
+2. Натиснути «Sign in» у верхньому меню.
+3. Натиснути посилання «Forgot your Password?».
+4. У поле «Email address» ввести: shopline.it.tc019@example.com
+5. Натиснути кнопку «Set New Password».
+6. Закрити вкладку.</t>
+        </is>
+      </c>
+      <c r="F20" s="2" t="inlineStr">
+        <is>
+          <t>Після кроку 1: головна сторінка з каталогом; у меню — «Sign in».
+Після кроку 2: сторінка входу (адреса містить /auth/login); є посилання «Forgot your Password?».
+Після кроку 3: відкрито форму відновлення пароля (адреса містить /auth/forgot-password): заголовок «Forgot Password», поле «Email address», кнопка «Set New Password» (F-30).
+Після кроку 4: у полі «Email address» — shopline.it.tc019@example.com.
+Після кроку 5: форму надіслано; на сторінці текстове повідомлення про надсилання листа для встановлення нового пароля (F-30; SRS 1.1 точного тексту не задає); повідомлень про помилку під полем немає.
+Після кроку 6: вкладку закрито.</t>
+        </is>
+      </c>
+      <c r="G20" s="2" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="H20" s="2" t="inlineStr">
+        <is>
+          <t>позитивний</t>
+        </is>
+      </c>
+      <c r="I20" s="2" t="inlineStr">
+        <is>
+          <t>Клас «зареєстрована адреса» для F-30. Через UI спостерігаються форма і реакція сторінки після надсилання; час передачі листа поштовому сервісу (1 с) і доставку на demo перевірити не можна (Coverage, примітка до F-30). Адреса вигадана з домену example.com.</t>
+        </is>
+      </c>
+      <c r="J20" s="2" t="inlineStr">
+        <is>
+          <t>Тимчак А. (ІТ)</t>
+        </is>
+      </c>
       <c r="K20" s="2" t="n"/>
       <c r="L20" s="2" t="n"/>
-      <c r="M20" s="2" t="n"/>
+      <c r="M20" s="2" t="inlineStr">
+        <is>
+          <t>draft</t>
+        </is>
+      </c>
       <c r="N20" s="2" t="n"/>
     </row>
     <row r="21">

</xml_diff>

<commit_message>
SCRUM-118, SCRUM-119: зведений test-cases.xlsx, кейси TC-020–024, Review (фаза 1)
     - Аркуш Test cases: зведено TC-001–004 (ТА), TC-009–014 (КТ), TC-015–019 (ІТ), TC-020–024 (СМ, draft)
     - Coverage: без змін (ТА)
     - Review: фаза 1 для TC-001–019 (СМ, 27.10.2026)

     @Олександра: прошу рецензію TC-020–024 — рядки в аркуші Review (8 пунктів, дата, зауваження).
     Зауваження фази 1 для авторок — у стовпці «Зауваження» аркуша Review.
</commit_message>
<xml_diff>
--- a/docs/sprint3/test-cases.xlsx
+++ b/docs/sprint3/test-cases.xlsx
@@ -9,6 +9,7 @@
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test cases" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Coverage" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Review" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Test cases'!$A$1:$N$41</definedName>
@@ -37,7 +38,7 @@
       <color rgb="00808080"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="4">
     <fill>
       <patternFill/>
     </fill>
@@ -47,6 +48,11 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00D9E1F2"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00F8CBAD"/>
       </patternFill>
     </fill>
   </fills>
@@ -76,7 +82,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
@@ -88,6 +94,12 @@
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -547,323 +559,1432 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="2" t="n"/>
-      <c r="B2" s="2" t="n"/>
-      <c r="C2" s="2" t="n"/>
-      <c r="D2" s="2" t="n"/>
-      <c r="E2" s="2" t="n"/>
-      <c r="F2" s="2" t="n"/>
-      <c r="G2" s="2" t="n"/>
-      <c r="H2" s="2" t="n"/>
-      <c r="I2" s="2" t="n"/>
-      <c r="J2" s="2" t="n"/>
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>TC-001</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>F-60</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>Пошук товарів за частиною назви, введеною в нижньому регістрі, без входу</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>Chrome (поточна стабільна версія), нова сесія (вікно інкогніто), без входу. У каталозі є товари зі словом «Pliers» у назві (стан demo 25.10.2026: Combination Pliers, Pliers, Long Nose Pliers, Slip Joint Pliers).</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>1. Відкрити https://practicesoftwaretesting.com у Chrome (нова сесія).
+2. У поле пошуку «Search» ввести pliers.
+3. Натиснути кнопку «Search».
+4. Переглянути назви всіх карток у списку результатів.
+5. Закрити вкладку.</t>
+        </is>
+      </c>
+      <c r="F2" s="2" t="inlineStr">
+        <is>
+          <t>1. Головна сторінка з каталогом карток, полем «Search» і кнопками «X» та «Search».
+2. У полі «Search» показано текст pliers.
+3. Список карток оновлено; результати під заголовком «Searched for: pliers».
+4. Кожна назва містить «pliers» без урахування регістру (наприклад, «Combination Pliers»); карток без цього слова немає.
+5. Вкладку закрито.</t>
+        </is>
+      </c>
+      <c r="G2" s="2" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="H2" s="2" t="inlineStr">
+        <is>
+          <t>позитивний</t>
+        </is>
+      </c>
+      <c r="I2" s="2" t="inlineStr">
+        <is>
+          <t>Клас «підрядок, що є в назвах товарів». Запит у нижньому регістрі, а в назвах — «Pliers» з великої літери: перевіряє умову F-60 «без урахування регістру літер».</t>
+        </is>
+      </c>
+      <c r="J2" s="2" t="inlineStr">
+        <is>
+          <t>Коротка К. (ТА)</t>
+        </is>
+      </c>
       <c r="K2" s="2" t="n"/>
       <c r="L2" s="2" t="n"/>
-      <c r="M2" s="2" t="n"/>
+      <c r="M2" s="2" t="inlineStr">
+        <is>
+          <t>draft</t>
+        </is>
+      </c>
       <c r="N2" s="2" t="n"/>
     </row>
     <row r="3">
-      <c r="A3" s="2" t="n"/>
-      <c r="B3" s="2" t="n"/>
-      <c r="C3" s="2" t="n"/>
-      <c r="D3" s="2" t="n"/>
-      <c r="E3" s="2" t="n"/>
-      <c r="F3" s="2" t="n"/>
-      <c r="G3" s="2" t="n"/>
-      <c r="H3" s="2" t="n"/>
-      <c r="I3" s="2" t="n"/>
-      <c r="J3" s="2" t="n"/>
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>TC-002</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>GUI-30</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>Додавання товару в кошик із кількістю 99 (верхня межа) без входу</t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t>Chrome (поточна стабільна версія), нова сесія (вікно інкогніто), без входу. Кошик порожній. Товар «Combination Pliers» є на першій сторінці каталогу і в наявності.</t>
+        </is>
+      </c>
+      <c r="E3" s="2" t="inlineStr">
+        <is>
+          <t>1. Відкрити https://practicesoftwaretesting.com у Chrome (нова сесія).
+2. Натиснути на картку товару «Combination Pliers».
+3. У поле «Quantity» ввести 99 (замість значення 1).
+4. Натиснути кнопку «Add to cart».
+5. Натиснути піктограму кошика у верхньому меню.
+6. У рядку «Combination Pliers» натиснути червону кнопку видалення.
+7. Закрити вкладку.</t>
+        </is>
+      </c>
+      <c r="F3" s="2" t="inlineStr">
+        <is>
+          <t>1. Головна сторінка з каталогом; є картка «Combination Pliers».
+2. Сторінка товару «Combination Pliers»: ціна; поле «Quantity» зі значенням 1 і кнопками «−» та «+»; кнопка «Add to cart».
+3. У полі «Quantity» — 99; під полем повідомлень про помилку немає.
+4. Не пізніше ніж за 2 с — повідомлення «Product added to shopping cart.»; на піктограмі кошика в меню — 99.
+5. Крок «Cart»: один рядок «Combination Pliers», «Quantity» — 99, «Total» = 99 × ціна з кроку 2.
+6. Рядок видалено; замість таблиці — текстове повідомлення про порожній кошик (на demo 25.10.2026 — «The cart is empty. Nothing to display.»).
+7. Вкладку закрито.</t>
+        </is>
+      </c>
+      <c r="G3" s="2" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="H3" s="2" t="inlineStr">
+        <is>
+          <t>позитивний</t>
+        </is>
+      </c>
+      <c r="I3" s="2" t="inlineStr">
+        <is>
+          <t>Граничне значення: верхня межа діапазону 1–99 (GUI-30), клас «допустима кількість». Негативна пара — TC-003 (100).</t>
+        </is>
+      </c>
+      <c r="J3" s="2" t="inlineStr">
+        <is>
+          <t>Коротка К. (ТА)</t>
+        </is>
+      </c>
       <c r="K3" s="2" t="n"/>
       <c r="L3" s="2" t="n"/>
-      <c r="M3" s="2" t="n"/>
+      <c r="M3" s="2" t="inlineStr">
+        <is>
+          <t>draft</t>
+        </is>
+      </c>
       <c r="N3" s="2" t="n"/>
     </row>
     <row r="4">
-      <c r="A4" s="2" t="n"/>
-      <c r="B4" s="2" t="n"/>
-      <c r="C4" s="2" t="n"/>
-      <c r="D4" s="2" t="n"/>
-      <c r="E4" s="2" t="n"/>
-      <c r="F4" s="2" t="n"/>
-      <c r="G4" s="2" t="n"/>
-      <c r="H4" s="2" t="n"/>
-      <c r="I4" s="2" t="n"/>
-      <c r="J4" s="2" t="n"/>
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>TC-003</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>GUI-30</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>Спроба додати товар у кошик із кількістю 100 (більше верхньої межі) без входу</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>Chrome (поточна стабільна версія), нова сесія (вікно інкогніто), без входу. Кошик порожній. Товар «Combination Pliers» є на першій сторінці каталогу і в наявності.</t>
+        </is>
+      </c>
+      <c r="E4" s="2" t="inlineStr">
+        <is>
+          <t>1. Відкрити https://practicesoftwaretesting.com у Chrome (нова сесія).
+2. Натиснути на картку товару «Combination Pliers».
+3. У поле «Quantity» ввести 100 (замість значення 1).
+4. Натиснути кнопку «Add to cart».
+5. В адресному рядку відкрити https://practicesoftwaretesting.com/checkout.
+6. Закрити вкладку.</t>
+        </is>
+      </c>
+      <c r="F4" s="2" t="inlineStr">
+        <is>
+          <t>1. Головна сторінка з каталогом; є картка «Combination Pliers».
+2. Сторінка товару «Combination Pliers»: поле «Quantity» зі значенням 1 і кнопками «−» та «+»; кнопка «Add to cart».
+3. Значення 100 не прийнято: поле «Quantity» приймає лише цілі значення від 1 до 99 (GUI-30).
+4. Товар у кількості 100 не додано: на піктограмі кошика в меню немає числа 100.
+5. Крок «Cart»: рядка «Combination Pliers» з кількістю 100 немає.
+6. Вкладку закрито.</t>
+        </is>
+      </c>
+      <c r="G4" s="2" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="H4" s="2" t="inlineStr">
+        <is>
+          <t>негативний</t>
+        </is>
+      </c>
+      <c r="I4" s="2" t="inlineStr">
+        <is>
+          <t>Граничне значення: b+1 для діапазону 1–99 (GUI-30), клас «кількість більша за 99». Позитивна пара — TC-002 (99).</t>
+        </is>
+      </c>
+      <c r="J4" s="2" t="inlineStr">
+        <is>
+          <t>Коротка К. (ТА)</t>
+        </is>
+      </c>
       <c r="K4" s="2" t="n"/>
       <c r="L4" s="2" t="n"/>
-      <c r="M4" s="2" t="n"/>
+      <c r="M4" s="2" t="inlineStr">
+        <is>
+          <t>draft</t>
+        </is>
+      </c>
       <c r="N4" s="2" t="n"/>
     </row>
     <row r="5">
-      <c r="A5" s="2" t="n"/>
-      <c r="B5" s="2" t="n"/>
-      <c r="C5" s="2" t="n"/>
-      <c r="D5" s="2" t="n"/>
-      <c r="E5" s="2" t="n"/>
-      <c r="F5" s="2" t="n"/>
-      <c r="G5" s="2" t="n"/>
-      <c r="H5" s="2" t="n"/>
-      <c r="I5" s="2" t="n"/>
-      <c r="J5" s="2" t="n"/>
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>TC-004</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>F-20</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>Вхід із незареєстрованою адресою електронної пошти</t>
+        </is>
+      </c>
+      <c r="D5" s="2" t="inlineStr">
+        <is>
+          <t>Chrome (поточна стабільна версія), нова сесія (вікно інкогніто), без входу. Адреса shopline.ta.test@example.com на demo не зареєстрована.</t>
+        </is>
+      </c>
+      <c r="E5" s="2" t="inlineStr">
+        <is>
+          <t>1. Відкрити https://practicesoftwaretesting.com у Chrome (нова сесія).
+2. Натиснути «Sign in» у верхньому меню.
+3. У поле «Email address» ввести shopline.ta.test@example.com.
+4. У поле «Password» ввести Test-pass1.
+5. Натиснути кнопку «Login».
+6. Закрити вкладку.</t>
+        </is>
+      </c>
+      <c r="F5" s="2" t="inlineStr">
+        <is>
+          <t>1. Головна сторінка з каталогом; у меню — «Sign in».
+2. Сторінка входу (адреса містить /auth/login): поля «Email address» і «Password», кнопка «Login».
+3. У полі «Email address» — shopline.ta.test@example.com.
+4. Символи пароля замасковано.
+5. Повідомлення «Invalid email or password»; адреса не змінилася (/auth/login); у меню — «Sign in» (сеанс не створено).
+6. Вкладку закрито.</t>
+        </is>
+      </c>
+      <c r="G5" s="2" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="H5" s="2" t="inlineStr">
+        <is>
+          <t>негативний</t>
+        </is>
+      </c>
+      <c r="I5" s="2" t="inlineStr">
+        <is>
+          <t>Клас «неправильна пара адреса — пароль» (F-20): вигадана незареєстрована адреса з домену example.com. Спільний обліковий запис customer@… не використано, щоб невдалі спроби входу не вплинули на інших користувачів demo (п. 5.4).</t>
+        </is>
+      </c>
+      <c r="J5" s="2" t="inlineStr">
+        <is>
+          <t>Коротка К. (ТА)</t>
+        </is>
+      </c>
       <c r="K5" s="2" t="n"/>
       <c r="L5" s="2" t="n"/>
-      <c r="M5" s="2" t="n"/>
+      <c r="M5" s="2" t="inlineStr">
+        <is>
+          <t>draft</t>
+        </is>
+      </c>
       <c r="N5" s="2" t="n"/>
     </row>
     <row r="6">
-      <c r="A6" s="2" t="n"/>
-      <c r="B6" s="2" t="n"/>
-      <c r="C6" s="2" t="n"/>
-      <c r="D6" s="2" t="n"/>
-      <c r="E6" s="2" t="n"/>
-      <c r="F6" s="2" t="n"/>
-      <c r="G6" s="2" t="n"/>
-      <c r="H6" s="2" t="n"/>
-      <c r="I6" s="2" t="n"/>
-      <c r="J6" s="2" t="n"/>
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>TC-009</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>F-140, GUI-50</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="inlineStr">
+        <is>
+          <t>Контактна форма: повідомлення з 49 символів (нижче межі) не надсилається</t>
+        </is>
+      </c>
+      <c r="D6" s="2" t="inlineStr">
+        <is>
+          <t>Chrome 120 або новіший, вікно 1280×800; demo доступне (збірка v2.5 від 2026-10-11 за написом у підвалі сторінки; стан звірено 25.10.2026); обліковий запис не потрібен (звернення від анонімного відвідувача); дані лише вигадані.</t>
+        </is>
+      </c>
+      <c r="E6" s="2" t="inlineStr">
+        <is>
+          <t>1. Відкрити https://practicesoftwaretesting.com/contact у Chrome (нова сесія).
+2. У поле «Your first name» ввести: Test
+3. У поле «Your last name» ввести: Tester
+4. У поле «Your email» ввести: tester.tc009@example.com
+5. У списку «Select a subject» вибрати: Customer service
+6. У поле «Message» ввести 49 символів: abcdefghijabcdefghijabcdefghijabcdefghijabcdefghi
+7. Натиснути «Send».
+8. Закрити вкладку.</t>
+        </is>
+      </c>
+      <c r="F6" s="2" t="inlineStr">
+        <is>
+          <t>Після кроку 1: відкрито сторінку «Contact», усі поля порожні.
+Після кроків 2–5: у полях відображено введені значення: Test, Tester, tester.tc009@example.com, Customer service.
+Після кроку 6: у полі «Message» 49 символів.
+Після кроку 7: форму не надіслано, сторінка «Contact» залишається відкритою; під полем «Message» текстове повідомлення про помилку, яке називає межу в 50 символів (F-140, GUI-50; SRS 1.1 точного тексту не задає); під іншими полями повідомлень про помилки немає; повідомлення про прийняття звернення над формою відсутнє.
+Після кроку 8: вкладку закрито.</t>
+        </is>
+      </c>
+      <c r="G6" s="2" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="H6" s="2" t="inlineStr">
+        <is>
+          <t>негативний</t>
+        </is>
+      </c>
+      <c r="I6" s="2" t="inlineStr">
+        <is>
+          <t>Допустима довжина повідомлення 50–250 (F-140). 49 — на 1 менше за нижню межу, клас недопустимих значень. Решта полів валідні, тому відхилення можливе лише через довжину.</t>
+        </is>
+      </c>
+      <c r="J6" s="2" t="inlineStr">
+        <is>
+          <t>Горбонос О. (КТ)</t>
+        </is>
+      </c>
       <c r="K6" s="2" t="n"/>
       <c r="L6" s="2" t="n"/>
-      <c r="M6" s="2" t="n"/>
+      <c r="M6" s="2" t="inlineStr">
+        <is>
+          <t>draft</t>
+        </is>
+      </c>
       <c r="N6" s="2" t="n"/>
     </row>
     <row r="7">
-      <c r="A7" s="2" t="n"/>
-      <c r="B7" s="2" t="n"/>
-      <c r="C7" s="2" t="n"/>
-      <c r="D7" s="2" t="n"/>
-      <c r="E7" s="2" t="n"/>
-      <c r="F7" s="2" t="n"/>
-      <c r="G7" s="2" t="n"/>
-      <c r="H7" s="2" t="n"/>
-      <c r="I7" s="2" t="n"/>
-      <c r="J7" s="2" t="n"/>
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>TC-010</t>
+        </is>
+      </c>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>F-140, GUI-90</t>
+        </is>
+      </c>
+      <c r="C7" s="2" t="inlineStr">
+        <is>
+          <t>Контактна форма: повідомлення з 50 символів (нижня межа) приймається, показано підтвердження</t>
+        </is>
+      </c>
+      <c r="D7" s="2" t="inlineStr">
+        <is>
+          <t>Chrome 120 або новіший, вікно 1280×800; demo доступне (збірка v2.5 від 2026-10-11 за написом у підвалі сторінки; стан звірено 25.10.2026); обліковий запис не потрібен (звернення від анонімного відвідувача); дані лише вигадані.</t>
+        </is>
+      </c>
+      <c r="E7" s="2" t="inlineStr">
+        <is>
+          <t>1. Відкрити https://practicesoftwaretesting.com/contact у Chrome (нова сесія).
+2. У поле «Your first name» ввести: Test
+3. У поле «Your last name» ввести: Tester
+4. У поле «Your email» ввести: tester.tc010@example.com
+5. У списку «Select a subject» вибрати: Customer service
+6. У поле «Message» ввести 50 символів: abcdefghijabcdefghijabcdefghijabcdefghijabcdefghij
+7. Натиснути «Send».
+8. Закрити вкладку.</t>
+        </is>
+      </c>
+      <c r="F7" s="2" t="inlineStr">
+        <is>
+          <t>Після кроку 1: відкрито сторінку «Contact»; є поля імені, прізвища й адреси електронної пошти, розкривний список теми, багаторядкове поле «Message», елемент вибору файла «Attachment» і кнопка «Send» (GUI-90).
+Після кроків 2–5: у полях відображено введені значення: Test, Tester, tester.tc010@example.com, Customer service.
+Після кроку 6: у полі «Message» 50 символів.
+Після кроку 7: звернення прийнято; над формою виводиться текстове повідомлення про прийняття звернення (F-140, GUI-90). SRS 1.1 точного тексту не задає; на demo 26.10.2026 текст такий: «Thanks for your message! We will contact you shortly.» (джерело — спостереження на demo, не SRS). Повідомлень про помилки під полями немає.
+Після кроку 8: вкладку закрито.</t>
+        </is>
+      </c>
+      <c r="G7" s="2" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="H7" s="2" t="inlineStr">
+        <is>
+          <t>позитивний</t>
+        </is>
+      </c>
+      <c r="I7" s="2" t="inlineStr">
+        <is>
+          <t>50 — нижня межа допустимого діапазону 50–250 (перше допустиме значення). Вкладення не додається, щоб один кейс відповідав одному набору даних.</t>
+        </is>
+      </c>
+      <c r="J7" s="2" t="inlineStr">
+        <is>
+          <t>Горбонос О. (КТ)</t>
+        </is>
+      </c>
       <c r="K7" s="2" t="n"/>
       <c r="L7" s="2" t="n"/>
-      <c r="M7" s="2" t="n"/>
+      <c r="M7" s="2" t="inlineStr">
+        <is>
+          <t>draft</t>
+        </is>
+      </c>
       <c r="N7" s="2" t="n"/>
     </row>
     <row r="8">
-      <c r="A8" s="2" t="n"/>
-      <c r="B8" s="2" t="n"/>
-      <c r="C8" s="2" t="n"/>
-      <c r="D8" s="2" t="n"/>
-      <c r="E8" s="2" t="n"/>
-      <c r="F8" s="2" t="n"/>
-      <c r="G8" s="2" t="n"/>
-      <c r="H8" s="2" t="n"/>
-      <c r="I8" s="2" t="n"/>
-      <c r="J8" s="2" t="n"/>
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>TC-011</t>
+        </is>
+      </c>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>F-140</t>
+        </is>
+      </c>
+      <c r="C8" s="2" t="inlineStr">
+        <is>
+          <t>Контактна форма: повідомлення з 250 символів (верхня межа) приймається</t>
+        </is>
+      </c>
+      <c r="D8" s="2" t="inlineStr">
+        <is>
+          <t>Chrome 120 або новіший, вікно 1280×800; demo доступне (збірка v2.5 від 2026-10-11 за написом у підвалі сторінки; стан звірено 25.10.2026); обліковий запис не потрібен (звернення від анонімного відвідувача); дані лише вигадані.</t>
+        </is>
+      </c>
+      <c r="E8" s="2" t="inlineStr">
+        <is>
+          <t>1. Відкрити https://practicesoftwaretesting.com/contact у Chrome (нова сесія).
+2. У поле «Your first name» ввести: Test
+3. У поле «Your last name» ввести: Tester
+4. У поле «Your email» ввести: tester.tc011@example.com
+5. У списку «Select a subject» вибрати: Customer service
+6. У поле «Message» ввести 250 символів: abcdefghijabcdefghijabcdefghijabcdefghijabcdefghijabcdefghijabcdefghijabcdefghijabcdefghijabcdefghijabcdefghijabcdefghijabcdefghijabcdefghijabcdefghijabcdefghijabcdefghijabcdefghijabcdefghijabcdefghijabcdefghijabcdefghijabcdefghijabcdefghijabcdefghij
+7. Натиснути «Send».
+8. Закрити вкладку.</t>
+        </is>
+      </c>
+      <c r="F8" s="2" t="inlineStr">
+        <is>
+          <t>Після кроку 1: відкрито сторінку «Contact», усі поля порожні.
+Після кроків 2–5: у полях відображено введені значення: Test, Tester, tester.tc011@example.com, Customer service.
+Після кроку 6: у полі «Message» 250 символів.
+Після кроку 7: звернення прийнято; над формою виводиться текстове повідомлення про прийняття звернення (F-140); повідомлень про помилки під полями немає.
+Після кроку 8: вкладку закрито.</t>
+        </is>
+      </c>
+      <c r="G8" s="2" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="H8" s="2" t="inlineStr">
+        <is>
+          <t>позитивний</t>
+        </is>
+      </c>
+      <c r="I8" s="2" t="inlineStr">
+        <is>
+          <t>250 — верхня межа допустимого діапазону 50–250 (останнє допустиме значення).</t>
+        </is>
+      </c>
+      <c r="J8" s="2" t="inlineStr">
+        <is>
+          <t>Горбонос О. (КТ)</t>
+        </is>
+      </c>
       <c r="K8" s="2" t="n"/>
       <c r="L8" s="2" t="n"/>
-      <c r="M8" s="2" t="n"/>
+      <c r="M8" s="2" t="inlineStr">
+        <is>
+          <t>draft</t>
+        </is>
+      </c>
       <c r="N8" s="2" t="n"/>
     </row>
     <row r="9">
-      <c r="A9" s="2" t="n"/>
-      <c r="B9" s="2" t="n"/>
-      <c r="C9" s="2" t="n"/>
-      <c r="D9" s="2" t="n"/>
-      <c r="E9" s="2" t="n"/>
-      <c r="F9" s="2" t="n"/>
-      <c r="G9" s="2" t="n"/>
-      <c r="H9" s="2" t="n"/>
-      <c r="I9" s="2" t="n"/>
-      <c r="J9" s="2" t="n"/>
+      <c r="A9" s="2" t="inlineStr">
+        <is>
+          <t>TC-012</t>
+        </is>
+      </c>
+      <c r="B9" s="2" t="inlineStr">
+        <is>
+          <t>F-140, GUI-50</t>
+        </is>
+      </c>
+      <c r="C9" s="2" t="inlineStr">
+        <is>
+          <t>Контактна форма: повідомлення з 251 символу (вище межі) не надсилається</t>
+        </is>
+      </c>
+      <c r="D9" s="2" t="inlineStr">
+        <is>
+          <t>Chrome 120 або новіший, вікно 1280×800; demo доступне (збірка v2.5 від 2026-10-11 за написом у підвалі сторінки; стан звірено 25.10.2026); обліковий запис не потрібен (звернення від анонімного відвідувача); дані лише вигадані.</t>
+        </is>
+      </c>
+      <c r="E9" s="2" t="inlineStr">
+        <is>
+          <t>1. Відкрити https://practicesoftwaretesting.com/contact у Chrome (нова сесія).
+2. У поле «Your first name» ввести: Test
+3. У поле «Your last name» ввести: Tester
+4. У поле «Your email» ввести: tester.tc012@example.com
+5. У списку «Select a subject» вибрати: Customer service
+6. У поле «Message» ввести 251 символ: abcdefghijabcdefghijabcdefghijabcdefghijabcdefghijabcdefghijabcdefghijabcdefghijabcdefghijabcdefghijabcdefghijabcdefghijabcdefghijabcdefghijabcdefghijabcdefghijabcdefghijabcdefghijabcdefghijabcdefghijabcdefghijabcdefghijabcdefghijabcdefghijabcdefghija
+7. Натиснути «Send».
+8. Закрити вкладку.</t>
+        </is>
+      </c>
+      <c r="F9" s="2" t="inlineStr">
+        <is>
+          <t>Після кроку 1: відкрито сторінку «Contact», усі поля порожні.
+Після кроків 2–5: у полях відображено введені значення: Test, Tester, tester.tc012@example.com, Customer service.
+Після кроку 6: у полі «Message» 251 символ.
+Після кроку 7: форму не надіслано, сторінка «Contact» залишається відкритою; під полем «Message» текстове повідомлення про помилку, яке називає межу в 250 символів (F-140, GUI-50; SRS 1.1 точного тексту не задає); під іншими полями повідомлень про помилки немає; повідомлення про прийняття звернення над формою відсутнє.
+Після кроку 8: вкладку закрито.</t>
+        </is>
+      </c>
+      <c r="G9" s="2" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="H9" s="2" t="inlineStr">
+        <is>
+          <t>негативний</t>
+        </is>
+      </c>
+      <c r="I9" s="2" t="inlineStr">
+        <is>
+          <t>251 — на 1 більше за верхню межу діапазону 50–250, клас недопустимих значень. Решта полів валідні.</t>
+        </is>
+      </c>
+      <c r="J9" s="2" t="inlineStr">
+        <is>
+          <t>Горбонос О. (КТ)</t>
+        </is>
+      </c>
       <c r="K9" s="2" t="n"/>
       <c r="L9" s="2" t="n"/>
-      <c r="M9" s="2" t="n"/>
+      <c r="M9" s="2" t="inlineStr">
+        <is>
+          <t>draft</t>
+        </is>
+      </c>
       <c r="N9" s="2" t="n"/>
     </row>
     <row r="10">
-      <c r="A10" s="2" t="n"/>
-      <c r="B10" s="2" t="n"/>
-      <c r="C10" s="2" t="n"/>
-      <c r="D10" s="2" t="n"/>
-      <c r="E10" s="2" t="n"/>
-      <c r="F10" s="2" t="n"/>
-      <c r="G10" s="2" t="n"/>
-      <c r="H10" s="2" t="n"/>
-      <c r="I10" s="2" t="n"/>
-      <c r="J10" s="2" t="n"/>
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t>TC-013</t>
+        </is>
+      </c>
+      <c r="B10" s="2" t="inlineStr">
+        <is>
+          <t>F-140, GUI-50</t>
+        </is>
+      </c>
+      <c r="C10" s="2" t="inlineStr">
+        <is>
+          <t>Контактна форма: вкладення недопустимого формату (.png) блокує надсилання</t>
+        </is>
+      </c>
+      <c r="D10" s="2" t="inlineStr">
+        <is>
+          <t>Chrome 120 або новіший, вікно 1280×800; demo доступне (збірка v2.5 від 2026-10-11 за написом у підвалі сторінки; стан звірено 25.10.2026); обліковий запис не потрібен (звернення від анонімного відвідувача); дані лише вигадані. На комп'ютері є файл note.png розміром до 100 КБ з вигаданим зображенням без особистих даних.</t>
+        </is>
+      </c>
+      <c r="E10" s="2" t="inlineStr">
+        <is>
+          <t>1. Відкрити https://practicesoftwaretesting.com/contact у Chrome (нова сесія).
+2. У поле «Your first name» ввести: Test
+3. У поле «Your last name» ввести: Tester
+4. У поле «Your email» ввести: tester.tc013@example.com
+5. У списку «Select a subject» вибрати: Customer service
+6. У поле «Message» ввести 50 символів: abcdefghijabcdefghijabcdefghijabcdefghijabcdefghij
+7. Натиснути кнопку вибору файла в полі «Attachment».
+8. У вікні вибору файла обрати файл note.png.
+9. Натиснути «Send».
+10. Закрити вкладку.</t>
+        </is>
+      </c>
+      <c r="F10" s="2" t="inlineStr">
+        <is>
+          <t>Після кроку 1: відкрито сторінку «Contact», усі поля порожні.
+Після кроків 2–5: у полях відображено введені значення: Test, Tester, tester.tc013@example.com, Customer service.
+Після кроку 6: у полі «Message» 50 символів (допустима довжина).
+Після кроку 7: відкрито вікно вибору файла.
+Після кроку 8: у полі «Attachment» відображається назва файла note.png.
+Після кроку 9: форму не надіслано, сторінка «Contact» залишається відкритою; біля поля «Attachment» текстове повідомлення про помилку: файл недопустимий (F-140, GUI-50); повідомлення про прийняття звернення над формою відсутнє.
+Після кроку 10: вкладку закрито.</t>
+        </is>
+      </c>
+      <c r="G10" s="2" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="H10" s="2" t="inlineStr">
+        <is>
+          <t>негативний</t>
+        </is>
+      </c>
+      <c r="I10" s="2" t="inlineStr">
+        <is>
+          <t>Файл .png — недопустимий формат (допускається один файл .txt до 500 КБ, F-140). Довжина повідомлення 50 і решта полів валідні, тож єдина причина відхилення — вкладення.</t>
+        </is>
+      </c>
+      <c r="J10" s="2" t="inlineStr">
+        <is>
+          <t>Горбонос О. (КТ)</t>
+        </is>
+      </c>
       <c r="K10" s="2" t="n"/>
       <c r="L10" s="2" t="n"/>
-      <c r="M10" s="2" t="n"/>
+      <c r="M10" s="2" t="inlineStr">
+        <is>
+          <t>draft</t>
+        </is>
+      </c>
       <c r="N10" s="2" t="n"/>
     </row>
     <row r="11">
-      <c r="A11" s="2" t="n"/>
-      <c r="B11" s="2" t="n"/>
-      <c r="C11" s="2" t="n"/>
-      <c r="D11" s="2" t="n"/>
-      <c r="E11" s="2" t="n"/>
-      <c r="F11" s="2" t="n"/>
-      <c r="G11" s="2" t="n"/>
-      <c r="H11" s="2" t="n"/>
-      <c r="I11" s="2" t="n"/>
-      <c r="J11" s="2" t="n"/>
+      <c r="A11" s="2" t="inlineStr">
+        <is>
+          <t>TC-014</t>
+        </is>
+      </c>
+      <c r="B11" s="2" t="inlineStr">
+        <is>
+          <t>F-100, GUI-70</t>
+        </is>
+      </c>
+      <c r="C11" s="2" t="inlineStr">
+        <is>
+          <t>Крок «Cart»: зміна кількості перераховує «Total», видалення рядка показує порожній кошик</t>
+        </is>
+      </c>
+      <c r="D11" s="2" t="inlineStr">
+        <is>
+          <t>Chrome 120 або новіший, вікно 1280×800; demo доступне (збірка v2.5 від 2026-10-11 за написом у підвалі сторінки; стан звірено 25.10.2026); кошик порожній (нова сесія); обліковий запис не потрібен; у каталозі є товар «Combination Pliers» (на збірці 2026-10-11 його ціна $14.15).</t>
+        </is>
+      </c>
+      <c r="E11" s="2" t="inlineStr">
+        <is>
+          <t>1. Відкрити https://practicesoftwaretesting.com/ у Chrome (нова сесія).
+2. У каталозі натиснути картку «Combination Pliers».
+3. На сторінці товару натиснути «Add to cart».
+4. У шапці натиснути піктограму кошика.
+5. У полі кількості рядка «Combination Pliers» замінити значення 1 на 3.
+6. Перемістити фокус з поля кількості, натиснувши Tab.
+7. Натиснути піктограму видалення в рядку «Combination Pliers».
+8. Закрити вкладку.</t>
+        </is>
+      </c>
+      <c r="F11" s="2" t="inlineStr">
+        <is>
+          <t>Після кроку 1: відкрито головну сторінку з каталогом; є картка «Combination Pliers».
+Після кроку 2: відкрито сторінку товару «Combination Pliers» з ціною і кнопкою «Add to cart».
+Після кроку 3: не пізніше ніж за 2 с виводиться повідомлення «Product added to shopping cart.» (F-90, SRS 1.1).
+Після кроку 4: відкрито крок «Cart»; таблиця має колонки «Item», «Quantity» (поле для редагування), «Price», «Total» і піктограму видалення; єдиний рядок: «Combination Pliers», кількість 1, ціна дорівнює ціні на сторінці товару (на збірці 2026-10-11 — $14.15), сума рядка дорівнює ціні; під таблицею підсумок «Total» дорівнює сумі рядка і кнопка «Proceed to checkout» (GUI-70).
+Після кроку 5: у полі кількості рядка «Combination Pliers» значення 3.
+Після кроку 6: сума рядка дорівнює 3 × ціна з кроку 4 (на збірці 2026-10-11 — $14.15 × 3 = $42.45), підсумок «Total» дорівнює сумі рядка; перерахунок виконано одразу після зміни кількості, без додаткових дій користувача (F-100).
+Після кроку 7: рядок «Combination Pliers» вилучено; таблиці немає; замість неї текстове повідомлення про порожній кошик (F-100, GUI-70).
+Після кроку 8: вкладку закрито.</t>
+        </is>
+      </c>
+      <c r="G11" s="2" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="H11" s="2" t="inlineStr">
+        <is>
+          <t>позитивний</t>
+        </is>
+      </c>
+      <c r="I11" s="2" t="inlineStr">
+        <is>
+          <t>Кількість 3 — типове значення допустимого класу 1–99; межі 0 / 1 / 99 / 100 перевіряють кейси GUI-30. Очікувана сума задана формулою (3 × ціна), бо ціна на demo може змінитися; числа $14.15 і $42.45 — приклад для збірки 2026-10-11.</t>
+        </is>
+      </c>
+      <c r="J11" s="2" t="inlineStr">
+        <is>
+          <t>Горбонос О. (КТ)</t>
+        </is>
+      </c>
       <c r="K11" s="2" t="n"/>
       <c r="L11" s="2" t="n"/>
-      <c r="M11" s="2" t="n"/>
+      <c r="M11" s="2" t="inlineStr">
+        <is>
+          <t>draft</t>
+        </is>
+      </c>
       <c r="N11" s="2" t="n"/>
     </row>
     <row r="12">
-      <c r="A12" s="2" t="n"/>
-      <c r="B12" s="2" t="n"/>
-      <c r="C12" s="2" t="n"/>
-      <c r="D12" s="2" t="n"/>
-      <c r="E12" s="2" t="n"/>
-      <c r="F12" s="2" t="n"/>
-      <c r="G12" s="2" t="n"/>
-      <c r="H12" s="2" t="n"/>
-      <c r="I12" s="2" t="n"/>
-      <c r="J12" s="2" t="n"/>
+      <c r="A12" s="2" t="inlineStr">
+        <is>
+          <t>TC-015</t>
+        </is>
+      </c>
+      <c r="B12" s="2" t="inlineStr">
+        <is>
+          <t>F-20, GUI-60, GUI-10</t>
+        </is>
+      </c>
+      <c r="C12" s="2" t="inlineStr">
+        <is>
+          <t>Вхід зареєстрованого покупця з правильною парою адреса — пароль</t>
+        </is>
+      </c>
+      <c r="D12" s="2" t="inlineStr">
+        <is>
+          <t>Chrome 120 або новіший, вікно 1280×800; demo доступне (збірка v2.5 від 2026-10-11 за написом у підвалі сторінки; стан звірено 26.10.2026); нова сесія, без входу; спільний обліковий запис покупця customer@practicesoftwaretesting.com / welcome01 (SRS 1.1, розд. 2.2); пароль спільного облікового запису не змінювати (методичка, п. 5.4).</t>
+        </is>
+      </c>
+      <c r="E12" s="2" t="inlineStr">
+        <is>
+          <t>1. Відкрити https://practicesoftwaretesting.com у Chrome (нова сесія).
+2. Натиснути «Sign in» у верхньому меню.
+3. У поле «Email address» ввести: customer@practicesoftwaretesting.com
+4. У поле «Password» ввести: welcome01
+5. Натиснути кнопку «Login».
+6. Натиснути ім'я користувача у верхньому меню.
+7. У розкривному меню натиснути «Sign out».
+8. Закрити вкладку.</t>
+        </is>
+      </c>
+      <c r="F12" s="2" t="inlineStr">
+        <is>
+          <t>Після кроку 1: головна сторінка з каталогом; у шапці логотип, пункти «Home», «Categories», «Contact», «Sign in» і перемикач мови (GUI-10).
+Після кроку 2: сторінка входу (адреса містить /auth/login): заголовок «Login»; поля «Email address» і «Password» (з кнопкою показати / приховати пароль); кнопки «Login» і «Sign in with Google»; посилання «Register your account» і «Forgot your Password?» (GUI-60).
+Після кроку 3: у полі «Email address» — customer@practicesoftwaretesting.com.
+Після кроку 4: символи пароля замасковано.
+Після кроку 5: відкрито сторінку особистого кабінету, адреса містить /account (F-20); у шапці замість «Sign in» — ім'я користувача (GUI-10).
+Після кроку 6: розкривне меню з розділами кабінету і пунктом «Sign out» (GUI-10).
+Після кроку 7: сеанс завершено; у шапці знову «Sign in».
+Після кроку 8: вкладку закрито.</t>
+        </is>
+      </c>
+      <c r="G12" s="2" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="H12" s="2" t="inlineStr">
+        <is>
+          <t>позитивний</t>
+        </is>
+      </c>
+      <c r="I12" s="2" t="inlineStr">
+        <is>
+          <t>Клас «правильна пара адреса — пароль» (F-20). Дані — тестовий обліковий запис покупця з SRS 1.1 (розд. 2.2); вхід і вихід не змінюють даних облікового запису. Вихід на кроці 7 лишає demo в початковому стані для наступних кейсів. Негативні пари — TC-016 (зареєстрована адреса, неправильний пароль) і TC-004 (незареєстрована адреса).</t>
+        </is>
+      </c>
+      <c r="J12" s="2" t="inlineStr">
+        <is>
+          <t>Тимчак А. (ІТ)</t>
+        </is>
+      </c>
       <c r="K12" s="2" t="n"/>
       <c r="L12" s="2" t="n"/>
-      <c r="M12" s="2" t="n"/>
+      <c r="M12" s="2" t="inlineStr">
+        <is>
+          <t>draft</t>
+        </is>
+      </c>
       <c r="N12" s="2" t="n"/>
     </row>
     <row r="13">
-      <c r="A13" s="2" t="n"/>
-      <c r="B13" s="2" t="n"/>
-      <c r="C13" s="2" t="n"/>
-      <c r="D13" s="2" t="n"/>
-      <c r="E13" s="2" t="n"/>
-      <c r="F13" s="2" t="n"/>
-      <c r="G13" s="2" t="n"/>
-      <c r="H13" s="2" t="n"/>
-      <c r="I13" s="2" t="n"/>
-      <c r="J13" s="2" t="n"/>
+      <c r="A13" s="2" t="inlineStr">
+        <is>
+          <t>TC-016</t>
+        </is>
+      </c>
+      <c r="B13" s="2" t="inlineStr">
+        <is>
+          <t>F-20</t>
+        </is>
+      </c>
+      <c r="C13" s="2" t="inlineStr">
+        <is>
+          <t>Вхід із зареєстрованою адресою і неправильним паролем</t>
+        </is>
+      </c>
+      <c r="D13" s="2" t="inlineStr">
+        <is>
+          <t>Chrome 120 або новіший, вікно 1280×800; demo доступне (збірка v2.5 від 2026-10-11 за написом у підвалі сторінки; стан звірено 26.10.2026); нова сесія, без входу. Адреса customer@practicesoftwaretesting.com зареєстрована на demo (SRS 1.1, розд. 2.2). Лише одна спроба з неправильним паролем за виконання кейсу, щоб не заблокувати спільний обліковий запис для інших користувачів demo (методичка, п. 5.4).</t>
+        </is>
+      </c>
+      <c r="E13" s="2" t="inlineStr">
+        <is>
+          <t>1. Відкрити https://practicesoftwaretesting.com у Chrome (нова сесія).
+2. Натиснути «Sign in» у верхньому меню.
+3. У поле «Email address» ввести: customer@practicesoftwaretesting.com
+4. У поле «Password» ввести: Wrong-pass1
+5. Натиснути кнопку «Login».
+6. Закрити вкладку.</t>
+        </is>
+      </c>
+      <c r="F13" s="2" t="inlineStr">
+        <is>
+          <t>Після кроку 1: головна сторінка з каталогом; у меню — «Sign in».
+Після кроку 2: сторінка входу (адреса містить /auth/login): поля «Email address» і «Password», кнопка «Login».
+Після кроку 3: у полі «Email address» — customer@practicesoftwaretesting.com.
+Після кроку 4: символи пароля замасковано.
+Після кроку 5: повідомлення «Invalid email or password» (F-20); адреса не змінилася (/auth/login); у меню — «Sign in» (сеанс не створено).
+Після кроку 6: вкладку закрито.</t>
+        </is>
+      </c>
+      <c r="G13" s="2" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="H13" s="2" t="inlineStr">
+        <is>
+          <t>негативний</t>
+        </is>
+      </c>
+      <c r="I13" s="2" t="inlineStr">
+        <is>
+          <t>Клас «зареєстрована адреса, неправильний пароль» (F-20) — інший клас, ніж у TC-004 (незареєстрована адреса): перевіряє, що для правильної адреси система показує те саме повідомлення і не створює сеанс. Пароль Wrong-pass1 вигаданий і відрізняється від welcome01. Позитивна пара — TC-015.</t>
+        </is>
+      </c>
+      <c r="J13" s="2" t="inlineStr">
+        <is>
+          <t>Тимчак А. (ІТ)</t>
+        </is>
+      </c>
       <c r="K13" s="2" t="n"/>
       <c r="L13" s="2" t="n"/>
-      <c r="M13" s="2" t="n"/>
+      <c r="M13" s="2" t="inlineStr">
+        <is>
+          <t>draft</t>
+        </is>
+      </c>
       <c r="N13" s="2" t="n"/>
     </row>
     <row r="14">
-      <c r="A14" s="2" t="n"/>
-      <c r="B14" s="2" t="n"/>
-      <c r="C14" s="2" t="n"/>
-      <c r="D14" s="2" t="n"/>
-      <c r="E14" s="2" t="n"/>
-      <c r="F14" s="2" t="n"/>
-      <c r="G14" s="2" t="n"/>
-      <c r="H14" s="2" t="n"/>
-      <c r="I14" s="2" t="n"/>
-      <c r="J14" s="2" t="n"/>
+      <c r="A14" s="2" t="inlineStr">
+        <is>
+          <t>TC-017</t>
+        </is>
+      </c>
+      <c r="B14" s="2" t="inlineStr">
+        <is>
+          <t>F-110</t>
+        </is>
+      </c>
+      <c r="C14" s="2" t="inlineStr">
+        <is>
+          <t>Оформлення замовлення у 4 кроки з входом на кроці «Sign in» і оплатою «Cash on Delivery»</t>
+        </is>
+      </c>
+      <c r="D14" s="2" t="inlineStr">
+        <is>
+          <t>Chrome 120 або новіший, вікно 1280×800; demo доступне (збірка v2.5 від 2026-10-11 за написом у підвалі сторінки; стан звірено 26.10.2026); нова сесія, без входу, кошик порожній; спільний обліковий запис покупця customer@practicesoftwaretesting.com / welcome01 (SRS 1.1, розд. 2.2); пароль спільного облікового запису не змінювати (методичка, п. 5.4). Товар «Combination Pliers» є в каталозі і в наявності. Адреса доставки вигадана.</t>
+        </is>
+      </c>
+      <c r="E14" s="2" t="inlineStr">
+        <is>
+          <t>1. Відкрити https://practicesoftwaretesting.com у Chrome (нова сесія).
+2. Натиснути картку товару «Combination Pliers».
+3. Натиснути кнопку «Add to cart».
+4. Натиснути піктограму кошика у верхньому меню.
+5. Натиснути «Proceed to checkout».
+6. У поле «Email address» ввести: customer@practicesoftwaretesting.com
+7. У поле «Password» ввести: welcome01
+8. Натиснути кнопку «Login».
+9. У поле «Street» ввести (замість поточного значення): Testova 1
+10. У поле «City» ввести (замість поточного значення): Kyiv
+11. У поле «State» ввести (замість поточного значення): Kyiv
+12. У поле «Country» ввести (замість поточного значення): Ukraine
+13. У поле «Postal code» ввести (замість поточного значення): 01001
+14. Натиснути «Proceed to checkout».
+15. У списку способів оплати вибрати «Cash on Delivery».
+16. Натиснути «Confirm».
+17. Закрити вкладку.</t>
+        </is>
+      </c>
+      <c r="F14" s="2" t="inlineStr">
+        <is>
+          <t>Після кроку 1: головна сторінка з каталогом; є картка «Combination Pliers».
+Після кроку 2: сторінка товару «Combination Pliers» з ціною і кнопкою «Add to cart».
+Після кроку 3: не пізніше ніж за 2 с — повідомлення «Product added to shopping cart.» (F-90).
+Після кроку 4: крок «Cart» (1 з 4); над таблицею — чотири кроки «Cart», «Sign in», «Billing Address», «Payment» (F-110); один рядок «Combination Pliers», кількість 1, «Total» дорівнює ціні з кроку 2 (сума товарів, F-110).
+Після кроку 5: крок «Sign in» (2 з 4): форма входу з полями «Email address» і «Password», кнопка «Login».
+Після кроку 6: у полі «Email address» — customer@practicesoftwaretesting.com.
+Після кроку 7: символи пароля замасковано.
+Після кроку 8: вхід виконано, відкрито крок «Billing Address» (3 з 4) (F-20, F-110); є поля «Street», «City», «State», «Country», «Postal code».
+Після кроків 9–13: у полях відображено введені значення: Testova 1, Kyiv, Kyiv, Ukraine, 01001.
+Після кроку 14: крок «Payment» (4 з 4); список способів оплати містить банківський переказ, оплату при отриманні, кредитну картку, «купити зараз — заплатити пізніше» і подарункову картку (F-110).
+Після кроку 15: вибрано «Cash on Delivery»; кнопка «Confirm» доступна.
+Після кроку 16: замовлення підтверджено; показано текстове повідомлення з номером рахунку-інвойсу (F-110; SRS 1.1 точного тексту не задає).
+Після кроку 17: вкладку закрито.</t>
+        </is>
+      </c>
+      <c r="G14" s="2" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="H14" s="2" t="inlineStr">
+        <is>
+          <t>позитивний</t>
+        </is>
+      </c>
+      <c r="I14" s="2" t="inlineStr">
+        <is>
+          <t>Основний сценарій F-110: неавторизований покупець проходить усі 4 кроки і входить на кроці 2 (клас «вхід під час оформлення»). Оплата при отриманні не потребує платіжних даних; реальна оплата на demo не проводиться (SRS 1.1, розд. 2.3). Адреса вигадана, поля заповнюються явно, щоб кейс не залежав від даних профілю. Знижки і вартість доставки (BL-50 – BL-80) не перевіряються: модуль лояльності не інтегровано в demo (SRS 1.1, розд. 2.3).</t>
+        </is>
+      </c>
+      <c r="J14" s="2" t="inlineStr">
+        <is>
+          <t>Тимчак А. (ІТ)</t>
+        </is>
+      </c>
       <c r="K14" s="2" t="n"/>
       <c r="L14" s="2" t="n"/>
-      <c r="M14" s="2" t="n"/>
+      <c r="M14" s="2" t="inlineStr">
+        <is>
+          <t>draft</t>
+        </is>
+      </c>
       <c r="N14" s="2" t="n"/>
     </row>
     <row r="15">
-      <c r="A15" s="2" t="n"/>
-      <c r="B15" s="2" t="n"/>
-      <c r="C15" s="2" t="n"/>
-      <c r="D15" s="2" t="n"/>
-      <c r="E15" s="2" t="n"/>
-      <c r="F15" s="2" t="n"/>
-      <c r="G15" s="2" t="n"/>
-      <c r="H15" s="2" t="n"/>
-      <c r="I15" s="2" t="n"/>
-      <c r="J15" s="2" t="n"/>
+      <c r="A15" s="2" t="inlineStr">
+        <is>
+          <t>TC-018</t>
+        </is>
+      </c>
+      <c r="B15" s="2" t="inlineStr">
+        <is>
+          <t>GUI-40, F-120</t>
+        </is>
+      </c>
+      <c r="C15" s="2" t="inlineStr">
+        <is>
+          <t>«Add to favourites» без входу: повідомлення про відмову, товар не додано</t>
+        </is>
+      </c>
+      <c r="D15" s="2" t="inlineStr">
+        <is>
+          <t>Chrome 120 або новіший, вікно 1280×800; demo доступне (збірка v2.5 від 2026-10-11 за написом у підвалі сторінки; стан звірено 26.10.2026); нова сесія, без входу. Товар «Combination Pliers» є в каталозі.</t>
+        </is>
+      </c>
+      <c r="E15" s="2" t="inlineStr">
+        <is>
+          <t>1. Відкрити https://practicesoftwaretesting.com у Chrome (нова сесія).
+2. Натиснути картку товару «Combination Pliers».
+3. Натиснути кнопку «Add to favourites».
+4. Закрити вкладку.</t>
+        </is>
+      </c>
+      <c r="F15" s="2" t="inlineStr">
+        <is>
+          <t>Після кроку 1: головна сторінка з каталогом; у меню — «Sign in»; є картка «Combination Pliers».
+Після кроку 2: сторінка товару «Combination Pliers»; кнопка «Add to favourites» відображається (GUI-40).
+Після кроку 3: повідомлення «Unauthorized, can not add product to your favorite list» (GUI-40); відкрита та сама сторінка товару; у меню — «Sign in» (товар до обраного не додано, F-120).
+Після кроку 4: вкладку закрито.</t>
+        </is>
+      </c>
+      <c r="G15" s="2" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="H15" s="2" t="inlineStr">
+        <is>
+          <t>негативний</t>
+        </is>
+      </c>
+      <c r="I15" s="2" t="inlineStr">
+        <is>
+          <t>Клас «неавторизований покупець» для F-120 / GUI-40. Текст повідомлення — з GUI-40 SRS 1.1; на demo 26.10.2026 він виводиться з крапкою в кінці. Позитивна пара (додавання після входу, перегляд у «My favorites», видалення) — резервний кейс ІТ (TC-025+).</t>
+        </is>
+      </c>
+      <c r="J15" s="2" t="inlineStr">
+        <is>
+          <t>Тимчак А. (ІТ)</t>
+        </is>
+      </c>
       <c r="K15" s="2" t="n"/>
       <c r="L15" s="2" t="n"/>
-      <c r="M15" s="2" t="n"/>
+      <c r="M15" s="2" t="inlineStr">
+        <is>
+          <t>draft</t>
+        </is>
+      </c>
       <c r="N15" s="2" t="n"/>
     </row>
     <row r="16">
-      <c r="A16" s="2" t="n"/>
-      <c r="B16" s="2" t="n"/>
-      <c r="C16" s="2" t="n"/>
-      <c r="D16" s="2" t="n"/>
-      <c r="E16" s="2" t="n"/>
-      <c r="F16" s="2" t="n"/>
-      <c r="G16" s="2" t="n"/>
-      <c r="H16" s="2" t="n"/>
-      <c r="I16" s="2" t="n"/>
-      <c r="J16" s="2" t="n"/>
+      <c r="A16" s="2" t="inlineStr">
+        <is>
+          <t>TC-019</t>
+        </is>
+      </c>
+      <c r="B16" s="2" t="inlineStr">
+        <is>
+          <t>F-30</t>
+        </is>
+      </c>
+      <c r="C16" s="2" t="inlineStr">
+        <is>
+          <t>Форма відновлення пароля: перехід за посиланням «Forgot your Password?» і надсилання адреси</t>
+        </is>
+      </c>
+      <c r="D16" s="2" t="inlineStr">
+        <is>
+          <t>Chrome 120 або новіший, вікно 1280×800; demo доступне (збірка v2.5 від 2026-10-11 за написом у підвалі сторінки; стан звірено 26.10.2026); нова сесія, без входу. Обліковий запис shopline.it.tc019@example.com зареєстровано заздалегідь через «Register your account» з вигаданими даними. Спільні облікові записи customer@… і admin@… не використовувати: відновлення може змінити їхній пароль (методичка, п. 5.4). Доставку листа на demo не спостерігаємо: адреса вигадана.</t>
+        </is>
+      </c>
+      <c r="E16" s="2" t="inlineStr">
+        <is>
+          <t>1. Відкрити https://practicesoftwaretesting.com у Chrome (нова сесія).
+2. Натиснути «Sign in» у верхньому меню.
+3. Натиснути посилання «Forgot your Password?».
+4. У поле «Email address» ввести: shopline.it.tc019@example.com
+5. Натиснути кнопку «Set New Password».
+6. Закрити вкладку.</t>
+        </is>
+      </c>
+      <c r="F16" s="2" t="inlineStr">
+        <is>
+          <t>Після кроку 1: головна сторінка з каталогом; у меню — «Sign in».
+Після кроку 2: сторінка входу (адреса містить /auth/login); є посилання «Forgot your Password?».
+Після кроку 3: відкрито форму відновлення пароля (адреса містить /auth/forgot-password): заголовок «Forgot Password», поле «Email address», кнопка «Set New Password» (F-30).
+Після кроку 4: у полі «Email address» — shopline.it.tc019@example.com.
+Після кроку 5: форму надіслано; на сторінці текстове повідомлення про надсилання листа для встановлення нового пароля (F-30; SRS 1.1 точного тексту не задає); повідомлень про помилку під полем немає.
+Після кроку 6: вкладку закрито.</t>
+        </is>
+      </c>
+      <c r="G16" s="2" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="H16" s="2" t="inlineStr">
+        <is>
+          <t>позитивний</t>
+        </is>
+      </c>
+      <c r="I16" s="2" t="inlineStr">
+        <is>
+          <t>Клас «зареєстрована адреса» для F-30. Через UI спостерігаються форма і реакція сторінки після надсилання; час передачі листа поштовому сервісу (1 с) і доставку на demo перевірити не можна (Coverage, примітка до F-30). Адреса вигадана з домену example.com.</t>
+        </is>
+      </c>
+      <c r="J16" s="2" t="inlineStr">
+        <is>
+          <t>Тимчак А. (ІТ)</t>
+        </is>
+      </c>
       <c r="K16" s="2" t="n"/>
       <c r="L16" s="2" t="n"/>
-      <c r="M16" s="2" t="n"/>
+      <c r="M16" s="2" t="inlineStr">
+        <is>
+          <t>draft</t>
+        </is>
+      </c>
       <c r="N16" s="2" t="n"/>
     </row>
     <row r="17">
-      <c r="A17" s="2" t="n"/>
-      <c r="B17" s="2" t="n"/>
-      <c r="C17" s="2" t="n"/>
-      <c r="D17" s="2" t="n"/>
-      <c r="E17" s="2" t="n"/>
-      <c r="F17" s="2" t="n"/>
-      <c r="G17" s="2" t="n"/>
-      <c r="H17" s="2" t="n"/>
-      <c r="I17" s="2" t="n"/>
-      <c r="J17" s="2" t="n"/>
+      <c r="A17" s="2" t="inlineStr">
+        <is>
+          <t>TC-020</t>
+        </is>
+      </c>
+      <c r="B17" s="2" t="inlineStr">
+        <is>
+          <t>F-40, GUI-20</t>
+        </is>
+      </c>
+      <c r="C17" s="2" t="inlineStr">
+        <is>
+          <t>Каталог на головній сторінці: 9 карток у три колонки, вміст картки, посторінкова навігація</t>
+        </is>
+      </c>
+      <c r="D17" s="2" t="inlineStr">
+        <is>
+          <t>Chrome 120 або новіший, вікно 1280×800; demo доступне (збірка v2.5 від 2026-10-11 за написом у підвалі сторінки, стан зафіксовано ІТ 26.10.2026); нова сесія, без входу. Активних фільтрів, сортування і пошукового запиту немає; у каталозі понад 9 товарів.</t>
+        </is>
+      </c>
+      <c r="E17" s="2" t="inlineStr">
+        <is>
+          <t>1. Відкрити https://practicesoftwaretesting.com у Chrome (нова сесія).
+2. Порахувати картки товарів на сторінці 1 і записати назви першої та останньої.
+3. У посторінковій навігації під каталогом натиснути «2».
+4. Натиснути кнопку ««» у посторінковій навігації.
+5. Натиснути першу картку на сторінці.
+6. Закрити вкладку.</t>
+        </is>
+      </c>
+      <c r="F17" s="2" t="inlineStr">
+        <is>
+          <t>Після кроку 1: головна сторінка з каталогом; під каталогом — посторінкова навігація з номерами сторінок і кнопками ««» і «»» (F-40).
+Після кроку 2: на сторінці рівно 9 карток, розміщених сіткою у три колонки (3 ряди по 3) (F-40, GUI-20); кожна картка містить зображення, назву, шкалу класу CO2 і ціну (GUI-20).
+Після кроку 3: відкрито сторінку 2; на ній 9 карток (або менше, якщо сторінка остання); жодна назва не збігається з назвами першої та останньої карток із кроку 2.
+Після кроку 4: знову відкрито сторінку 1; перша й остання картки мають ті самі назви, що на кроці 2.
+Після кроку 5: відкрито сторінку товару з тією самою назвою, що на картці (F-40).
+Після кроку 6: вкладку закрито.</t>
+        </is>
+      </c>
+      <c r="G17" s="2" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="H17" s="2" t="inlineStr">
+        <is>
+          <t>позитивний</t>
+        </is>
+      </c>
+      <c r="I17" s="2" t="inlineStr">
+        <is>
+          <t>Кількість 9 і сітка у 3 колонки — з F-40 і GUI-20. Порівняння назв сторінок 1 і 2 перевіряє, що навігація показує інші товари, а повернення ««» — що сторінка 1 стабільна. «Out of stock» не перевіряємо: SRS не називає товару з нульовим залишком (task-board.md, розд. 3).</t>
+        </is>
+      </c>
+      <c r="J17" s="2" t="inlineStr">
+        <is>
+          <t>Дрєпіна А. (СМ)</t>
+        </is>
+      </c>
       <c r="K17" s="2" t="n"/>
       <c r="L17" s="2" t="n"/>
-      <c r="M17" s="2" t="n"/>
+      <c r="M17" s="2" t="inlineStr">
+        <is>
+          <t>draft</t>
+        </is>
+      </c>
       <c r="N17" s="2" t="n"/>
     </row>
     <row r="18">
-      <c r="A18" s="2" t="n"/>
-      <c r="B18" s="2" t="n"/>
-      <c r="C18" s="2" t="n"/>
-      <c r="D18" s="2" t="n"/>
-      <c r="E18" s="2" t="n"/>
-      <c r="F18" s="2" t="n"/>
-      <c r="G18" s="2" t="n"/>
-      <c r="H18" s="2" t="n"/>
-      <c r="I18" s="2" t="n"/>
-      <c r="J18" s="2" t="n"/>
+      <c r="A18" s="2" t="inlineStr">
+        <is>
+          <t>TC-021</t>
+        </is>
+      </c>
+      <c r="B18" s="2" t="inlineStr">
+        <is>
+          <t>F-50</t>
+        </is>
+      </c>
+      <c r="C18" s="2" t="inlineStr">
+        <is>
+          <t>Фільтр за однією категорією «Power Tools» звужує каталог без перезавантаження сторінки</t>
+        </is>
+      </c>
+      <c r="D18" s="2" t="inlineStr">
+        <is>
+          <t>Chrome 120 або новіший, вікно 1280×800; demo доступне (збірка v2.5 від 2026-10-11 за написом у підвалі сторінки, стан зафіксовано ІТ 26.10.2026); нова сесія, без входу. Активних фільтрів, сортування і пошукового запиту немає.</t>
+        </is>
+      </c>
+      <c r="E18" s="2" t="inlineStr">
+        <is>
+          <t>1. Відкрити https://practicesoftwaretesting.com у Chrome (нова сесія).
+2. У блоці фільтрів за категорією записати назви підкатегорій під прапорцем «Power Tools».
+3. Позначити прапорець «Power Tools».
+4. Порахувати картки на сторінці 1.
+5. Натиснути першу картку на сторінці.
+6. Закрити вкладку.</t>
+        </is>
+      </c>
+      <c r="F18" s="2" t="inlineStr">
+        <is>
+          <t>Після кроку 1: головна сторінка з каталогом; ліворуч блок фільтрів із прапорцями груп «Hand Tools», «Power Tools», «Other» і їх підкатегорій, прапорцями брендів, повзунком ціни і «Eco-Friendly Products» (F-50).
+Після кроку 2: під «Power Tools» є щонайменше одна підкатегорія; назви записано.
+Після кроку 3: прапорець «Power Tools» позначено; список карток оновився без перезавантаження сторінки (сторінка не стає порожньою, позначка прапорця і прокрутка зберігаються) (F-50).
+Після кроку 4: на сторінці від 1 до 9 карток (F-40).
+Після кроку 5: сторінка товару; поле категорії — «Power Tools» або одна з підкатегорій, записаних на кроці 2 (F-50, F-80).
+Після кроку 6: вкладку закрито.</t>
+        </is>
+      </c>
+      <c r="G18" s="2" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="H18" s="2" t="inlineStr">
+        <is>
+          <t>позитивний</t>
+        </is>
+      </c>
+      <c r="I18" s="2" t="inlineStr">
+        <is>
+          <t>Клас «одна категорія, без інших фільтрів»: один набір даних (task-board.md, розд. 3). Категорію товару на картці не видно, тому її перевіряємо на сторінці товару (F-80). «Power Tools» обрано як групу з підкатегоріями: перевіряє, що фільтр групи охоплює підкатегорії. Повзунок ціни 1–200 — резервний кейс КТ.</t>
+        </is>
+      </c>
+      <c r="J18" s="2" t="inlineStr">
+        <is>
+          <t>Дрєпіна А. (СМ)</t>
+        </is>
+      </c>
       <c r="K18" s="2" t="n"/>
       <c r="L18" s="2" t="n"/>
-      <c r="M18" s="2" t="n"/>
+      <c r="M18" s="2" t="inlineStr">
+        <is>
+          <t>draft</t>
+        </is>
+      </c>
       <c r="N18" s="2" t="n"/>
     </row>
     <row r="19">
-      <c r="A19" s="2" t="n"/>
-      <c r="B19" s="2" t="n"/>
-      <c r="C19" s="2" t="n"/>
-      <c r="D19" s="2" t="n"/>
-      <c r="E19" s="2" t="n"/>
-      <c r="F19" s="2" t="n"/>
-      <c r="G19" s="2" t="n"/>
-      <c r="H19" s="2" t="n"/>
-      <c r="I19" s="2" t="n"/>
-      <c r="J19" s="2" t="n"/>
+      <c r="A19" s="2" t="inlineStr">
+        <is>
+          <t>TC-022</t>
+        </is>
+      </c>
+      <c r="B19" s="2" t="inlineStr">
+        <is>
+          <t>F-60</t>
+        </is>
+      </c>
+      <c r="C19" s="2" t="inlineStr">
+        <is>
+          <t>Пошук «Hammer» з результатом і очищення запиту кнопкою «X» повертає повний каталог</t>
+        </is>
+      </c>
+      <c r="D19" s="2" t="inlineStr">
+        <is>
+          <t>Chrome 120 або новіший, вікно 1280×800; demo доступне (збірка v2.5 від 2026-10-11 за написом у підвалі сторінки, стан зафіксовано ІТ 26.10.2026); нова сесія, без входу. Активних фільтрів і сортування немає; у каталозі є товари зі словом «Hammer» у назві.</t>
+        </is>
+      </c>
+      <c r="E19" s="2" t="inlineStr">
+        <is>
+          <t>1. Відкрити https://practicesoftwaretesting.com у Chrome (нова сесія).
+2. Записати назву першої картки каталогу.
+3. У поле пошуку «Search» ввести: Hammer
+4. Натиснути кнопку «Search».
+5. Натиснути кнопку «X» біля поля пошуку.
+6. Закрити вкладку.</t>
+        </is>
+      </c>
+      <c r="F19" s="2" t="inlineStr">
+        <is>
+          <t>Після кроку 1: головна сторінка з каталогом, полем «Search» і кнопками «X» та «Search».
+Після кроку 2: назву записано.
+Після кроку 3: у полі «Search» — Hammer.
+Після кроку 4: результати під заголовком «Searched for: Hammer»; є щонайменше одна картка; назва кожної картки містить «hammer» без урахування регістру; карток без цього слова немає (F-60).
+Після кроку 5: поле «Search» порожнє; заголовка «Searched for:» немає; показано повний каталог, перша картка має ту саму назву, що на кроці 2 (F-60).
+Після кроку 6: вкладку закрито.</t>
+        </is>
+      </c>
+      <c r="G19" s="2" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="H19" s="2" t="inlineStr">
+        <is>
+          <t>позитивний</t>
+        </is>
+      </c>
+      <c r="I19" s="2" t="inlineStr">
+        <is>
+          <t>Клас «підрядок, що є в назвах». Кейс доповнює TC-001 (регістр літер): тут перевіряється кнопка «X» і повернення повного каталогу. Негативна пара (запит без результатів) — резервний кейс СМ (TC-025+).</t>
+        </is>
+      </c>
+      <c r="J19" s="2" t="inlineStr">
+        <is>
+          <t>Дрєпіна А. (СМ)</t>
+        </is>
+      </c>
       <c r="K19" s="2" t="n"/>
       <c r="L19" s="2" t="n"/>
-      <c r="M19" s="2" t="n"/>
+      <c r="M19" s="2" t="inlineStr">
+        <is>
+          <t>draft</t>
+        </is>
+      </c>
       <c r="N19" s="2" t="n"/>
     </row>
     <row r="20">
-      <c r="A20" s="2" t="n"/>
-      <c r="B20" s="2" t="n"/>
-      <c r="C20" s="2" t="n"/>
-      <c r="D20" s="2" t="n"/>
-      <c r="E20" s="2" t="n"/>
-      <c r="F20" s="2" t="n"/>
-      <c r="G20" s="2" t="n"/>
-      <c r="H20" s="2" t="n"/>
-      <c r="I20" s="2" t="n"/>
-      <c r="J20" s="2" t="n"/>
+      <c r="A20" s="2" t="inlineStr">
+        <is>
+          <t>TC-023</t>
+        </is>
+      </c>
+      <c r="B20" s="2" t="inlineStr">
+        <is>
+          <t>F-70</t>
+        </is>
+      </c>
+      <c r="C20" s="2" t="inlineStr">
+        <is>
+          <t>Сортування каталогу Price (Low–High) застосовується до сторінок 1 і 2 без входу</t>
+        </is>
+      </c>
+      <c r="D20" s="2" t="inlineStr">
+        <is>
+          <t>Chrome 120 або новіший, вікно 1280×800; demo доступне (збірка v2.5 від 2026-10-11 за написом у підвалі сторінки, стан зафіксовано ІТ 26.10.2026); нова сесія, без входу. Активних фільтрів і пошукового запиту немає; у каталозі не менше двох сторінок.</t>
+        </is>
+      </c>
+      <c r="E20" s="2" t="inlineStr">
+        <is>
+          <t>1. Відкрити https://practicesoftwaretesting.com у Chrome (нова сесія).
+2. У списку «Sort» вибрати: Price (Low–High).
+3. Записати ціни всіх карток сторінки 1 у порядку зліва направо, згори донизу.
+4. У посторінковій навігації під каталогом натиснути «2».
+5. Записати ціни всіх карток сторінки 2 у тому самому порядку.
+6. Закрити вкладку.</t>
+        </is>
+      </c>
+      <c r="F20" s="2" t="inlineStr">
+        <is>
+          <t>Після кроку 1: головна сторінка з каталогом; є список «Sort» і посторінкова навігація.
+Після кроку 2: у списку «Sort» показано Price (Low–High); список містить рівно шість варіантів: Name (A–Z), Name (Z–A), Price (High–Low), Price (Low–High), CO2 Rating (A–E), CO2 Rating (E–A) (F-70); каталог оновлено.
+Після кроку 3: кожна наступна ціна не менша за попередню.
+Після кроку 4: відкрито сторінку 2; у списку «Sort» і далі вибрано Price (Low–High).
+Після кроку 5: кожна наступна ціна не менша за попередню; перша ціна сторінки 2 не менша за останню ціну сторінки 1 (порядок застосовано до всіх сторінок, F-70).
+Після кроку 6: вкладку закрито.</t>
+        </is>
+      </c>
+      <c r="G20" s="2" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="H20" s="2" t="inlineStr">
+        <is>
+          <t>позитивний</t>
+        </is>
+      </c>
+      <c r="I20" s="2" t="inlineStr">
+        <is>
+          <t>Price (Low–High) обрано, бо порядок перевіряється числами, які видно на картках. Перевірка межі сторінок 1 і 2 покриває умову F-70 «застосовується до всіх сторінок». Конкретні ціни не задано: вони надходять із системи обліку і можуть змінитися (SRS 1.1, розд. 2.3).</t>
+        </is>
+      </c>
+      <c r="J20" s="2" t="inlineStr">
+        <is>
+          <t>Дрєпіна А. (СМ)</t>
+        </is>
+      </c>
       <c r="K20" s="2" t="n"/>
       <c r="L20" s="2" t="n"/>
-      <c r="M20" s="2" t="n"/>
+      <c r="M20" s="2" t="inlineStr">
+        <is>
+          <t>draft</t>
+        </is>
+      </c>
       <c r="N20" s="2" t="n"/>
     </row>
     <row r="21">
-      <c r="A21" s="2" t="n"/>
-      <c r="B21" s="2" t="n"/>
-      <c r="C21" s="2" t="n"/>
-      <c r="D21" s="2" t="n"/>
-      <c r="E21" s="2" t="n"/>
-      <c r="F21" s="2" t="n"/>
-      <c r="G21" s="2" t="n"/>
-      <c r="H21" s="2" t="n"/>
-      <c r="I21" s="2" t="n"/>
-      <c r="J21" s="2" t="n"/>
+      <c r="A21" s="2" t="inlineStr">
+        <is>
+          <t>TC-024</t>
+        </is>
+      </c>
+      <c r="B21" s="2" t="inlineStr">
+        <is>
+          <t>F-80, F-90</t>
+        </is>
+      </c>
+      <c r="C21" s="2" t="inlineStr">
+        <is>
+          <t>Сторінка товару «Combination Pliers»: склад даних і кнопок, одне додавання в кошик із кількістю 1</t>
+        </is>
+      </c>
+      <c r="D21" s="2" t="inlineStr">
+        <is>
+          <t>Chrome 120 або новіший, вікно 1280×800; demo доступне (збірка v2.5 від 2026-10-11 за написом у підвалі сторінки, стан зафіксовано ІТ 26.10.2026); нова сесія, без входу. Кошик порожній; товар «Combination Pliers» є в каталозі і в наявності.</t>
+        </is>
+      </c>
+      <c r="E21" s="2" t="inlineStr">
+        <is>
+          <t>1. Відкрити https://practicesoftwaretesting.com у Chrome (нова сесія).
+2. Натиснути картку товару «Combination Pliers».
+3. Натиснути кнопку «Add to cart».
+4. Натиснути піктограму кошика у верхньому меню.
+5. Закрити вкладку.</t>
+        </is>
+      </c>
+      <c r="F21" s="2" t="inlineStr">
+        <is>
+          <t>Після кроку 1: головна сторінка з каталогом; є картка «Combination Pliers».
+Після кроку 2: сторінка товару містить назву «Combination Pliers», категорію, бренд, ціну, клас CO2 (одна з літер A–E), опис, таблицю характеристик і блок «Related products»; поле «Quantity» зі значенням 1 і кнопками «−» і «+»; кнопки «Add to cart» (доступна), «Add to favourites», «Compare» (F-80).
+Після кроку 3: не пізніше ніж за 2 с — повідомлення «Product added to shopping cart.» (F-90); на піктограмі кошика в меню — 1.
+Після кроку 4: крок «Cart»: один рядок «Combination Pliers», кількість 1 (кількість із поля «Quantity», F-90); ціна дорівнює ціні з кроку 2.
+Після кроку 5: вкладку закрито.</t>
+        </is>
+      </c>
+      <c r="G21" s="2" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="H21" s="2" t="inlineStr">
+        <is>
+          <t>позитивний</t>
+        </is>
+      </c>
+      <c r="I21" s="2" t="inlineStr">
+        <is>
+          <t>Товар у наявності (ІТ і КТ використовують його у TC-014, TC-017), тож «Add to cart» має бути доступна. Одне додавання з кількістю за замовчуванням 1 — один набір даних (task-board.md, розд. 3). Повторне додавання (F-90, BL-20) — резервний кейс СМ (TC-025+).</t>
+        </is>
+      </c>
+      <c r="J21" s="2" t="inlineStr">
+        <is>
+          <t>Дрєпіна А. (СМ)</t>
+        </is>
+      </c>
       <c r="K21" s="2" t="n"/>
       <c r="L21" s="2" t="n"/>
-      <c r="M21" s="2" t="n"/>
+      <c r="M21" s="2" t="inlineStr">
+        <is>
+          <t>draft</t>
+        </is>
+      </c>
       <c r="N21" s="2" t="n"/>
     </row>
     <row r="22">
@@ -2425,4 +3546,1237 @@
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:N23"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="9" customWidth="1" min="1" max="1"/>
+    <col width="17" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="5" customWidth="1" min="4" max="4"/>
+    <col width="5" customWidth="1" min="5" max="5"/>
+    <col width="5" customWidth="1" min="6" max="6"/>
+    <col width="5" customWidth="1" min="7" max="7"/>
+    <col width="5" customWidth="1" min="8" max="8"/>
+    <col width="5" customWidth="1" min="9" max="9"/>
+    <col width="5" customWidth="1" min="10" max="10"/>
+    <col width="5" customWidth="1" min="11" max="11"/>
+    <col width="70" customWidth="1" min="12" max="12"/>
+    <col width="12" customWidth="1" min="13" max="13"/>
+    <col width="16" customWidth="1" min="14" max="14"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="5" t="inlineStr">
+        <is>
+          <t>TC-ID</t>
+        </is>
+      </c>
+      <c r="B1" s="5" t="inlineStr">
+        <is>
+          <t>Рецензент</t>
+        </is>
+      </c>
+      <c r="C1" s="5" t="inlineStr">
+        <is>
+          <t>Дата</t>
+        </is>
+      </c>
+      <c r="D1" s="5" t="inlineStr">
+        <is>
+          <t>П1</t>
+        </is>
+      </c>
+      <c r="E1" s="5" t="inlineStr">
+        <is>
+          <t>П2</t>
+        </is>
+      </c>
+      <c r="F1" s="5" t="inlineStr">
+        <is>
+          <t>П3</t>
+        </is>
+      </c>
+      <c r="G1" s="5" t="inlineStr">
+        <is>
+          <t>П4</t>
+        </is>
+      </c>
+      <c r="H1" s="5" t="inlineStr">
+        <is>
+          <t>П5</t>
+        </is>
+      </c>
+      <c r="I1" s="5" t="inlineStr">
+        <is>
+          <t>П6</t>
+        </is>
+      </c>
+      <c r="J1" s="5" t="inlineStr">
+        <is>
+          <t>П7</t>
+        </is>
+      </c>
+      <c r="K1" s="5" t="inlineStr">
+        <is>
+          <t>П8</t>
+        </is>
+      </c>
+      <c r="L1" s="5" t="inlineStr">
+        <is>
+          <t>Зауваження</t>
+        </is>
+      </c>
+      <c r="M1" s="5" t="inlineStr">
+        <is>
+          <t>Виправлено</t>
+        </is>
+      </c>
+      <c r="N1" s="5" t="inlineStr">
+        <is>
+          <t>Дата повторного підтвердження</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>TC-001</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>Дрєпіна А. (СМ)</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>27.10.2026</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>так</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>так</t>
+        </is>
+      </c>
+      <c r="F2" s="2" t="inlineStr">
+        <is>
+          <t>так</t>
+        </is>
+      </c>
+      <c r="G2" s="6" t="inlineStr">
+        <is>
+          <t>ні</t>
+        </is>
+      </c>
+      <c r="H2" s="2" t="inlineStr">
+        <is>
+          <t>так</t>
+        </is>
+      </c>
+      <c r="I2" s="2" t="inlineStr">
+        <is>
+          <t>так</t>
+        </is>
+      </c>
+      <c r="J2" s="2" t="inlineStr">
+        <is>
+          <t>так</t>
+        </is>
+      </c>
+      <c r="K2" s="2" t="inlineStr">
+        <is>
+          <t>так</t>
+        </is>
+      </c>
+      <c r="L2" s="2" t="inlineStr">
+        <is>
+          <t>П4: браузер без версії («поточна стабільна версія») і без розміру вікна, не вказано збірку та дату стану demo. Узгодити з рештою кейсів: «Chrome 120 або новіший, вікно 1280×800; збірка v2.5 від 2026-10-11».
+Поза чек-листом (для КТ): за task-board.md, розд. 3, ТА пише TC-001–004 за F-10/GUI-65 і TC-005–008 за GUI-30 (0 / 1 / 99 / 100), а F-60 належить СМ. Фактичні TC-001–004 не збігаються з розподілом; TC-005–008 у файлі немає.</t>
+        </is>
+      </c>
+      <c r="M2" s="2" t="n"/>
+      <c r="N2" s="2" t="n"/>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>TC-002</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>Дрєпіна А. (СМ)</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>27.10.2026</t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t>так</t>
+        </is>
+      </c>
+      <c r="E3" s="2" t="inlineStr">
+        <is>
+          <t>так</t>
+        </is>
+      </c>
+      <c r="F3" s="2" t="inlineStr">
+        <is>
+          <t>так</t>
+        </is>
+      </c>
+      <c r="G3" s="6" t="inlineStr">
+        <is>
+          <t>ні</t>
+        </is>
+      </c>
+      <c r="H3" s="2" t="inlineStr">
+        <is>
+          <t>так</t>
+        </is>
+      </c>
+      <c r="I3" s="2" t="inlineStr">
+        <is>
+          <t>так</t>
+        </is>
+      </c>
+      <c r="J3" s="2" t="inlineStr">
+        <is>
+          <t>так</t>
+        </is>
+      </c>
+      <c r="K3" s="2" t="inlineStr">
+        <is>
+          <t>так</t>
+        </is>
+      </c>
+      <c r="L3" s="2" t="inlineStr">
+        <is>
+          <t>П4: браузер без версії («поточна стабільна версія») і без розміру вікна, не вказано збірку та дату стану demo. Узгодити з рештою кейсів: «Chrome 120 або новіший, вікно 1280×800; збірка v2.5 від 2026-10-11».
+Поза чек-листом: за task-board.md кейси GUI-30 мають номери TC-005–008; нижня межа (0 / 1) ще не покрита.</t>
+        </is>
+      </c>
+      <c r="M3" s="2" t="n"/>
+      <c r="N3" s="2" t="n"/>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>TC-003</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>Дрєпіна А. (СМ)</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>27.10.2026</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>так</t>
+        </is>
+      </c>
+      <c r="E4" s="2" t="inlineStr">
+        <is>
+          <t>так</t>
+        </is>
+      </c>
+      <c r="F4" s="2" t="inlineStr">
+        <is>
+          <t>так</t>
+        </is>
+      </c>
+      <c r="G4" s="6" t="inlineStr">
+        <is>
+          <t>ні</t>
+        </is>
+      </c>
+      <c r="H4" s="2" t="inlineStr">
+        <is>
+          <t>так</t>
+        </is>
+      </c>
+      <c r="I4" s="6" t="inlineStr">
+        <is>
+          <t>ні</t>
+        </is>
+      </c>
+      <c r="J4" s="2" t="inlineStr">
+        <is>
+          <t>так</t>
+        </is>
+      </c>
+      <c r="K4" s="2" t="inlineStr">
+        <is>
+          <t>так</t>
+        </is>
+      </c>
+      <c r="L4" s="2" t="inlineStr">
+        <is>
+          <t>П4: браузер без версії («поточна стабільна версія») і без розміру вікна, не вказано збірку та дату стану demo. Узгодити з рештою кейсів: «Chrome 120 або новіший, вікно 1280×800; збірка v2.5 від 2026-10-11».
+П6: крок 3 «Значення 100 не прийнято» неперевірюваний. Указати, що саме видно: значення в полі «Quantity» не стає 100 і/або під полем текстове повідомлення про помилку (GUI-50).</t>
+        </is>
+      </c>
+      <c r="M4" s="2" t="n"/>
+      <c r="N4" s="2" t="n"/>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>TC-004</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>Дрєпіна А. (СМ)</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>27.10.2026</t>
+        </is>
+      </c>
+      <c r="D5" s="2" t="inlineStr">
+        <is>
+          <t>так</t>
+        </is>
+      </c>
+      <c r="E5" s="2" t="inlineStr">
+        <is>
+          <t>так</t>
+        </is>
+      </c>
+      <c r="F5" s="2" t="inlineStr">
+        <is>
+          <t>так</t>
+        </is>
+      </c>
+      <c r="G5" s="6" t="inlineStr">
+        <is>
+          <t>ні</t>
+        </is>
+      </c>
+      <c r="H5" s="2" t="inlineStr">
+        <is>
+          <t>так</t>
+        </is>
+      </c>
+      <c r="I5" s="2" t="inlineStr">
+        <is>
+          <t>так</t>
+        </is>
+      </c>
+      <c r="J5" s="2" t="inlineStr">
+        <is>
+          <t>так</t>
+        </is>
+      </c>
+      <c r="K5" s="2" t="inlineStr">
+        <is>
+          <t>так</t>
+        </is>
+      </c>
+      <c r="L5" s="2" t="inlineStr">
+        <is>
+          <t>П4: браузер без версії («поточна стабільна версія») і без розміру вікна, не вказано збірку та дату стану demo. Узгодити з рештою кейсів: «Chrome 120 або новіший, вікно 1280×800; збірка v2.5 від 2026-10-11».</t>
+        </is>
+      </c>
+      <c r="M5" s="2" t="n"/>
+      <c r="N5" s="2" t="n"/>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>TC-009</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>Дрєпіна А. (СМ)</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="inlineStr">
+        <is>
+          <t>27.10.2026</t>
+        </is>
+      </c>
+      <c r="D6" s="2" t="inlineStr">
+        <is>
+          <t>так</t>
+        </is>
+      </c>
+      <c r="E6" s="2" t="inlineStr">
+        <is>
+          <t>так</t>
+        </is>
+      </c>
+      <c r="F6" s="2" t="inlineStr">
+        <is>
+          <t>так</t>
+        </is>
+      </c>
+      <c r="G6" s="2" t="inlineStr">
+        <is>
+          <t>так</t>
+        </is>
+      </c>
+      <c r="H6" s="2" t="inlineStr">
+        <is>
+          <t>так</t>
+        </is>
+      </c>
+      <c r="I6" s="6" t="inlineStr">
+        <is>
+          <t>ні</t>
+        </is>
+      </c>
+      <c r="J6" s="2" t="inlineStr">
+        <is>
+          <t>так</t>
+        </is>
+      </c>
+      <c r="K6" s="2" t="inlineStr">
+        <is>
+          <t>так</t>
+        </is>
+      </c>
+      <c r="L6" s="2" t="inlineStr">
+        <is>
+          <t>П6: «повідомлення, яке називає межу в 50 символів» — SRS 1.1 (F-140, GUI-50) цього не вимагає; через це кейс може дати хибний failed. Залишити: текстове повідомлення про помилку безпосередньо під полем «Message»; форму не надіслано. Довжину рядка перевірено: 49 символів.</t>
+        </is>
+      </c>
+      <c r="M6" s="2" t="n"/>
+      <c r="N6" s="2" t="n"/>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>TC-010</t>
+        </is>
+      </c>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>Дрєпіна А. (СМ)</t>
+        </is>
+      </c>
+      <c r="C7" s="2" t="inlineStr">
+        <is>
+          <t>27.10.2026</t>
+        </is>
+      </c>
+      <c r="D7" s="2" t="inlineStr">
+        <is>
+          <t>так</t>
+        </is>
+      </c>
+      <c r="E7" s="2" t="inlineStr">
+        <is>
+          <t>так</t>
+        </is>
+      </c>
+      <c r="F7" s="2" t="inlineStr">
+        <is>
+          <t>так</t>
+        </is>
+      </c>
+      <c r="G7" s="2" t="inlineStr">
+        <is>
+          <t>так</t>
+        </is>
+      </c>
+      <c r="H7" s="2" t="inlineStr">
+        <is>
+          <t>так</t>
+        </is>
+      </c>
+      <c r="I7" s="2" t="inlineStr">
+        <is>
+          <t>так</t>
+        </is>
+      </c>
+      <c r="J7" s="2" t="inlineStr">
+        <is>
+          <t>так</t>
+        </is>
+      </c>
+      <c r="K7" s="2" t="inlineStr">
+        <is>
+          <t>так</t>
+        </is>
+      </c>
+      <c r="L7" s="2" t="inlineStr">
+        <is>
+          <t>Зауважень немає. Довжину рядка перевірено: 50 символів.</t>
+        </is>
+      </c>
+      <c r="M7" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="N7" s="2" t="n"/>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>TC-011</t>
+        </is>
+      </c>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>Дрєпіна А. (СМ)</t>
+        </is>
+      </c>
+      <c r="C8" s="2" t="inlineStr">
+        <is>
+          <t>27.10.2026</t>
+        </is>
+      </c>
+      <c r="D8" s="2" t="inlineStr">
+        <is>
+          <t>так</t>
+        </is>
+      </c>
+      <c r="E8" s="2" t="inlineStr">
+        <is>
+          <t>так</t>
+        </is>
+      </c>
+      <c r="F8" s="2" t="inlineStr">
+        <is>
+          <t>так</t>
+        </is>
+      </c>
+      <c r="G8" s="2" t="inlineStr">
+        <is>
+          <t>так</t>
+        </is>
+      </c>
+      <c r="H8" s="2" t="inlineStr">
+        <is>
+          <t>так</t>
+        </is>
+      </c>
+      <c r="I8" s="2" t="inlineStr">
+        <is>
+          <t>так</t>
+        </is>
+      </c>
+      <c r="J8" s="2" t="inlineStr">
+        <is>
+          <t>так</t>
+        </is>
+      </c>
+      <c r="K8" s="2" t="inlineStr">
+        <is>
+          <t>так</t>
+        </is>
+      </c>
+      <c r="L8" s="2" t="inlineStr">
+        <is>
+          <t>Зауважень немає. Довжину рядка перевірено: 250 символів.</t>
+        </is>
+      </c>
+      <c r="M8" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="N8" s="2" t="n"/>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="inlineStr">
+        <is>
+          <t>TC-012</t>
+        </is>
+      </c>
+      <c r="B9" s="2" t="inlineStr">
+        <is>
+          <t>Дрєпіна А. (СМ)</t>
+        </is>
+      </c>
+      <c r="C9" s="2" t="inlineStr">
+        <is>
+          <t>27.10.2026</t>
+        </is>
+      </c>
+      <c r="D9" s="2" t="inlineStr">
+        <is>
+          <t>так</t>
+        </is>
+      </c>
+      <c r="E9" s="2" t="inlineStr">
+        <is>
+          <t>так</t>
+        </is>
+      </c>
+      <c r="F9" s="2" t="inlineStr">
+        <is>
+          <t>так</t>
+        </is>
+      </c>
+      <c r="G9" s="2" t="inlineStr">
+        <is>
+          <t>так</t>
+        </is>
+      </c>
+      <c r="H9" s="2" t="inlineStr">
+        <is>
+          <t>так</t>
+        </is>
+      </c>
+      <c r="I9" s="6" t="inlineStr">
+        <is>
+          <t>ні</t>
+        </is>
+      </c>
+      <c r="J9" s="2" t="inlineStr">
+        <is>
+          <t>так</t>
+        </is>
+      </c>
+      <c r="K9" s="2" t="inlineStr">
+        <is>
+          <t>так</t>
+        </is>
+      </c>
+      <c r="L9" s="2" t="inlineStr">
+        <is>
+          <t>П6: «повідомлення, яке називає межу в 250 символів» — SRS 1.1 (F-140, GUI-50) цього не вимагає; через це кейс може дати хибний failed. Залишити: текстове повідомлення про помилку безпосередньо під полем «Message»; форму не надіслано. Довжину рядка перевірено: 251 символ.</t>
+        </is>
+      </c>
+      <c r="M9" s="2" t="n"/>
+      <c r="N9" s="2" t="n"/>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t>TC-013</t>
+        </is>
+      </c>
+      <c r="B10" s="2" t="inlineStr">
+        <is>
+          <t>Дрєпіна А. (СМ)</t>
+        </is>
+      </c>
+      <c r="C10" s="2" t="inlineStr">
+        <is>
+          <t>27.10.2026</t>
+        </is>
+      </c>
+      <c r="D10" s="2" t="inlineStr">
+        <is>
+          <t>так</t>
+        </is>
+      </c>
+      <c r="E10" s="2" t="inlineStr">
+        <is>
+          <t>так</t>
+        </is>
+      </c>
+      <c r="F10" s="2" t="inlineStr">
+        <is>
+          <t>так</t>
+        </is>
+      </c>
+      <c r="G10" s="2" t="inlineStr">
+        <is>
+          <t>так</t>
+        </is>
+      </c>
+      <c r="H10" s="2" t="inlineStr">
+        <is>
+          <t>так</t>
+        </is>
+      </c>
+      <c r="I10" s="2" t="inlineStr">
+        <is>
+          <t>так</t>
+        </is>
+      </c>
+      <c r="J10" s="2" t="inlineStr">
+        <is>
+          <t>так</t>
+        </is>
+      </c>
+      <c r="K10" s="2" t="inlineStr">
+        <is>
+          <t>так</t>
+        </is>
+      </c>
+      <c r="L10" s="2" t="inlineStr">
+        <is>
+          <t>Зауважень немає. Довжину повідомлення перевірено: 50 символів.</t>
+        </is>
+      </c>
+      <c r="M10" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="N10" s="2" t="n"/>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="inlineStr">
+        <is>
+          <t>TC-014</t>
+        </is>
+      </c>
+      <c r="B11" s="2" t="inlineStr">
+        <is>
+          <t>Дрєпіна А. (СМ)</t>
+        </is>
+      </c>
+      <c r="C11" s="2" t="inlineStr">
+        <is>
+          <t>27.10.2026</t>
+        </is>
+      </c>
+      <c r="D11" s="2" t="inlineStr">
+        <is>
+          <t>так</t>
+        </is>
+      </c>
+      <c r="E11" s="2" t="inlineStr">
+        <is>
+          <t>так</t>
+        </is>
+      </c>
+      <c r="F11" s="2" t="inlineStr">
+        <is>
+          <t>так</t>
+        </is>
+      </c>
+      <c r="G11" s="2" t="inlineStr">
+        <is>
+          <t>так</t>
+        </is>
+      </c>
+      <c r="H11" s="2" t="inlineStr">
+        <is>
+          <t>так</t>
+        </is>
+      </c>
+      <c r="I11" s="2" t="inlineStr">
+        <is>
+          <t>так</t>
+        </is>
+      </c>
+      <c r="J11" s="2" t="inlineStr">
+        <is>
+          <t>так</t>
+        </is>
+      </c>
+      <c r="K11" s="2" t="inlineStr">
+        <is>
+          <t>так</t>
+        </is>
+      </c>
+      <c r="L11" s="2" t="inlineStr">
+        <is>
+          <t>Зауважень немає.</t>
+        </is>
+      </c>
+      <c r="M11" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="N11" s="2" t="n"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="inlineStr">
+        <is>
+          <t>TC-015</t>
+        </is>
+      </c>
+      <c r="B12" s="2" t="inlineStr">
+        <is>
+          <t>Дрєпіна А. (СМ)</t>
+        </is>
+      </c>
+      <c r="C12" s="2" t="inlineStr">
+        <is>
+          <t>27.10.2026</t>
+        </is>
+      </c>
+      <c r="D12" s="2" t="inlineStr">
+        <is>
+          <t>так</t>
+        </is>
+      </c>
+      <c r="E12" s="2" t="inlineStr">
+        <is>
+          <t>так</t>
+        </is>
+      </c>
+      <c r="F12" s="2" t="inlineStr">
+        <is>
+          <t>так</t>
+        </is>
+      </c>
+      <c r="G12" s="2" t="inlineStr">
+        <is>
+          <t>так</t>
+        </is>
+      </c>
+      <c r="H12" s="2" t="inlineStr">
+        <is>
+          <t>так</t>
+        </is>
+      </c>
+      <c r="I12" s="2" t="inlineStr">
+        <is>
+          <t>так</t>
+        </is>
+      </c>
+      <c r="J12" s="2" t="inlineStr">
+        <is>
+          <t>так</t>
+        </is>
+      </c>
+      <c r="K12" s="2" t="inlineStr">
+        <is>
+          <t>так</t>
+        </is>
+      </c>
+      <c r="L12" s="2" t="inlineStr">
+        <is>
+          <t>Зауважень за чек-листом немає. Дрібне: посилання «методичка, п. 5.4» — в sprint3-instruction етика demo описана в п. 1.7 (так само в TC-016–019 і Coverage).</t>
+        </is>
+      </c>
+      <c r="M12" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="N12" s="2" t="n"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="inlineStr">
+        <is>
+          <t>TC-016</t>
+        </is>
+      </c>
+      <c r="B13" s="2" t="inlineStr">
+        <is>
+          <t>Дрєпіна А. (СМ)</t>
+        </is>
+      </c>
+      <c r="C13" s="2" t="inlineStr">
+        <is>
+          <t>27.10.2026</t>
+        </is>
+      </c>
+      <c r="D13" s="2" t="inlineStr">
+        <is>
+          <t>так</t>
+        </is>
+      </c>
+      <c r="E13" s="2" t="inlineStr">
+        <is>
+          <t>так</t>
+        </is>
+      </c>
+      <c r="F13" s="2" t="inlineStr">
+        <is>
+          <t>так</t>
+        </is>
+      </c>
+      <c r="G13" s="2" t="inlineStr">
+        <is>
+          <t>так</t>
+        </is>
+      </c>
+      <c r="H13" s="2" t="inlineStr">
+        <is>
+          <t>так</t>
+        </is>
+      </c>
+      <c r="I13" s="2" t="inlineStr">
+        <is>
+          <t>так</t>
+        </is>
+      </c>
+      <c r="J13" s="2" t="inlineStr">
+        <is>
+          <t>так</t>
+        </is>
+      </c>
+      <c r="K13" s="2" t="inlineStr">
+        <is>
+          <t>так</t>
+        </is>
+      </c>
+      <c r="L13" s="2" t="inlineStr">
+        <is>
+          <t>Зауважень немає.</t>
+        </is>
+      </c>
+      <c r="M13" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="N13" s="2" t="n"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="inlineStr">
+        <is>
+          <t>TC-017</t>
+        </is>
+      </c>
+      <c r="B14" s="2" t="inlineStr">
+        <is>
+          <t>Дрєпіна А. (СМ)</t>
+        </is>
+      </c>
+      <c r="C14" s="2" t="inlineStr">
+        <is>
+          <t>27.10.2026</t>
+        </is>
+      </c>
+      <c r="D14" s="2" t="inlineStr">
+        <is>
+          <t>так</t>
+        </is>
+      </c>
+      <c r="E14" s="2" t="inlineStr">
+        <is>
+          <t>так</t>
+        </is>
+      </c>
+      <c r="F14" s="2" t="inlineStr">
+        <is>
+          <t>так</t>
+        </is>
+      </c>
+      <c r="G14" s="2" t="inlineStr">
+        <is>
+          <t>так</t>
+        </is>
+      </c>
+      <c r="H14" s="2" t="inlineStr">
+        <is>
+          <t>так</t>
+        </is>
+      </c>
+      <c r="I14" s="2" t="inlineStr">
+        <is>
+          <t>так</t>
+        </is>
+      </c>
+      <c r="J14" s="2" t="inlineStr">
+        <is>
+          <t>так</t>
+        </is>
+      </c>
+      <c r="K14" s="2" t="inlineStr">
+        <is>
+          <t>так</t>
+        </is>
+      </c>
+      <c r="L14" s="2" t="inlineStr">
+        <is>
+          <t>Зауважень немає.</t>
+        </is>
+      </c>
+      <c r="M14" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="N14" s="2" t="n"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="2" t="inlineStr">
+        <is>
+          <t>TC-018</t>
+        </is>
+      </c>
+      <c r="B15" s="2" t="inlineStr">
+        <is>
+          <t>Дрєпіна А. (СМ)</t>
+        </is>
+      </c>
+      <c r="C15" s="2" t="inlineStr">
+        <is>
+          <t>27.10.2026</t>
+        </is>
+      </c>
+      <c r="D15" s="2" t="inlineStr">
+        <is>
+          <t>так</t>
+        </is>
+      </c>
+      <c r="E15" s="2" t="inlineStr">
+        <is>
+          <t>так</t>
+        </is>
+      </c>
+      <c r="F15" s="2" t="inlineStr">
+        <is>
+          <t>так</t>
+        </is>
+      </c>
+      <c r="G15" s="2" t="inlineStr">
+        <is>
+          <t>так</t>
+        </is>
+      </c>
+      <c r="H15" s="2" t="inlineStr">
+        <is>
+          <t>так</t>
+        </is>
+      </c>
+      <c r="I15" s="2" t="inlineStr">
+        <is>
+          <t>так</t>
+        </is>
+      </c>
+      <c r="J15" s="2" t="inlineStr">
+        <is>
+          <t>так</t>
+        </is>
+      </c>
+      <c r="K15" s="2" t="inlineStr">
+        <is>
+          <t>так</t>
+        </is>
+      </c>
+      <c r="L15" s="2" t="inlineStr">
+        <is>
+          <t>Зауважень немає.</t>
+        </is>
+      </c>
+      <c r="M15" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="N15" s="2" t="n"/>
+    </row>
+    <row r="16">
+      <c r="A16" s="2" t="inlineStr">
+        <is>
+          <t>TC-019</t>
+        </is>
+      </c>
+      <c r="B16" s="2" t="inlineStr">
+        <is>
+          <t>Дрєпіна А. (СМ)</t>
+        </is>
+      </c>
+      <c r="C16" s="2" t="inlineStr">
+        <is>
+          <t>27.10.2026</t>
+        </is>
+      </c>
+      <c r="D16" s="2" t="inlineStr">
+        <is>
+          <t>так</t>
+        </is>
+      </c>
+      <c r="E16" s="2" t="inlineStr">
+        <is>
+          <t>так</t>
+        </is>
+      </c>
+      <c r="F16" s="6" t="inlineStr">
+        <is>
+          <t>ні</t>
+        </is>
+      </c>
+      <c r="G16" s="6" t="inlineStr">
+        <is>
+          <t>ні</t>
+        </is>
+      </c>
+      <c r="H16" s="2" t="inlineStr">
+        <is>
+          <t>так</t>
+        </is>
+      </c>
+      <c r="I16" s="2" t="inlineStr">
+        <is>
+          <t>так</t>
+        </is>
+      </c>
+      <c r="J16" s="2" t="inlineStr">
+        <is>
+          <t>так</t>
+        </is>
+      </c>
+      <c r="K16" s="6" t="inlineStr">
+        <is>
+          <t>ні</t>
+        </is>
+      </c>
+      <c r="L16" s="2" t="inlineStr">
+        <is>
+          <t>П3, П4: кейс спирається на обліковий запис, «зареєстрований заздалегідь»; дані demo скидаються (SRS 1.1, розд. 2.3), тож кейс залежить від стану з попереднього сеансу. Додати реєстрацію в кроки кейсу або вказати, хто і коли створює запис перед виконанням.
+П8: для форми відновлення пароля немає негативної пари (напр., порожнє поле «Email address» → помилка під полем, GUI-50) — додати як TC-025+.</t>
+        </is>
+      </c>
+      <c r="M16" s="2" t="n"/>
+      <c r="N16" s="2" t="n"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="2" t="inlineStr">
+        <is>
+          <t>TC-020</t>
+        </is>
+      </c>
+      <c r="B17" s="2" t="inlineStr">
+        <is>
+          <t>Горбонос О. (КТ)</t>
+        </is>
+      </c>
+      <c r="C17" s="2" t="n"/>
+      <c r="D17" s="2" t="n"/>
+      <c r="E17" s="2" t="n"/>
+      <c r="F17" s="2" t="n"/>
+      <c r="G17" s="2" t="n"/>
+      <c r="H17" s="2" t="n"/>
+      <c r="I17" s="2" t="n"/>
+      <c r="J17" s="2" t="n"/>
+      <c r="K17" s="2" t="n"/>
+      <c r="L17" s="2" t="n"/>
+      <c r="M17" s="2" t="n"/>
+      <c r="N17" s="2" t="n"/>
+    </row>
+    <row r="18">
+      <c r="A18" s="2" t="inlineStr">
+        <is>
+          <t>TC-021</t>
+        </is>
+      </c>
+      <c r="B18" s="2" t="inlineStr">
+        <is>
+          <t>Горбонос О. (КТ)</t>
+        </is>
+      </c>
+      <c r="C18" s="2" t="n"/>
+      <c r="D18" s="2" t="n"/>
+      <c r="E18" s="2" t="n"/>
+      <c r="F18" s="2" t="n"/>
+      <c r="G18" s="2" t="n"/>
+      <c r="H18" s="2" t="n"/>
+      <c r="I18" s="2" t="n"/>
+      <c r="J18" s="2" t="n"/>
+      <c r="K18" s="2" t="n"/>
+      <c r="L18" s="2" t="n"/>
+      <c r="M18" s="2" t="n"/>
+      <c r="N18" s="2" t="n"/>
+    </row>
+    <row r="19">
+      <c r="A19" s="2" t="inlineStr">
+        <is>
+          <t>TC-022</t>
+        </is>
+      </c>
+      <c r="B19" s="2" t="inlineStr">
+        <is>
+          <t>Горбонос О. (КТ)</t>
+        </is>
+      </c>
+      <c r="C19" s="2" t="n"/>
+      <c r="D19" s="2" t="n"/>
+      <c r="E19" s="2" t="n"/>
+      <c r="F19" s="2" t="n"/>
+      <c r="G19" s="2" t="n"/>
+      <c r="H19" s="2" t="n"/>
+      <c r="I19" s="2" t="n"/>
+      <c r="J19" s="2" t="n"/>
+      <c r="K19" s="2" t="n"/>
+      <c r="L19" s="2" t="n"/>
+      <c r="M19" s="2" t="n"/>
+      <c r="N19" s="2" t="n"/>
+    </row>
+    <row r="20">
+      <c r="A20" s="2" t="inlineStr">
+        <is>
+          <t>TC-023</t>
+        </is>
+      </c>
+      <c r="B20" s="2" t="inlineStr">
+        <is>
+          <t>Горбонос О. (КТ)</t>
+        </is>
+      </c>
+      <c r="C20" s="2" t="n"/>
+      <c r="D20" s="2" t="n"/>
+      <c r="E20" s="2" t="n"/>
+      <c r="F20" s="2" t="n"/>
+      <c r="G20" s="2" t="n"/>
+      <c r="H20" s="2" t="n"/>
+      <c r="I20" s="2" t="n"/>
+      <c r="J20" s="2" t="n"/>
+      <c r="K20" s="2" t="n"/>
+      <c r="L20" s="2" t="n"/>
+      <c r="M20" s="2" t="n"/>
+      <c r="N20" s="2" t="n"/>
+    </row>
+    <row r="21">
+      <c r="A21" s="2" t="inlineStr">
+        <is>
+          <t>TC-024</t>
+        </is>
+      </c>
+      <c r="B21" s="2" t="inlineStr">
+        <is>
+          <t>Горбонос О. (КТ)</t>
+        </is>
+      </c>
+      <c r="C21" s="2" t="n"/>
+      <c r="D21" s="2" t="n"/>
+      <c r="E21" s="2" t="n"/>
+      <c r="F21" s="2" t="n"/>
+      <c r="G21" s="2" t="n"/>
+      <c r="H21" s="2" t="n"/>
+      <c r="I21" s="2" t="n"/>
+      <c r="J21" s="2" t="n"/>
+      <c r="K21" s="2" t="n"/>
+      <c r="L21" s="2" t="n"/>
+      <c r="M21" s="2" t="n"/>
+      <c r="N21" s="2" t="n"/>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>П1 шість полів, унікальний TC-NNN · П2 вимога з SRS 1.1, кейс перевіряє саме її · П3 незалежний (відкриття → вихід/закриття) · П4 передумови повні · П5 одна дія на крок, конкретні дані · П6 перевірювані очікувані результати · П7 заголовок і тип · П8 граничні значення / негативна пара</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <dataValidations count="2">
+    <dataValidation sqref="D2:K21" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"так,ні"</formula1>
+    </dataValidation>
+    <dataValidation sqref="M2:M21" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"так,ні,—"</formula1>
+    </dataValidation>
+  </dataValidations>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
SCRUM-118: Review фаза 2 (TC-001–004, TC-019).
фаза 1 (TC-005–008, TC-025, TC-026); 14 кейсів reviewed
</commit_message>
<xml_diff>
--- a/docs/sprint3/test-cases.xlsx
+++ b/docs/sprint3/test-cases.xlsx
@@ -617,11 +617,19 @@
           <t>Коротка К. (ТА)</t>
         </is>
       </c>
-      <c r="K2" s="2" t="n"/>
-      <c r="L2" s="2" t="n"/>
+      <c r="K2" s="2" t="inlineStr">
+        <is>
+          <t>Дрєпіна А. (СМ)</t>
+        </is>
+      </c>
+      <c r="L2" s="2" t="inlineStr">
+        <is>
+          <t>28.10.2026</t>
+        </is>
+      </c>
       <c r="M2" s="2" t="inlineStr">
         <is>
-          <t>draft</t>
+          <t>reviewed</t>
         </is>
       </c>
       <c r="N2" s="2" t="n"/>
@@ -689,11 +697,19 @@
           <t>Коротка К. (ТА)</t>
         </is>
       </c>
-      <c r="K3" s="2" t="n"/>
-      <c r="L3" s="2" t="n"/>
+      <c r="K3" s="2" t="inlineStr">
+        <is>
+          <t>Дрєпіна А. (СМ)</t>
+        </is>
+      </c>
+      <c r="L3" s="2" t="inlineStr">
+        <is>
+          <t>28.10.2026</t>
+        </is>
+      </c>
       <c r="M3" s="2" t="inlineStr">
         <is>
-          <t>draft</t>
+          <t>reviewed</t>
         </is>
       </c>
       <c r="N3" s="2" t="n"/>
@@ -759,11 +775,19 @@
           <t>Коротка К. (ТА)</t>
         </is>
       </c>
-      <c r="K4" s="2" t="n"/>
-      <c r="L4" s="2" t="n"/>
+      <c r="K4" s="2" t="inlineStr">
+        <is>
+          <t>Дрєпіна А. (СМ)</t>
+        </is>
+      </c>
+      <c r="L4" s="2" t="inlineStr">
+        <is>
+          <t>28.10.2026</t>
+        </is>
+      </c>
       <c r="M4" s="2" t="inlineStr">
         <is>
-          <t>draft</t>
+          <t>reviewed</t>
         </is>
       </c>
       <c r="N4" s="2" t="n"/>
@@ -829,11 +853,19 @@
           <t>Коротка К. (ТА)</t>
         </is>
       </c>
-      <c r="K5" s="2" t="n"/>
-      <c r="L5" s="2" t="n"/>
+      <c r="K5" s="2" t="inlineStr">
+        <is>
+          <t>Дрєпіна А. (СМ)</t>
+        </is>
+      </c>
+      <c r="L5" s="2" t="inlineStr">
+        <is>
+          <t>28.10.2026</t>
+        </is>
+      </c>
       <c r="M5" s="2" t="inlineStr">
         <is>
-          <t>draft</t>
+          <t>reviewed</t>
         </is>
       </c>
       <c r="N5" s="2" t="n"/>
@@ -1167,11 +1199,19 @@
           <t>Коротка К. (ТА)</t>
         </is>
       </c>
-      <c r="K9" s="2" t="n"/>
-      <c r="L9" s="2" t="n"/>
+      <c r="K9" s="2" t="inlineStr">
+        <is>
+          <t>Дрєпіна А. (СМ)</t>
+        </is>
+      </c>
+      <c r="L9" s="2" t="inlineStr">
+        <is>
+          <t>28.10.2026</t>
+        </is>
+      </c>
       <c r="M9" s="2" t="inlineStr">
         <is>
-          <t>draft</t>
+          <t>reviewed</t>
         </is>
       </c>
       <c r="N9" s="2" t="n"/>
@@ -1309,11 +1349,19 @@
           <t>Горбонос О. (КТ)</t>
         </is>
       </c>
-      <c r="K11" s="2" t="n"/>
-      <c r="L11" s="2" t="n"/>
+      <c r="K11" s="2" t="inlineStr">
+        <is>
+          <t>Дрєпіна А. (СМ)</t>
+        </is>
+      </c>
+      <c r="L11" s="2" t="inlineStr">
+        <is>
+          <t>28.10.2026</t>
+        </is>
+      </c>
       <c r="M11" s="2" t="inlineStr">
         <is>
-          <t>draft</t>
+          <t>reviewed</t>
         </is>
       </c>
       <c r="N11" s="2" t="n"/>
@@ -1380,11 +1428,19 @@
           <t>Горбонос О. (КТ)</t>
         </is>
       </c>
-      <c r="K12" s="2" t="n"/>
-      <c r="L12" s="2" t="n"/>
+      <c r="K12" s="2" t="inlineStr">
+        <is>
+          <t>Дрєпіна А. (СМ)</t>
+        </is>
+      </c>
+      <c r="L12" s="2" t="inlineStr">
+        <is>
+          <t>28.10.2026</t>
+        </is>
+      </c>
       <c r="M12" s="2" t="inlineStr">
         <is>
-          <t>draft</t>
+          <t>reviewed</t>
         </is>
       </c>
       <c r="N12" s="2" t="n"/>
@@ -1526,11 +1582,19 @@
           <t>Горбонос О. (КТ)</t>
         </is>
       </c>
-      <c r="K14" s="2" t="n"/>
-      <c r="L14" s="2" t="n"/>
+      <c r="K14" s="2" t="inlineStr">
+        <is>
+          <t>Дрєпіна А. (СМ)</t>
+        </is>
+      </c>
+      <c r="L14" s="2" t="inlineStr">
+        <is>
+          <t>28.10.2026</t>
+        </is>
+      </c>
       <c r="M14" s="2" t="inlineStr">
         <is>
-          <t>draft</t>
+          <t>reviewed</t>
         </is>
       </c>
       <c r="N14" s="2" t="n"/>
@@ -1600,11 +1664,19 @@
           <t>Горбонос О. (КТ)</t>
         </is>
       </c>
-      <c r="K15" s="2" t="n"/>
-      <c r="L15" s="2" t="n"/>
+      <c r="K15" s="2" t="inlineStr">
+        <is>
+          <t>Дрєпіна А. (СМ)</t>
+        </is>
+      </c>
+      <c r="L15" s="2" t="inlineStr">
+        <is>
+          <t>28.10.2026</t>
+        </is>
+      </c>
       <c r="M15" s="2" t="inlineStr">
         <is>
-          <t>draft</t>
+          <t>reviewed</t>
         </is>
       </c>
       <c r="N15" s="2" t="n"/>
@@ -1674,11 +1746,19 @@
           <t>Тимчак А. (ІТ)</t>
         </is>
       </c>
-      <c r="K16" s="2" t="n"/>
-      <c r="L16" s="2" t="n"/>
+      <c r="K16" s="2" t="inlineStr">
+        <is>
+          <t>Дрєпіна А. (СМ)</t>
+        </is>
+      </c>
+      <c r="L16" s="2" t="inlineStr">
+        <is>
+          <t>28.10.2026</t>
+        </is>
+      </c>
       <c r="M16" s="2" t="inlineStr">
         <is>
-          <t>draft</t>
+          <t>reviewed</t>
         </is>
       </c>
       <c r="N16" s="2" t="n"/>
@@ -1744,11 +1824,19 @@
           <t>Тимчак А. (ІТ)</t>
         </is>
       </c>
-      <c r="K17" s="2" t="n"/>
-      <c r="L17" s="2" t="n"/>
+      <c r="K17" s="2" t="inlineStr">
+        <is>
+          <t>Дрєпіна А. (СМ)</t>
+        </is>
+      </c>
+      <c r="L17" s="2" t="inlineStr">
+        <is>
+          <t>28.10.2026</t>
+        </is>
+      </c>
       <c r="M17" s="2" t="inlineStr">
         <is>
-          <t>draft</t>
+          <t>reviewed</t>
         </is>
       </c>
       <c r="N17" s="2" t="n"/>
@@ -1832,11 +1920,19 @@
           <t>Тимчак А. (ІТ)</t>
         </is>
       </c>
-      <c r="K18" s="2" t="n"/>
-      <c r="L18" s="2" t="n"/>
+      <c r="K18" s="2" t="inlineStr">
+        <is>
+          <t>Дрєпіна А. (СМ)</t>
+        </is>
+      </c>
+      <c r="L18" s="2" t="inlineStr">
+        <is>
+          <t>28.10.2026</t>
+        </is>
+      </c>
       <c r="M18" s="2" t="inlineStr">
         <is>
-          <t>draft</t>
+          <t>reviewed</t>
         </is>
       </c>
       <c r="N18" s="2" t="n"/>
@@ -1898,11 +1994,19 @@
           <t>Тимчак А. (ІТ)</t>
         </is>
       </c>
-      <c r="K19" s="2" t="n"/>
-      <c r="L19" s="2" t="n"/>
+      <c r="K19" s="2" t="inlineStr">
+        <is>
+          <t>Дрєпіна А. (СМ)</t>
+        </is>
+      </c>
+      <c r="L19" s="2" t="inlineStr">
+        <is>
+          <t>28.10.2026</t>
+        </is>
+      </c>
       <c r="M19" s="2" t="inlineStr">
         <is>
-          <t>draft</t>
+          <t>reviewed</t>
         </is>
       </c>
       <c r="N19" s="2" t="n"/>
@@ -2400,11 +2504,19 @@
           <t>Тимчак А. (ІТ)</t>
         </is>
       </c>
-      <c r="K26" s="2" t="n"/>
-      <c r="L26" s="2" t="n"/>
+      <c r="K26" s="2" t="inlineStr">
+        <is>
+          <t>Дрєпіна А. (СМ)</t>
+        </is>
+      </c>
+      <c r="L26" s="2" t="inlineStr">
+        <is>
+          <t>28.10.2026</t>
+        </is>
+      </c>
       <c r="M26" s="2" t="inlineStr">
         <is>
-          <t>draft</t>
+          <t>reviewed</t>
         </is>
       </c>
       <c r="N26" s="2" t="n"/>
@@ -4027,7 +4139,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N23"/>
+  <dimension ref="A1:N29"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -4149,9 +4261,9 @@
           <t>так</t>
         </is>
       </c>
-      <c r="G2" s="6" t="inlineStr">
-        <is>
-          <t>ні</t>
+      <c r="G2" s="2" t="inlineStr">
+        <is>
+          <t>так</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr">
@@ -4177,11 +4289,20 @@
       <c r="L2" s="2" t="inlineStr">
         <is>
           <t>П4: браузер без версії («поточна стабільна версія») і без розміру вікна, не вказано збірку та дату стану demo. Узгодити з рештою кейсів: «Chrome 120 або новіший, вікно 1280×800; збірка v2.5 від 2026-10-11».
-Поза чек-листом (для КТ): за task-board.md, розд. 3, ТА пише TC-001–004 за F-10/GUI-65 і TC-005–008 за GUI-30 (0 / 1 / 99 / 100), а F-60 належить СМ. Фактичні TC-001–004 не збігаються з розподілом; TC-005–008 у файлі немає.</t>
-        </is>
-      </c>
-      <c r="M2" s="2" t="n"/>
-      <c r="N2" s="2" t="n"/>
+Поза чек-листом (для КТ): за task-board.md, розд. 3, ТА пише TC-001–004 за F-10/GUI-65 і TC-005–008 за GUI-30 (0 / 1 / 99 / 100), а F-60 належить СМ. Фактичні TC-001–004 не збігаються з розподілом; TC-005–008 у файлі немає.
+Фаза 2 (28.10.2026, коміт a07b300): П4 виправлено.</t>
+        </is>
+      </c>
+      <c r="M2" s="2" t="inlineStr">
+        <is>
+          <t>так</t>
+        </is>
+      </c>
+      <c r="N2" s="2" t="inlineStr">
+        <is>
+          <t>28.10.2026</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
@@ -4214,9 +4335,9 @@
           <t>так</t>
         </is>
       </c>
-      <c r="G3" s="6" t="inlineStr">
-        <is>
-          <t>ні</t>
+      <c r="G3" s="2" t="inlineStr">
+        <is>
+          <t>так</t>
         </is>
       </c>
       <c r="H3" s="2" t="inlineStr">
@@ -4242,11 +4363,20 @@
       <c r="L3" s="2" t="inlineStr">
         <is>
           <t>П4: браузер без версії («поточна стабільна версія») і без розміру вікна, не вказано збірку та дату стану demo. Узгодити з рештою кейсів: «Chrome 120 або новіший, вікно 1280×800; збірка v2.5 від 2026-10-11».
-Поза чек-листом: за task-board.md кейси GUI-30 мають номери TC-005–008; нижня межа (0 / 1) ще не покрита.</t>
-        </is>
-      </c>
-      <c r="M3" s="2" t="n"/>
-      <c r="N3" s="2" t="n"/>
+Поза чек-листом: за task-board.md кейси GUI-30 мають номери TC-005–008; нижня межа (0 / 1) ще не покрита.
+Фаза 2 (28.10.2026, коміт a07b300): П4 виправлено.</t>
+        </is>
+      </c>
+      <c r="M3" s="2" t="inlineStr">
+        <is>
+          <t>так</t>
+        </is>
+      </c>
+      <c r="N3" s="2" t="inlineStr">
+        <is>
+          <t>28.10.2026</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
@@ -4279,9 +4409,9 @@
           <t>так</t>
         </is>
       </c>
-      <c r="G4" s="6" t="inlineStr">
-        <is>
-          <t>ні</t>
+      <c r="G4" s="2" t="inlineStr">
+        <is>
+          <t>так</t>
         </is>
       </c>
       <c r="H4" s="2" t="inlineStr">
@@ -4289,9 +4419,9 @@
           <t>так</t>
         </is>
       </c>
-      <c r="I4" s="6" t="inlineStr">
-        <is>
-          <t>ні</t>
+      <c r="I4" s="2" t="inlineStr">
+        <is>
+          <t>так</t>
         </is>
       </c>
       <c r="J4" s="2" t="inlineStr">
@@ -4307,11 +4437,20 @@
       <c r="L4" s="2" t="inlineStr">
         <is>
           <t>П4: браузер без версії («поточна стабільна версія») і без розміру вікна, не вказано збірку та дату стану demo. Узгодити з рештою кейсів: «Chrome 120 або новіший, вікно 1280×800; збірка v2.5 від 2026-10-11».
-П6: крок 3 «Значення 100 не прийнято» неперевірюваний. Указати, що саме видно: значення в полі «Quantity» не стає 100 і/або під полем текстове повідомлення про помилку (GUI-50).</t>
-        </is>
-      </c>
-      <c r="M4" s="2" t="n"/>
-      <c r="N4" s="2" t="n"/>
+П6: крок 3 «Значення 100 не прийнято» неперевірюваний. Указати, що саме видно: значення в полі «Quantity» не стає 100 і/або під полем текстове повідомлення про помилку (GUI-50).
+Фаза 2 (28.10.2026, коміт a07b300): П4 виправлено, П6 виправлено.</t>
+        </is>
+      </c>
+      <c r="M4" s="2" t="inlineStr">
+        <is>
+          <t>так</t>
+        </is>
+      </c>
+      <c r="N4" s="2" t="inlineStr">
+        <is>
+          <t>28.10.2026</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
@@ -4344,9 +4483,9 @@
           <t>так</t>
         </is>
       </c>
-      <c r="G5" s="6" t="inlineStr">
-        <is>
-          <t>ні</t>
+      <c r="G5" s="2" t="inlineStr">
+        <is>
+          <t>так</t>
         </is>
       </c>
       <c r="H5" s="2" t="inlineStr">
@@ -4371,16 +4510,25 @@
       </c>
       <c r="L5" s="2" t="inlineStr">
         <is>
-          <t>П4: браузер без версії («поточна стабільна версія») і без розміру вікна, не вказано збірку та дату стану demo. Узгодити з рештою кейсів: «Chrome 120 або новіший, вікно 1280×800; збірка v2.5 від 2026-10-11».</t>
-        </is>
-      </c>
-      <c r="M5" s="2" t="n"/>
-      <c r="N5" s="2" t="n"/>
+          <t>П4: браузер без версії («поточна стабільна версія») і без розміру вікна, не вказано збірку та дату стану demo. Узгодити з рештою кейсів: «Chrome 120 або новіший, вікно 1280×800; збірка v2.5 від 2026-10-11».
+Фаза 2 (28.10.2026, коміт a07b300): П4 виправлено.</t>
+        </is>
+      </c>
+      <c r="M5" s="2" t="inlineStr">
+        <is>
+          <t>так</t>
+        </is>
+      </c>
+      <c r="N5" s="2" t="inlineStr">
+        <is>
+          <t>28.10.2026</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>TC-009</t>
+          <t>TC-005</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
@@ -4390,7 +4538,7 @@
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>27.10.2026</t>
+          <t>28.10.2026</t>
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr">
@@ -4403,9 +4551,9 @@
           <t>так</t>
         </is>
       </c>
-      <c r="F6" s="2" t="inlineStr">
-        <is>
-          <t>так</t>
+      <c r="F6" s="6" t="inlineStr">
+        <is>
+          <t>ні</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr">
@@ -4413,16 +4561,16 @@
           <t>так</t>
         </is>
       </c>
-      <c r="H6" s="2" t="inlineStr">
-        <is>
-          <t>так</t>
-        </is>
-      </c>
-      <c r="I6" s="6" t="inlineStr">
+      <c r="H6" s="6" t="inlineStr">
         <is>
           <t>ні</t>
         </is>
       </c>
+      <c r="I6" s="2" t="inlineStr">
+        <is>
+          <t>так</t>
+        </is>
+      </c>
       <c r="J6" s="2" t="inlineStr">
         <is>
           <t>так</t>
@@ -4435,7 +4583,8 @@
       </c>
       <c r="L6" s="2" t="inlineStr">
         <is>
-          <t>П6: «повідомлення, яке називає межу в 50 символів» — SRS 1.1 (F-140, GUI-50) цього не вимагає; через це кейс може дати хибний failed. Залишити: текстове повідомлення про помилку безпосередньо під полем «Message»; форму не надіслано. Довжину рядка перевірено: 49 символів.</t>
+          <t>П3: адреса shopline.ta005@example.com фіксована — після першого виконання вона зареєстрована, тож повторне виконання (ІТ повторює кожен failed; спринти 4–5) впаде на кроці 16. Додати дату виконання, як у TC-019: shopline.ta005.ДДММРРРР@example.com.
+П5: крок 20 «У меню користувача натиснути Sign out» — дві дії; розбити: натиснути ім'я користувача / натиснути «Sign out».</t>
         </is>
       </c>
       <c r="M6" s="2" t="n"/>
@@ -4444,7 +4593,7 @@
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>TC-010</t>
+          <t>TC-006</t>
         </is>
       </c>
       <c r="B7" s="2" t="inlineStr">
@@ -4454,7 +4603,7 @@
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
-          <t>27.10.2026</t>
+          <t>28.10.2026</t>
         </is>
       </c>
       <c r="D7" s="2" t="inlineStr">
@@ -4467,9 +4616,9 @@
           <t>так</t>
         </is>
       </c>
-      <c r="F7" s="2" t="inlineStr">
-        <is>
-          <t>так</t>
+      <c r="F7" s="6" t="inlineStr">
+        <is>
+          <t>ні</t>
         </is>
       </c>
       <c r="G7" s="2" t="inlineStr">
@@ -4499,20 +4648,16 @@
       </c>
       <c r="L7" s="2" t="inlineStr">
         <is>
-          <t>Зауважень немає. Довжину рядка перевірено: 50 символів.</t>
-        </is>
-      </c>
-      <c r="M7" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
+          <t>П3: адреса shopline.ta006@example.com фіксована — після першого виконання вона зареєстрована, тож повторне виконання (ІТ повторює кожен failed; спринти 4–5) впаде на кроці 16. Додати дату виконання, як у TC-019: shopline.ta006.ДДММРРРР@example.com. Межа a−1 (7 символів) і склад пароля перевірено.</t>
+        </is>
+      </c>
+      <c r="M7" s="2" t="n"/>
       <c r="N7" s="2" t="n"/>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>TC-011</t>
+          <t>TC-007</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
@@ -4522,7 +4667,7 @@
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>27.10.2026</t>
+          <t>28.10.2026</t>
         </is>
       </c>
       <c r="D8" s="2" t="inlineStr">
@@ -4535,9 +4680,9 @@
           <t>так</t>
         </is>
       </c>
-      <c r="F8" s="2" t="inlineStr">
-        <is>
-          <t>так</t>
+      <c r="F8" s="6" t="inlineStr">
+        <is>
+          <t>ні</t>
         </is>
       </c>
       <c r="G8" s="2" t="inlineStr">
@@ -4545,9 +4690,9 @@
           <t>так</t>
         </is>
       </c>
-      <c r="H8" s="2" t="inlineStr">
-        <is>
-          <t>так</t>
+      <c r="H8" s="6" t="inlineStr">
+        <is>
+          <t>ні</t>
         </is>
       </c>
       <c r="I8" s="2" t="inlineStr">
@@ -4567,20 +4712,17 @@
       </c>
       <c r="L8" s="2" t="inlineStr">
         <is>
-          <t>Зауважень немає. Довжину рядка перевірено: 250 символів.</t>
-        </is>
-      </c>
-      <c r="M8" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
+          <t>П3: адреса shopline.ta007@example.com фіксована — після першого виконання вона зареєстрована, тож повторне виконання (ІТ повторює кожен failed; спринти 4–5) впаде на кроці 16. Додати дату виконання, як у TC-019: shopline.ta007.ДДММРРРР@example.com.
+П5: крок 20 «У меню користувача натиснути Sign out» — дві дії; розбити: натиснути ім'я користувача / натиснути «Sign out». Межа a = 8 перевірено.</t>
+        </is>
+      </c>
+      <c r="M8" s="2" t="n"/>
       <c r="N8" s="2" t="n"/>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>TC-012</t>
+          <t>TC-008</t>
         </is>
       </c>
       <c r="B9" s="2" t="inlineStr">
@@ -4590,7 +4732,7 @@
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
-          <t>27.10.2026</t>
+          <t>28.10.2026</t>
         </is>
       </c>
       <c r="D9" s="2" t="inlineStr">
@@ -4618,9 +4760,9 @@
           <t>так</t>
         </is>
       </c>
-      <c r="I9" s="6" t="inlineStr">
-        <is>
-          <t>ні</t>
+      <c r="I9" s="2" t="inlineStr">
+        <is>
+          <t>так</t>
         </is>
       </c>
       <c r="J9" s="2" t="inlineStr">
@@ -4635,16 +4777,24 @@
       </c>
       <c r="L9" s="2" t="inlineStr">
         <is>
-          <t>П6: «повідомлення, яке називає межу в 250 символів» — SRS 1.1 (F-140, GUI-50) цього не вимагає; через це кейс може дати хибний failed. Залишити: текстове повідомлення про помилку безпосередньо під полем «Message»; форму не надіслано. Довжину рядка перевірено: 251 символ.</t>
-        </is>
-      </c>
-      <c r="M9" s="2" t="n"/>
-      <c r="N9" s="2" t="n"/>
+          <t>Зауважень немає.</t>
+        </is>
+      </c>
+      <c r="M9" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="N9" s="2" t="inlineStr">
+        <is>
+          <t>28.10.2026</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>TC-013</t>
+          <t>TC-009</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
@@ -4682,9 +4832,9 @@
           <t>так</t>
         </is>
       </c>
-      <c r="I10" s="2" t="inlineStr">
-        <is>
-          <t>так</t>
+      <c r="I10" s="6" t="inlineStr">
+        <is>
+          <t>ні</t>
         </is>
       </c>
       <c r="J10" s="2" t="inlineStr">
@@ -4699,20 +4849,16 @@
       </c>
       <c r="L10" s="2" t="inlineStr">
         <is>
-          <t>Зауважень немає. Довжину повідомлення перевірено: 50 символів.</t>
-        </is>
-      </c>
-      <c r="M10" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
+          <t>П6: «повідомлення, яке називає межу в 50 символів» — SRS 1.1 (F-140, GUI-50) цього не вимагає; через це кейс може дати хибний failed. Залишити: текстове повідомлення про помилку безпосередньо під полем «Message»; форму не надіслано. Довжину рядка перевірено: 49 символів.</t>
+        </is>
+      </c>
+      <c r="M10" s="2" t="n"/>
       <c r="N10" s="2" t="n"/>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>TC-014</t>
+          <t>TC-010</t>
         </is>
       </c>
       <c r="B11" s="2" t="inlineStr">
@@ -4767,7 +4913,7 @@
       </c>
       <c r="L11" s="2" t="inlineStr">
         <is>
-          <t>Зауважень немає.</t>
+          <t>Зауважень немає. Довжину рядка перевірено: 50 символів.</t>
         </is>
       </c>
       <c r="M11" s="2" t="inlineStr">
@@ -4775,12 +4921,16 @@
           <t>—</t>
         </is>
       </c>
-      <c r="N11" s="2" t="n"/>
+      <c r="N11" s="2" t="inlineStr">
+        <is>
+          <t>28.10.2026</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>TC-015</t>
+          <t>TC-011</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
@@ -4835,7 +4985,7 @@
       </c>
       <c r="L12" s="2" t="inlineStr">
         <is>
-          <t>Зауважень за чек-листом немає. Дрібне: посилання «методичка, п. 5.4» — в sprint3-instruction етика demo описана в п. 1.7 (так само в TC-016–019 і Coverage).</t>
+          <t>Зауважень немає. Довжину рядка перевірено: 250 символів.</t>
         </is>
       </c>
       <c r="M12" s="2" t="inlineStr">
@@ -4843,12 +4993,16 @@
           <t>—</t>
         </is>
       </c>
-      <c r="N12" s="2" t="n"/>
+      <c r="N12" s="2" t="inlineStr">
+        <is>
+          <t>28.10.2026</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>TC-016</t>
+          <t>TC-012</t>
         </is>
       </c>
       <c r="B13" s="2" t="inlineStr">
@@ -4886,9 +5040,9 @@
           <t>так</t>
         </is>
       </c>
-      <c r="I13" s="2" t="inlineStr">
-        <is>
-          <t>так</t>
+      <c r="I13" s="6" t="inlineStr">
+        <is>
+          <t>ні</t>
         </is>
       </c>
       <c r="J13" s="2" t="inlineStr">
@@ -4903,20 +5057,16 @@
       </c>
       <c r="L13" s="2" t="inlineStr">
         <is>
-          <t>Зауважень немає.</t>
-        </is>
-      </c>
-      <c r="M13" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
+          <t>П6: «повідомлення, яке називає межу в 250 символів» — SRS 1.1 (F-140, GUI-50) цього не вимагає; через це кейс може дати хибний failed. Залишити: текстове повідомлення про помилку безпосередньо під полем «Message»; форму не надіслано. Довжину рядка перевірено: 251 символ.</t>
+        </is>
+      </c>
+      <c r="M13" s="2" t="n"/>
       <c r="N13" s="2" t="n"/>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>TC-017</t>
+          <t>TC-013</t>
         </is>
       </c>
       <c r="B14" s="2" t="inlineStr">
@@ -4971,7 +5121,7 @@
       </c>
       <c r="L14" s="2" t="inlineStr">
         <is>
-          <t>Зауважень немає.</t>
+          <t>Зауважень немає. Довжину повідомлення перевірено: 50 символів.</t>
         </is>
       </c>
       <c r="M14" s="2" t="inlineStr">
@@ -4979,12 +5129,16 @@
           <t>—</t>
         </is>
       </c>
-      <c r="N14" s="2" t="n"/>
+      <c r="N14" s="2" t="inlineStr">
+        <is>
+          <t>28.10.2026</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>TC-018</t>
+          <t>TC-014</t>
         </is>
       </c>
       <c r="B15" s="2" t="inlineStr">
@@ -5047,12 +5201,16 @@
           <t>—</t>
         </is>
       </c>
-      <c r="N15" s="2" t="n"/>
+      <c r="N15" s="2" t="inlineStr">
+        <is>
+          <t>28.10.2026</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>TC-019</t>
+          <t>TC-015</t>
         </is>
       </c>
       <c r="B16" s="2" t="inlineStr">
@@ -5075,14 +5233,14 @@
           <t>так</t>
         </is>
       </c>
-      <c r="F16" s="6" t="inlineStr">
-        <is>
-          <t>ні</t>
-        </is>
-      </c>
-      <c r="G16" s="6" t="inlineStr">
-        <is>
-          <t>ні</t>
+      <c r="F16" s="2" t="inlineStr">
+        <is>
+          <t>так</t>
+        </is>
+      </c>
+      <c r="G16" s="2" t="inlineStr">
+        <is>
+          <t>так</t>
         </is>
       </c>
       <c r="H16" s="2" t="inlineStr">
@@ -5100,124 +5258,319 @@
           <t>так</t>
         </is>
       </c>
-      <c r="K16" s="6" t="inlineStr">
-        <is>
-          <t>ні</t>
+      <c r="K16" s="2" t="inlineStr">
+        <is>
+          <t>так</t>
         </is>
       </c>
       <c r="L16" s="2" t="inlineStr">
         <is>
-          <t>П3, П4: кейс спирається на обліковий запис, «зареєстрований заздалегідь»; дані demo скидаються (SRS 1.1, розд. 2.3), тож кейс залежить від стану з попереднього сеансу. Додати реєстрацію в кроки кейсу або вказати, хто і коли створює запис перед виконанням.
-П8: для форми відновлення пароля немає негативної пари (напр., порожнє поле «Email address» → помилка під полем, GUI-50) — додати як TC-025+.</t>
+          <t>Зауважень за чек-листом немає. Дрібне: посилання «методичка, п. 5.4» — в sprint3-instruction етика demo описана в п. 1.7 (так само в TC-016–019 і Coverage).</t>
         </is>
       </c>
       <c r="M16" s="2" t="inlineStr">
         <is>
-          <t>П3, П4: реєстрацію облікового запису перенесено в кроки 2–15 кейсу (адреса з датою виконання), передумова «зареєстровано заздалегідь» прибрана. П8: негативна пара — TC-025 (порожнє поле «Email address», помилка під полем). Звірено з demo 28.10.2026.</t>
-        </is>
-      </c>
-      <c r="N16" s="2" t="n"/>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="N16" s="2" t="inlineStr">
+        <is>
+          <t>28.10.2026</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>TC-020</t>
+          <t>TC-016</t>
         </is>
       </c>
       <c r="B17" s="2" t="inlineStr">
         <is>
-          <t>Горбонос О. (КТ)</t>
-        </is>
-      </c>
-      <c r="C17" s="2" t="n"/>
-      <c r="D17" s="2" t="n"/>
-      <c r="E17" s="2" t="n"/>
-      <c r="F17" s="2" t="n"/>
-      <c r="G17" s="2" t="n"/>
-      <c r="H17" s="2" t="n"/>
-      <c r="I17" s="2" t="n"/>
-      <c r="J17" s="2" t="n"/>
-      <c r="K17" s="2" t="n"/>
-      <c r="L17" s="2" t="n"/>
-      <c r="M17" s="2" t="n"/>
-      <c r="N17" s="2" t="n"/>
+          <t>Дрєпіна А. (СМ)</t>
+        </is>
+      </c>
+      <c r="C17" s="2" t="inlineStr">
+        <is>
+          <t>27.10.2026</t>
+        </is>
+      </c>
+      <c r="D17" s="2" t="inlineStr">
+        <is>
+          <t>так</t>
+        </is>
+      </c>
+      <c r="E17" s="2" t="inlineStr">
+        <is>
+          <t>так</t>
+        </is>
+      </c>
+      <c r="F17" s="2" t="inlineStr">
+        <is>
+          <t>так</t>
+        </is>
+      </c>
+      <c r="G17" s="2" t="inlineStr">
+        <is>
+          <t>так</t>
+        </is>
+      </c>
+      <c r="H17" s="2" t="inlineStr">
+        <is>
+          <t>так</t>
+        </is>
+      </c>
+      <c r="I17" s="2" t="inlineStr">
+        <is>
+          <t>так</t>
+        </is>
+      </c>
+      <c r="J17" s="2" t="inlineStr">
+        <is>
+          <t>так</t>
+        </is>
+      </c>
+      <c r="K17" s="2" t="inlineStr">
+        <is>
+          <t>так</t>
+        </is>
+      </c>
+      <c r="L17" s="2" t="inlineStr">
+        <is>
+          <t>Зауважень немає.</t>
+        </is>
+      </c>
+      <c r="M17" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="N17" s="2" t="inlineStr">
+        <is>
+          <t>28.10.2026</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>TC-021</t>
+          <t>TC-017</t>
         </is>
       </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t>Горбонос О. (КТ)</t>
-        </is>
-      </c>
-      <c r="C18" s="2" t="n"/>
-      <c r="D18" s="2" t="n"/>
-      <c r="E18" s="2" t="n"/>
-      <c r="F18" s="2" t="n"/>
-      <c r="G18" s="2" t="n"/>
-      <c r="H18" s="2" t="n"/>
-      <c r="I18" s="2" t="n"/>
-      <c r="J18" s="2" t="n"/>
-      <c r="K18" s="2" t="n"/>
-      <c r="L18" s="2" t="n"/>
-      <c r="M18" s="2" t="n"/>
-      <c r="N18" s="2" t="n"/>
+          <t>Дрєпіна А. (СМ)</t>
+        </is>
+      </c>
+      <c r="C18" s="2" t="inlineStr">
+        <is>
+          <t>27.10.2026</t>
+        </is>
+      </c>
+      <c r="D18" s="2" t="inlineStr">
+        <is>
+          <t>так</t>
+        </is>
+      </c>
+      <c r="E18" s="2" t="inlineStr">
+        <is>
+          <t>так</t>
+        </is>
+      </c>
+      <c r="F18" s="2" t="inlineStr">
+        <is>
+          <t>так</t>
+        </is>
+      </c>
+      <c r="G18" s="2" t="inlineStr">
+        <is>
+          <t>так</t>
+        </is>
+      </c>
+      <c r="H18" s="2" t="inlineStr">
+        <is>
+          <t>так</t>
+        </is>
+      </c>
+      <c r="I18" s="2" t="inlineStr">
+        <is>
+          <t>так</t>
+        </is>
+      </c>
+      <c r="J18" s="2" t="inlineStr">
+        <is>
+          <t>так</t>
+        </is>
+      </c>
+      <c r="K18" s="2" t="inlineStr">
+        <is>
+          <t>так</t>
+        </is>
+      </c>
+      <c r="L18" s="2" t="inlineStr">
+        <is>
+          <t>Зауважень немає.</t>
+        </is>
+      </c>
+      <c r="M18" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="N18" s="2" t="inlineStr">
+        <is>
+          <t>28.10.2026</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>TC-022</t>
+          <t>TC-018</t>
         </is>
       </c>
       <c r="B19" s="2" t="inlineStr">
         <is>
-          <t>Горбонос О. (КТ)</t>
-        </is>
-      </c>
-      <c r="C19" s="2" t="n"/>
-      <c r="D19" s="2" t="n"/>
-      <c r="E19" s="2" t="n"/>
-      <c r="F19" s="2" t="n"/>
-      <c r="G19" s="2" t="n"/>
-      <c r="H19" s="2" t="n"/>
-      <c r="I19" s="2" t="n"/>
-      <c r="J19" s="2" t="n"/>
-      <c r="K19" s="2" t="n"/>
-      <c r="L19" s="2" t="n"/>
-      <c r="M19" s="2" t="n"/>
-      <c r="N19" s="2" t="n"/>
+          <t>Дрєпіна А. (СМ)</t>
+        </is>
+      </c>
+      <c r="C19" s="2" t="inlineStr">
+        <is>
+          <t>27.10.2026</t>
+        </is>
+      </c>
+      <c r="D19" s="2" t="inlineStr">
+        <is>
+          <t>так</t>
+        </is>
+      </c>
+      <c r="E19" s="2" t="inlineStr">
+        <is>
+          <t>так</t>
+        </is>
+      </c>
+      <c r="F19" s="2" t="inlineStr">
+        <is>
+          <t>так</t>
+        </is>
+      </c>
+      <c r="G19" s="2" t="inlineStr">
+        <is>
+          <t>так</t>
+        </is>
+      </c>
+      <c r="H19" s="2" t="inlineStr">
+        <is>
+          <t>так</t>
+        </is>
+      </c>
+      <c r="I19" s="2" t="inlineStr">
+        <is>
+          <t>так</t>
+        </is>
+      </c>
+      <c r="J19" s="2" t="inlineStr">
+        <is>
+          <t>так</t>
+        </is>
+      </c>
+      <c r="K19" s="2" t="inlineStr">
+        <is>
+          <t>так</t>
+        </is>
+      </c>
+      <c r="L19" s="2" t="inlineStr">
+        <is>
+          <t>Зауважень немає.
+28.10.2026: в «Обґрунтуванні даних» оновлено посилання на позитивну пару (TC-026), суть кейсу не змінилась.</t>
+        </is>
+      </c>
+      <c r="M19" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="N19" s="2" t="inlineStr">
+        <is>
+          <t>28.10.2026</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>TC-023</t>
+          <t>TC-019</t>
         </is>
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>Горбонос О. (КТ)</t>
-        </is>
-      </c>
-      <c r="C20" s="2" t="n"/>
-      <c r="D20" s="2" t="n"/>
-      <c r="E20" s="2" t="n"/>
-      <c r="F20" s="2" t="n"/>
-      <c r="G20" s="2" t="n"/>
-      <c r="H20" s="2" t="n"/>
-      <c r="I20" s="2" t="n"/>
-      <c r="J20" s="2" t="n"/>
-      <c r="K20" s="2" t="n"/>
-      <c r="L20" s="2" t="n"/>
-      <c r="M20" s="2" t="n"/>
+          <t>Дрєпіна А. (СМ)</t>
+        </is>
+      </c>
+      <c r="C20" s="2" t="inlineStr">
+        <is>
+          <t>27.10.2026</t>
+        </is>
+      </c>
+      <c r="D20" s="2" t="inlineStr">
+        <is>
+          <t>так</t>
+        </is>
+      </c>
+      <c r="E20" s="2" t="inlineStr">
+        <is>
+          <t>так</t>
+        </is>
+      </c>
+      <c r="F20" s="2" t="inlineStr">
+        <is>
+          <t>так</t>
+        </is>
+      </c>
+      <c r="G20" s="2" t="inlineStr">
+        <is>
+          <t>так</t>
+        </is>
+      </c>
+      <c r="H20" s="6" t="inlineStr">
+        <is>
+          <t>ні</t>
+        </is>
+      </c>
+      <c r="I20" s="2" t="inlineStr">
+        <is>
+          <t>так</t>
+        </is>
+      </c>
+      <c r="J20" s="2" t="inlineStr">
+        <is>
+          <t>так</t>
+        </is>
+      </c>
+      <c r="K20" s="2" t="inlineStr">
+        <is>
+          <t>так</t>
+        </is>
+      </c>
+      <c r="L20" s="2" t="inlineStr">
+        <is>
+          <t>П3, П4: кейс спирається на обліковий запис, «зареєстрований заздалегідь»; дані demo скидаються (SRS 1.1, розд. 2.3), тож кейс залежить від стану з попереднього сеансу. Додати реєстрацію в кроки кейсу або вказати, хто і коли створює запис перед виконанням.
+П8: для форми відновлення пароля немає негативної пари (напр., порожнє поле «Email address» → помилка під полем, GUI-50) — додати як TC-025+.
+Фаза 2 (28.10.2026, коміт 61bd56d): П3, П4 виправлено (реєстрація в кроках, адреса з датою); П8 виправлено (TC-025).
+Нове П5: крок 15 «ввести пароль і натиснути Register» — дві дії; розбити на два кроки.</t>
+        </is>
+      </c>
+      <c r="M20" s="6" t="inlineStr">
+        <is>
+          <t>ні</t>
+        </is>
+      </c>
       <c r="N20" s="2" t="n"/>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t>TC-024</t>
+          <t>TC-020</t>
         </is>
       </c>
       <c r="B21" s="2" t="inlineStr">
@@ -5238,8 +5591,241 @@
       <c r="M21" s="2" t="n"/>
       <c r="N21" s="2" t="n"/>
     </row>
+    <row r="22">
+      <c r="A22" s="2" t="inlineStr">
+        <is>
+          <t>TC-021</t>
+        </is>
+      </c>
+      <c r="B22" s="2" t="inlineStr">
+        <is>
+          <t>Горбонос О. (КТ)</t>
+        </is>
+      </c>
+      <c r="C22" s="2" t="n"/>
+      <c r="D22" s="2" t="n"/>
+      <c r="E22" s="2" t="n"/>
+      <c r="F22" s="2" t="n"/>
+      <c r="G22" s="2" t="n"/>
+      <c r="H22" s="2" t="n"/>
+      <c r="I22" s="2" t="n"/>
+      <c r="J22" s="2" t="n"/>
+      <c r="K22" s="2" t="n"/>
+      <c r="L22" s="2" t="n"/>
+      <c r="M22" s="2" t="n"/>
+      <c r="N22" s="2" t="n"/>
+    </row>
     <row r="23">
-      <c r="A23" t="inlineStr">
+      <c r="A23" s="2" t="inlineStr">
+        <is>
+          <t>TC-022</t>
+        </is>
+      </c>
+      <c r="B23" s="2" t="inlineStr">
+        <is>
+          <t>Горбонос О. (КТ)</t>
+        </is>
+      </c>
+      <c r="C23" s="2" t="n"/>
+      <c r="D23" s="2" t="n"/>
+      <c r="E23" s="2" t="n"/>
+      <c r="F23" s="2" t="n"/>
+      <c r="G23" s="2" t="n"/>
+      <c r="H23" s="2" t="n"/>
+      <c r="I23" s="2" t="n"/>
+      <c r="J23" s="2" t="n"/>
+      <c r="K23" s="2" t="n"/>
+      <c r="L23" s="2" t="n"/>
+      <c r="M23" s="2" t="n"/>
+      <c r="N23" s="2" t="n"/>
+    </row>
+    <row r="24">
+      <c r="A24" s="2" t="inlineStr">
+        <is>
+          <t>TC-023</t>
+        </is>
+      </c>
+      <c r="B24" s="2" t="inlineStr">
+        <is>
+          <t>Горбонос О. (КТ)</t>
+        </is>
+      </c>
+      <c r="C24" s="2" t="n"/>
+      <c r="D24" s="2" t="n"/>
+      <c r="E24" s="2" t="n"/>
+      <c r="F24" s="2" t="n"/>
+      <c r="G24" s="2" t="n"/>
+      <c r="H24" s="2" t="n"/>
+      <c r="I24" s="2" t="n"/>
+      <c r="J24" s="2" t="n"/>
+      <c r="K24" s="2" t="n"/>
+      <c r="L24" s="2" t="n"/>
+      <c r="M24" s="2" t="n"/>
+      <c r="N24" s="2" t="n"/>
+    </row>
+    <row r="25">
+      <c r="A25" s="2" t="inlineStr">
+        <is>
+          <t>TC-024</t>
+        </is>
+      </c>
+      <c r="B25" s="2" t="inlineStr">
+        <is>
+          <t>Горбонос О. (КТ)</t>
+        </is>
+      </c>
+      <c r="C25" s="2" t="n"/>
+      <c r="D25" s="2" t="n"/>
+      <c r="E25" s="2" t="n"/>
+      <c r="F25" s="2" t="n"/>
+      <c r="G25" s="2" t="n"/>
+      <c r="H25" s="2" t="n"/>
+      <c r="I25" s="2" t="n"/>
+      <c r="J25" s="2" t="n"/>
+      <c r="K25" s="2" t="n"/>
+      <c r="L25" s="2" t="n"/>
+      <c r="M25" s="2" t="n"/>
+      <c r="N25" s="2" t="n"/>
+    </row>
+    <row r="26">
+      <c r="A26" s="2" t="inlineStr">
+        <is>
+          <t>TC-025</t>
+        </is>
+      </c>
+      <c r="B26" s="2" t="inlineStr">
+        <is>
+          <t>Дрєпіна А. (СМ)</t>
+        </is>
+      </c>
+      <c r="C26" s="2" t="inlineStr">
+        <is>
+          <t>28.10.2026</t>
+        </is>
+      </c>
+      <c r="D26" s="2" t="inlineStr">
+        <is>
+          <t>так</t>
+        </is>
+      </c>
+      <c r="E26" s="2" t="inlineStr">
+        <is>
+          <t>так</t>
+        </is>
+      </c>
+      <c r="F26" s="2" t="inlineStr">
+        <is>
+          <t>так</t>
+        </is>
+      </c>
+      <c r="G26" s="2" t="inlineStr">
+        <is>
+          <t>так</t>
+        </is>
+      </c>
+      <c r="H26" s="2" t="inlineStr">
+        <is>
+          <t>так</t>
+        </is>
+      </c>
+      <c r="I26" s="2" t="inlineStr">
+        <is>
+          <t>так</t>
+        </is>
+      </c>
+      <c r="J26" s="2" t="inlineStr">
+        <is>
+          <t>так</t>
+        </is>
+      </c>
+      <c r="K26" s="2" t="inlineStr">
+        <is>
+          <t>так</t>
+        </is>
+      </c>
+      <c r="L26" s="2" t="inlineStr">
+        <is>
+          <t>Зауважень немає.</t>
+        </is>
+      </c>
+      <c r="M26" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="N26" s="2" t="inlineStr">
+        <is>
+          <t>28.10.2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="2" t="inlineStr">
+        <is>
+          <t>TC-026</t>
+        </is>
+      </c>
+      <c r="B27" s="2" t="inlineStr">
+        <is>
+          <t>Дрєпіна А. (СМ)</t>
+        </is>
+      </c>
+      <c r="C27" s="2" t="inlineStr">
+        <is>
+          <t>28.10.2026</t>
+        </is>
+      </c>
+      <c r="D27" s="2" t="inlineStr">
+        <is>
+          <t>так</t>
+        </is>
+      </c>
+      <c r="E27" s="2" t="inlineStr">
+        <is>
+          <t>так</t>
+        </is>
+      </c>
+      <c r="F27" s="2" t="inlineStr">
+        <is>
+          <t>так</t>
+        </is>
+      </c>
+      <c r="G27" s="6" t="inlineStr">
+        <is>
+          <t>ні</t>
+        </is>
+      </c>
+      <c r="H27" s="6" t="inlineStr">
+        <is>
+          <t>ні</t>
+        </is>
+      </c>
+      <c r="I27" s="2" t="inlineStr">
+        <is>
+          <t>так</t>
+        </is>
+      </c>
+      <c r="J27" s="2" t="inlineStr">
+        <is>
+          <t>так</t>
+        </is>
+      </c>
+      <c r="K27" s="2" t="inlineStr">
+        <is>
+          <t>так</t>
+        </is>
+      </c>
+      <c r="L27" s="2" t="inlineStr">
+        <is>
+          <t>П5: кроки 6, 10, 12 — по дві дії (ім'я користувача в меню + пункт меню); розбити.
+П4: у передумовах «у кроці 13 повертає список до початкового стану», а видалення — крок 11; виправити номер.</t>
+        </is>
+      </c>
+      <c r="M27" s="2" t="n"/>
+      <c r="N27" s="2" t="n"/>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
         <is>
           <t>П1 шість полів, унікальний TC-NNN · П2 вимога з SRS 1.1, кейс перевіряє саме її · П3 незалежний (відкриття → вихід/закриття) · П4 передумови повні · П5 одна дія на крок, конкретні дані · П6 перевірювані очікувані результати · П7 заголовок і тип · П8 граничні значення / негативна пара</t>
         </is>
@@ -5247,10 +5833,10 @@
     </row>
   </sheetData>
   <dataValidations count="2">
-    <dataValidation sqref="D2:K21" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="D2:K27" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"так,ні"</formula1>
     </dataValidation>
-    <dataValidation sqref="M2:M21" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="M2:M27" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"так,ні,—"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
SCRUM-118, SCRUM-119: злиття 8861526 (КТ);
TC-020–024 за рецензією КТ, TC-033 (F-60 негатив); Review фаза 2 TC-005–007, 009, 012; фаза 1 TC-027–032
</commit_message>
<xml_diff>
--- a/docs/sprint3/test-cases.xlsx
+++ b/docs/sprint3/test-cases.xlsx
@@ -951,11 +951,19 @@
           <t>Коротка К. (ТА)</t>
         </is>
       </c>
-      <c r="K6" s="2" t="n"/>
-      <c r="L6" s="2" t="n"/>
+      <c r="K6" s="2" t="inlineStr">
+        <is>
+          <t>Дрєпіна А. (СМ)</t>
+        </is>
+      </c>
+      <c r="L6" s="2" t="inlineStr">
+        <is>
+          <t>28.10.2026</t>
+        </is>
+      </c>
       <c r="M6" s="2" t="inlineStr">
         <is>
-          <t>draft</t>
+          <t>reviewed</t>
         </is>
       </c>
       <c r="N6" s="2" t="n"/>
@@ -1032,11 +1040,19 @@
           <t>Коротка К. (ТА)</t>
         </is>
       </c>
-      <c r="K7" s="2" t="n"/>
-      <c r="L7" s="2" t="n"/>
+      <c r="K7" s="2" t="inlineStr">
+        <is>
+          <t>Дрєпіна А. (СМ)</t>
+        </is>
+      </c>
+      <c r="L7" s="2" t="inlineStr">
+        <is>
+          <t>28.10.2026</t>
+        </is>
+      </c>
       <c r="M7" s="2" t="inlineStr">
         <is>
-          <t>draft</t>
+          <t>reviewed</t>
         </is>
       </c>
       <c r="N7" s="2" t="n"/>
@@ -1122,11 +1138,19 @@
           <t>Коротка К. (ТА)</t>
         </is>
       </c>
-      <c r="K8" s="2" t="n"/>
-      <c r="L8" s="2" t="n"/>
+      <c r="K8" s="2" t="inlineStr">
+        <is>
+          <t>Дрєпіна А. (СМ)</t>
+        </is>
+      </c>
+      <c r="L8" s="2" t="inlineStr">
+        <is>
+          <t>28.10.2026</t>
+        </is>
+      </c>
       <c r="M8" s="2" t="inlineStr">
         <is>
-          <t>draft</t>
+          <t>reviewed</t>
         </is>
       </c>
       <c r="N8" s="2" t="n"/>
@@ -1258,7 +1282,7 @@
           <t>Після кроку 1: відкрито сторінку «Contact», усі поля порожні.
 Після кроків 2–5: у полях відображено введені значення: Test, Tester, tester.tc009@example.com, Customer service.
 Після кроку 6: у полі «Message» 49 символів.
-Після кроку 7: форму не надіслано, сторінка «Contact» залишається відкритою; під полем «Message» текстове повідомлення про помилку, яке називає межу в 50 символів (F-140, GUI-50; SRS 1.1 точного тексту не задає); під іншими полями повідомлень про помилки немає; повідомлення про прийняття звернення над формою відсутнє.
+Після кроку 7: форму не надіслано, сторінка «Contact» залишається відкритою; під полем «Message» текстове повідомлення про помилку (F-140, GUI-50; SRS 1.1 точного тексту не задає); під іншими полями повідомлень про помилки немає; повідомлення про прийняття звернення над формою відсутнє.
 Після кроку 8: вкладку закрито.</t>
         </is>
       </c>
@@ -1274,7 +1298,7 @@
       </c>
       <c r="I10" s="2" t="inlineStr">
         <is>
-          <t>Допустима довжина повідомлення 50–250 (F-140). 49 — на 1 менше за нижню межу, клас недопустимих значень. Решта полів валідні, тому відхилення можливе лише через довжину.</t>
+          <t>Допустима довжина повідомлення 50–250 (F-140). 49 — на 1 менше за нижню межу, клас недопустимих значень. Решта полів валідні, тому відхилення можливе лише через довжину. Граничне значення a−1, таблиця SCRUM-108.</t>
         </is>
       </c>
       <c r="J10" s="2" t="inlineStr">
@@ -1282,11 +1306,19 @@
           <t>Горбонос О. (КТ)</t>
         </is>
       </c>
-      <c r="K10" s="2" t="n"/>
-      <c r="L10" s="2" t="n"/>
+      <c r="K10" s="2" t="inlineStr">
+        <is>
+          <t>Дрєпіна А. (СМ)</t>
+        </is>
+      </c>
+      <c r="L10" s="2" t="inlineStr">
+        <is>
+          <t>28.10.2026</t>
+        </is>
+      </c>
       <c r="M10" s="2" t="inlineStr">
         <is>
-          <t>draft</t>
+          <t>reviewed</t>
         </is>
       </c>
       <c r="N10" s="2" t="n"/>
@@ -1345,7 +1377,7 @@
       </c>
       <c r="I11" s="2" t="inlineStr">
         <is>
-          <t>50 — нижня межа допустимого діапазону 50–250 (перше допустиме значення). Вкладення не додається, щоб один кейс відповідав одному набору даних.</t>
+          <t>50 — нижня межа допустимого діапазону 50–250 (перше допустиме значення). Вкладення не додається, щоб один кейс відповідав одному набору даних. Граничне значення a, таблиця SCRUM-108.</t>
         </is>
       </c>
       <c r="J11" s="2" t="inlineStr">
@@ -1424,7 +1456,7 @@
       </c>
       <c r="I12" s="2" t="inlineStr">
         <is>
-          <t>250 — верхня межа допустимого діапазону 50–250 (останнє допустиме значення).</t>
+          <t>250 — верхня межа допустимого діапазону 50–250 (останнє допустиме значення). Граничне значення b, таблиця SCRUM-108.</t>
         </is>
       </c>
       <c r="J12" s="2" t="inlineStr">
@@ -1487,7 +1519,7 @@
           <t>Після кроку 1: відкрито сторінку «Contact», усі поля порожні.
 Після кроків 2–5: у полях відображено введені значення: Test, Tester, tester.tc012@example.com, Customer service.
 Після кроку 6: у полі «Message» 251 символ.
-Після кроку 7: форму не надіслано, сторінка «Contact» залишається відкритою; під полем «Message» текстове повідомлення про помилку, яке називає межу в 250 символів (F-140, GUI-50; SRS 1.1 точного тексту не задає); під іншими полями повідомлень про помилки немає; повідомлення про прийняття звернення над формою відсутнє.
+Після кроку 7: форму не надіслано, сторінка «Contact» залишається відкритою; під полем «Message» текстове повідомлення про помилку (F-140, GUI-50; SRS 1.1 точного тексту не задає); під іншими полями повідомлень про помилки немає; повідомлення про прийняття звернення над формою відсутнє.
 Після кроку 8: вкладку закрито.</t>
         </is>
       </c>
@@ -1503,7 +1535,7 @@
       </c>
       <c r="I13" s="2" t="inlineStr">
         <is>
-          <t>251 — на 1 більше за верхню межу діапазону 50–250, клас недопустимих значень. Решта полів валідні.</t>
+          <t>251 — на 1 більше за верхню межу діапазону 50–250, клас недопустимих значень. Решта полів валідні. Граничне значення b+1, таблиця SCRUM-108.</t>
         </is>
       </c>
       <c r="J13" s="2" t="inlineStr">
@@ -1511,11 +1543,19 @@
           <t>Горбонос О. (КТ)</t>
         </is>
       </c>
-      <c r="K13" s="2" t="n"/>
-      <c r="L13" s="2" t="n"/>
+      <c r="K13" s="2" t="inlineStr">
+        <is>
+          <t>Дрєпіна А. (СМ)</t>
+        </is>
+      </c>
+      <c r="L13" s="2" t="inlineStr">
+        <is>
+          <t>28.10.2026</t>
+        </is>
+      </c>
       <c r="M13" s="2" t="inlineStr">
         <is>
-          <t>draft</t>
+          <t>reviewed</t>
         </is>
       </c>
       <c r="N13" s="2" t="n"/>
@@ -2125,21 +2165,23 @@
       <c r="E21" s="2" t="inlineStr">
         <is>
           <t>1. Відкрити https://practicesoftwaretesting.com у Chrome (нова сесія).
-2. Порахувати картки товарів на сторінці 1 і записати назви першої та останньої.
-3. У посторінковій навігації під каталогом натиснути «2».
-4. Натиснути кнопку ««» у посторінковій навігації.
-5. Натиснути першу картку на сторінці.
-6. Закрити вкладку.</t>
+2. Порахувати картки товарів на сторінці 1.
+3. Записати назви першої та останньої карток на сторінці 1.
+4. У посторінковій навігації під каталогом натиснути «2».
+5. У посторінковій навігації натиснути кнопку «Previous» (знак «).
+6. Натиснути першу картку на сторінці.
+7. Закрити вкладку.</t>
         </is>
       </c>
       <c r="F21" s="2" t="inlineStr">
         <is>
-          <t>Після кроку 1: головна сторінка з каталогом; під каталогом — посторінкова навігація з номерами сторінок і кнопками ««» і «»» (F-40).
+          <t>Після кроку 1: головна сторінка з каталогом; під каталогом — посторінкова навігація з номерами сторінок і кнопками переходу назад («Previous», знак «) і вперед (знак ») (F-40).
 Після кроку 2: на сторінці рівно 9 карток, розміщених сіткою у три колонки (3 ряди по 3) (F-40, GUI-20); кожна картка містить зображення, назву, шкалу класу CO2 і ціну (GUI-20).
-Після кроку 3: відкрито сторінку 2; на ній 9 карток (або менше, якщо сторінка остання); жодна назва не збігається з назвами першої та останньої карток із кроку 2.
-Після кроку 4: знову відкрито сторінку 1; перша й остання картки мають ті самі назви, що на кроці 2.
-Після кроку 5: відкрито сторінку товару з тією самою назвою, що на картці (F-40).
-Після кроку 6: вкладку закрито.</t>
+Після кроку 3: назви першої та останньої карток записано.
+Після кроку 4: відкрито сторінку 2; на ній 9 карток (або менше, якщо сторінка остання); жодна назва не збігається з назвами, записаними на кроці 3.
+Після кроку 5: знову відкрито сторінку 1; перша й остання картки мають ті самі назви, що на кроці 3.
+Після кроку 6: відкрито сторінку товару з тією самою назвою, що на картці (F-40).
+Після кроку 7: вкладку закрито.</t>
         </is>
       </c>
       <c r="G21" s="2" t="inlineStr">
@@ -2197,19 +2239,21 @@
           <t>1. Відкрити https://practicesoftwaretesting.com у Chrome (нова сесія).
 2. У блоці фільтрів за категорією записати назви підкатегорій під прапорцем «Power Tools».
 3. Позначити прапорець «Power Tools».
-4. Порахувати картки на сторінці 1.
-5. Натиснути першу картку на сторінці.
-6. Закрити вкладку.</t>
+4. Дочекатися оновлення списку карток (до 5 с).
+5. Порахувати картки і записати їхні назви.
+6. Натиснути першу картку на сторінці.
+7. Закрити вкладку.</t>
         </is>
       </c>
       <c r="F22" s="2" t="inlineStr">
         <is>
-          <t>Після кроку 1: головна сторінка з каталогом; ліворуч блок фільтрів із прапорцями груп «Hand Tools», «Power Tools», «Other» і їх підкатегорій, прапорцями брендів, повзунком ціни і «Eco-Friendly Products» (F-50).
+          <t>Після кроку 1: головна сторінка з каталогом: 9 карток і посторінкова навігація; ліворуч блок фільтрів із прапорцями груп «Hand Tools», «Power Tools», «Other» і їх підкатегорій, прапорцями брендів, повзунком ціни і «Eco-Friendly Products» (F-50).
 Після кроку 2: під «Power Tools» є щонайменше одна підкатегорія; назви записано.
-Після кроку 3: прапорець «Power Tools» позначено; список карток оновився без перезавантаження сторінки (сторінка не стає порожньою, позначка прапорця і прокрутка зберігаються) (F-50).
-Після кроку 4: на сторінці від 1 до 9 карток (F-40).
-Після кроку 5: сторінка товару; поле категорії — «Power Tools» або одна з підкатегорій, записаних на кроці 2 (F-50, F-80).
-Після кроку 6: вкладку закрито.</t>
+Після кроку 3: прапорець «Power Tools» позначено.
+Після кроку 4: список карток оновився після вибору прапорця без натискання інших кнопок (F-50).
+Після кроку 5: кількість карток відрізняється від 9 на кроці 1; усі картки — товари групи Power Tools (на demo 28.10.2026 — 5 карток без посторінкової навігації: Sheet Sander, Belt Sander, Circular Saw, Cordless Drill 24V, Cordless Drill 12V) (F-50).
+Після кроку 6: сторінка товару; поле категорії — «Power Tools» або одна з підкатегорій, записаних на кроці 2 (F-50, F-80).
+Після кроку 7: вкладку закрито.</t>
         </is>
       </c>
       <c r="G22" s="2" t="inlineStr">
@@ -2224,7 +2268,7 @@
       </c>
       <c r="I22" s="2" t="inlineStr">
         <is>
-          <t>Клас «одна категорія, без інших фільтрів»: один набір даних (task-board.md, розд. 3). Категорію товару на картці не видно, тому її перевіряємо на сторінці товару (F-80). «Power Tools» обрано як групу з підкатегоріями: перевіряє, що фільтр групи охоплює підкатегорії. Повзунок ціни 1–200 — резервний кейс КТ.</t>
+          <t>Клас «одна категорія, без інших фільтрів»: один набір даних (task-board.md, розд. 3). Критерій фільтрації — змінена кількість карток і належність усіх карток до Power Tools; категорію першої картки підтверджує сторінка товару (F-80). Крок 4 потрібен, бо на demo 28.10.2026 список оновлюється із затримкою ≈3 с. Повзунок ціни 1–200 — резервний кейс КТ.</t>
         </is>
       </c>
       <c r="J22" s="2" t="inlineStr">
@@ -2294,7 +2338,7 @@
       </c>
       <c r="I23" s="2" t="inlineStr">
         <is>
-          <t>Клас «підрядок, що є в назвах». Кейс доповнює TC-001 (регістр літер): тут перевіряється кнопка «X» і повернення повного каталогу. Негативна пара (запит без результатів) — резервний кейс СМ (TC-025+).</t>
+          <t>Клас «підрядок, що є в назвах». Кейс доповнює TC-001 (регістр літер): тут перевіряється кнопка «X» і повернення повного каталогу. Негативна пара (запит без результатів) — TC-033.</t>
         </is>
       </c>
       <c r="J23" s="2" t="inlineStr">
@@ -2335,7 +2379,7 @@
       <c r="E24" s="2" t="inlineStr">
         <is>
           <t>1. Відкрити https://practicesoftwaretesting.com у Chrome (нова сесія).
-2. У списку «Sort» вибрати: Price (Low–High).
+2. У списку «Sort» вибрати Price (Low–High) (на demo підпис «Price (Low - High)»).
 3. Записати ціни всіх карток сторінки 1 у порядку зліва направо, згори донизу.
 4. У посторінковій навігації під каталогом натиснути «2».
 5. Записати ціни всіх карток сторінки 2 у тому самому порядку.
@@ -2345,7 +2389,7 @@
       <c r="F24" s="2" t="inlineStr">
         <is>
           <t>Після кроку 1: головна сторінка з каталогом; є список «Sort» і посторінкова навігація.
-Після кроку 2: у списку «Sort» показано Price (Low–High); список містить рівно шість варіантів: Name (A–Z), Name (Z–A), Price (High–Low), Price (Low–High), CO2 Rating (A–E), CO2 Rating (E–A) (F-70); каталог оновлено.
+Після кроку 2: список «Sort» містить рівно шість варіантів, що за змістом відповідають F-70: Name (A–Z), Name (Z–A), Price (High–Low), Price (Low–High), CO2 Rating (A–E), CO2 Rating (E–A). Критерій — збіг за змістом; відмінності пунктуації (на demo 28.10.2026 — «Price (Low - High)», «CO₂ Rating (A - E)») не є підставою для failed цього кейсу, їх фіксує ІТ окремим звітом. Вибрано Price (Low–High); каталог оновлено.
 Після кроку 3: кожна наступна ціна не менша за попередню.
 Після кроку 4: відкрито сторінку 2; у списку «Sort» і далі вибрано Price (Low–High).
 Після кроку 5: кожна наступна ціна не менша за попередню; перша ціна сторінки 2 не менша за останню ціну сторінки 1 (порядок застосовано до всіх сторінок, F-70).
@@ -2414,7 +2458,7 @@
       <c r="F25" s="2" t="inlineStr">
         <is>
           <t>Після кроку 1: головна сторінка з каталогом; є картка «Combination Pliers».
-Після кроку 2: сторінка товару містить назву «Combination Pliers», категорію, бренд, ціну, клас CO2 (одна з літер A–E), опис, таблицю характеристик і блок «Related products»; поле «Quantity» зі значенням 1 і кнопками «−» і «+»; кнопки «Add to cart» (доступна), «Add to favourites», «Compare» (F-80).
+Після кроку 2: сторінка товару містить назву «Combination Pliers», категорію, бренд, ціну, шкалу класу CO2 A–E з виділеним класом товару, опис, таблицю характеристик і блок «Related products»; поле «Quantity» зі значенням 1 і кнопками «−» і «+»; кнопки «Add to cart» (доступна), «Add to favourites», «Compare» (F-80).
 Після кроку 3: не пізніше ніж за 2 с — повідомлення «Product added to shopping cart.» (F-90); на піктограмі кошика в меню — 1.
 Після кроку 4: крок «Cart»: один рядок «Combination Pliers», кількість 1 (кількість із поля «Quantity», F-90); ціна дорівнює ціні з кроку 2.
 Після кроку 5: вкладку закрито.</t>
@@ -2685,11 +2729,19 @@
           <t>Коротка К. (ТА)</t>
         </is>
       </c>
-      <c r="K28" s="2" t="n"/>
-      <c r="L28" s="2" t="n"/>
+      <c r="K28" s="2" t="inlineStr">
+        <is>
+          <t>Дрєпіна А. (СМ)</t>
+        </is>
+      </c>
+      <c r="L28" s="2" t="inlineStr">
+        <is>
+          <t>28.10.2026</t>
+        </is>
+      </c>
       <c r="M28" s="2" t="inlineStr">
         <is>
-          <t>draft</t>
+          <t>reviewed</t>
         </is>
       </c>
       <c r="N28" s="2" t="n"/>
@@ -2767,93 +2819,412 @@
           <t>Коротка К. (ТА)</t>
         </is>
       </c>
-      <c r="K29" s="2" t="n"/>
-      <c r="L29" s="2" t="n"/>
+      <c r="K29" s="2" t="inlineStr">
+        <is>
+          <t>Дрєпіна А. (СМ)</t>
+        </is>
+      </c>
+      <c r="L29" s="2" t="inlineStr">
+        <is>
+          <t>28.10.2026</t>
+        </is>
+      </c>
       <c r="M29" s="2" t="inlineStr">
         <is>
-          <t>draft</t>
+          <t>reviewed</t>
         </is>
       </c>
       <c r="N29" s="2" t="n"/>
     </row>
     <row r="30">
-      <c r="A30" s="2" t="n"/>
-      <c r="B30" s="2" t="n"/>
-      <c r="C30" s="2" t="n"/>
-      <c r="D30" s="2" t="n"/>
-      <c r="E30" s="2" t="n"/>
-      <c r="F30" s="2" t="n"/>
-      <c r="G30" s="2" t="n"/>
-      <c r="H30" s="2" t="n"/>
-      <c r="I30" s="2" t="n"/>
-      <c r="J30" s="2" t="n"/>
+      <c r="A30" s="2" t="inlineStr">
+        <is>
+          <t>TC-027</t>
+        </is>
+      </c>
+      <c r="B30" s="2" t="inlineStr">
+        <is>
+          <t>GUI-30</t>
+        </is>
+      </c>
+      <c r="C30" s="2" t="inlineStr">
+        <is>
+          <t>Спроба додати товар у кошик із кількістю 0 (менше нижньої межі) без входу</t>
+        </is>
+      </c>
+      <c r="D30" s="2" t="inlineStr">
+        <is>
+          <t>Chrome 120 або новіший, вікно 1280×800; demo доступне (збірка v2.5 від 2026-10-11 за написом у підвалі сторінки; стан звірено 28.10.2026); нова сесія (вікно інкогніто), без входу. Кошик порожній. Товар «Combination Pliers» є на першій сторінці каталогу і в наявності.</t>
+        </is>
+      </c>
+      <c r="E30" s="2" t="inlineStr">
+        <is>
+          <t>1. Відкрити https://practicesoftwaretesting.com у Chrome (нова сесія).
+2. Натиснути на картку товару «Combination Pliers».
+3. У поле «Quantity» ввести 0 (замість значення 1).
+4. Натиснути кнопку «Add to cart».
+5. Натиснути піктограму кошика у верхньому меню.
+6. Закрити вкладку.</t>
+        </is>
+      </c>
+      <c r="F30" s="2" t="inlineStr">
+        <is>
+          <t>1. Головна сторінка з каталогом; є картка «Combination Pliers».
+2. Сторінка товару «Combination Pliers»: поле «Quantity» зі значенням 1 і кнопками «−» та «+»; кнопка «Add to cart».
+3. У полі «Quantity» значення не 0 (GUI-30: лише цілі від 1 до 99). Текст помилки SRS не задає; на demo 28.10.2026 поле одразу замінює 0 на 1 без повідомлення — це спостереження записати в журнал.
+4. Товар у кількості 0 не додано: на піктограмі кошика в меню немає числа 0.
+5. Крок «Cart»: рядка «Combination Pliers» з кількістю 0 немає.
+6. Вкладку закрито.</t>
+        </is>
+      </c>
+      <c r="G30" s="2" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="H30" s="2" t="inlineStr">
+        <is>
+          <t>негативний</t>
+        </is>
+      </c>
+      <c r="I30" s="2" t="inlineStr">
+        <is>
+          <t>Граничне значення: a−1 для діапазону 1–99 (GUI-30), клас «кількість менша за 1». Позитивна пара — TC-028 (1); таблиця граничних значень — SCRUM-108.</t>
+        </is>
+      </c>
+      <c r="J30" s="2" t="inlineStr">
+        <is>
+          <t>Горбонос О. (КТ)</t>
+        </is>
+      </c>
       <c r="K30" s="2" t="n"/>
       <c r="L30" s="2" t="n"/>
-      <c r="M30" s="2" t="n"/>
+      <c r="M30" s="2" t="inlineStr">
+        <is>
+          <t>draft</t>
+        </is>
+      </c>
       <c r="N30" s="2" t="n"/>
     </row>
     <row r="31">
-      <c r="A31" s="2" t="n"/>
-      <c r="B31" s="2" t="n"/>
-      <c r="C31" s="2" t="n"/>
-      <c r="D31" s="2" t="n"/>
-      <c r="E31" s="2" t="n"/>
-      <c r="F31" s="2" t="n"/>
-      <c r="G31" s="2" t="n"/>
-      <c r="H31" s="2" t="n"/>
-      <c r="I31" s="2" t="n"/>
-      <c r="J31" s="2" t="n"/>
-      <c r="K31" s="2" t="n"/>
-      <c r="L31" s="2" t="n"/>
-      <c r="M31" s="2" t="n"/>
+      <c r="A31" s="2" t="inlineStr">
+        <is>
+          <t>TC-028</t>
+        </is>
+      </c>
+      <c r="B31" s="2" t="inlineStr">
+        <is>
+          <t>GUI-30</t>
+        </is>
+      </c>
+      <c r="C31" s="2" t="inlineStr">
+        <is>
+          <t>Додавання товару в кошик із кількістю 1 (нижня межа) без входу</t>
+        </is>
+      </c>
+      <c r="D31" s="2" t="inlineStr">
+        <is>
+          <t>Chrome 120 або новіший, вікно 1280×800; demo доступне (збірка v2.5 від 2026-10-11 за написом у підвалі сторінки; стан звірено 28.10.2026); нова сесія (вікно інкогніто), без входу. Кошик порожній. Товар «Combination Pliers» є на першій сторінці каталогу і в наявності.</t>
+        </is>
+      </c>
+      <c r="E31" s="2" t="inlineStr">
+        <is>
+          <t>1. Відкрити https://practicesoftwaretesting.com у Chrome (нова сесія).
+2. Натиснути на картку товару «Combination Pliers».
+3. У поле «Quantity» ввести 1 (замість наявного значення).
+4. Натиснути кнопку «Add to cart».
+5. Натиснути піктограму кошика у верхньому меню.
+6. У рядку «Combination Pliers» натиснути червону кнопку видалення.
+7. Закрити вкладку.</t>
+        </is>
+      </c>
+      <c r="F31" s="2" t="inlineStr">
+        <is>
+          <t>1. Головна сторінка з каталогом; є картка «Combination Pliers».
+2. Сторінка товару «Combination Pliers»: ціна; поле «Quantity» зі значенням 1 і кнопками «−» та «+»; кнопка «Add to cart».
+3. У полі «Quantity» — 1; під полем повідомлень про помилку немає.
+4. Не пізніше ніж за 2 с — повідомлення «Product added to shopping cart.»; на піктограмі кошика в меню — 1.
+5. Крок «Cart»: один рядок «Combination Pliers», «Quantity» — 1, «Total» дорівнює ціні з кроку 2.
+6. Рядок видалено; замість таблиці — текстове повідомлення про порожній кошик (на demo 28.10.2026 — «The cart is empty. Nothing to display.»).
+7. Вкладку закрито.</t>
+        </is>
+      </c>
+      <c r="G31" s="2" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="H31" s="2" t="inlineStr">
+        <is>
+          <t>позитивний</t>
+        </is>
+      </c>
+      <c r="I31" s="2" t="inlineStr">
+        <is>
+          <t>Граничне значення: a, нижня межа діапазону 1–99 (GUI-30), клас «допустима кількість». Негативна пара — TC-027 (0); таблиця граничних значень — SCRUM-108.</t>
+        </is>
+      </c>
+      <c r="J31" s="2" t="inlineStr">
+        <is>
+          <t>Горбонос О. (КТ)</t>
+        </is>
+      </c>
+      <c r="K31" s="2" t="inlineStr">
+        <is>
+          <t>Дрєпіна А. (СМ)</t>
+        </is>
+      </c>
+      <c r="L31" s="2" t="inlineStr">
+        <is>
+          <t>28.10.2026</t>
+        </is>
+      </c>
+      <c r="M31" s="2" t="inlineStr">
+        <is>
+          <t>reviewed</t>
+        </is>
+      </c>
       <c r="N31" s="2" t="n"/>
     </row>
     <row r="32">
-      <c r="A32" s="2" t="n"/>
-      <c r="B32" s="2" t="n"/>
-      <c r="C32" s="2" t="n"/>
-      <c r="D32" s="2" t="n"/>
-      <c r="E32" s="2" t="n"/>
-      <c r="F32" s="2" t="n"/>
-      <c r="G32" s="2" t="n"/>
-      <c r="H32" s="2" t="n"/>
-      <c r="I32" s="2" t="n"/>
-      <c r="J32" s="2" t="n"/>
-      <c r="K32" s="2" t="n"/>
-      <c r="L32" s="2" t="n"/>
-      <c r="M32" s="2" t="n"/>
+      <c r="A32" s="2" t="inlineStr">
+        <is>
+          <t>TC-031</t>
+        </is>
+      </c>
+      <c r="B32" s="2" t="inlineStr">
+        <is>
+          <t>F-130</t>
+        </is>
+      </c>
+      <c r="C32" s="2" t="inlineStr">
+        <is>
+          <t>Особистий кабінет покупця: відкриваються розділи «My profile», «My favorites», «My invoices», «My messages»</t>
+        </is>
+      </c>
+      <c r="D32" s="2" t="inlineStr">
+        <is>
+          <t>Chrome 120 або новіший, вікно 1280×800; demo доступне (збірка v2.5 від 2026-10-11 за написом у підвалі сторінки; стан звірено 28.10.2026); нова сесія (вікно інкогніто), без входу. Спільний обліковий запис покупця customer@practicesoftwaretesting.com / welcome01 (SRS 1.1, розд. 2.2); пароль спільного облікового запису не змінювати (етика demo: інструкція спринта 3, п. 1.7; методичка, п. 5.4), дані профілю не редагувати. Кроки після входу записано за SRS 1.1 і будуть звірені на пробному прогоні.</t>
+        </is>
+      </c>
+      <c r="E32" s="2" t="inlineStr">
+        <is>
+          <t>1. Відкрити https://practicesoftwaretesting.com у Chrome (нова сесія).
+2. Натиснути «Sign in» у верхньому меню.
+3. У поле «Email address» ввести: customer@practicesoftwaretesting.com
+4. У поле «Password» ввести: welcome01
+5. Натиснути кнопку «Login».
+6. Натиснути ім'я користувача у верхньому меню.
+7. У розкривному меню натиснути «My profile».
+8. Натиснути ім'я користувача у верхньому меню.
+9. У розкривному меню натиснути «My favorites».
+10. Натиснути ім'я користувача у верхньому меню.
+11. У розкривному меню натиснути «My invoices».
+12. Натиснути ім'я користувача у верхньому меню.
+13. У розкривному меню натиснути «My messages».
+14. Натиснути ім'я користувача у верхньому меню.
+15. У розкривному меню натиснути «Sign out».
+16. Закрити вкладку.</t>
+        </is>
+      </c>
+      <c r="F32" s="2" t="inlineStr">
+        <is>
+          <t>Після кроку 1: головна сторінка з каталогом; у шапці замість імені користувача пункт «Sign in» (GUI-10).
+Після кроку 2: сторінка входу (адреса містить /auth/login) з полями «Email address» і «Password» та кнопкою «Login».
+Після кроків 3–4: у полі «Email address» — customer@practicesoftwaretesting.com; символи пароля замасковано.
+Після кроку 5: відкрито сторінку особистого кабінету (адреса містить /account); у шапці замість «Sign in» — ім'я користувача (GUI-10).
+Після кроку 6: розкривне меню з розділами «My profile», «My favorites», «My invoices», «My messages» і пунктом «Sign out» (F-130, GUI-10).
+Після кроку 7: відкрито розділ «My profile»: є дані імені, прізвища, адреси й телефону та поля зміни пароля — поточний пароль, новий пароль, підтвердження нового пароля (F-130). Дані не змінювати.
+Після кроку 8: розкривне меню відкрито.
+Після кроку 9: відкрито розділ «My favorites» (адреса містить /account/favorites); показано список обраного або порожній список (F-130).
+Після кроку 10: розкривне меню відкрито.
+Після кроку 11: відкрито розділ «My invoices»: список замовлень з колонками номер, дата, сума, статус або порожній список, якщо замовлень немає (F-130).
+Після кроку 12: розкривне меню відкрито.
+Після кроку 13: відкрито розділ «My messages»: перелік звернень і відповідей на них або порожній перелік (F-130).
+Після кроку 14: розкривне меню відкрито.
+Після кроку 15: сеанс завершено; у шапці знову «Sign in» (GUI-10).
+Після кроку 16: вкладку закрито.</t>
+        </is>
+      </c>
+      <c r="G32" s="2" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="H32" s="2" t="inlineStr">
+        <is>
+          <t>позитивний</t>
+        </is>
+      </c>
+      <c r="I32" s="2" t="inlineStr">
+        <is>
+          <t>Клас «авторизований покупець зі спільним тестовим обліковим записом» (SRS 1.1, розд. 2.2): розділи кабінету перевіряються лише переглядом. Зміна пароля й редагування профілю на спільному обліковому записі заборонені етикою demo, тому не виконуються. Деталі замовлення і завантаження PDF (F-130) не входять до цього кейсу: залежать від наявних замовлень у спільному обліковому записі; за потреби — окремий резервний кейс. Вихід на кроці 15 лишає demo в початковому стані.</t>
+        </is>
+      </c>
+      <c r="J32" s="2" t="inlineStr">
+        <is>
+          <t>Горбонос О. (КТ)</t>
+        </is>
+      </c>
+      <c r="K32" s="2" t="inlineStr">
+        <is>
+          <t>Дрєпіна А. (СМ)</t>
+        </is>
+      </c>
+      <c r="L32" s="2" t="inlineStr">
+        <is>
+          <t>28.10.2026</t>
+        </is>
+      </c>
+      <c r="M32" s="2" t="inlineStr">
+        <is>
+          <t>reviewed</t>
+        </is>
+      </c>
       <c r="N32" s="2" t="n"/>
     </row>
     <row r="33">
-      <c r="A33" s="2" t="n"/>
-      <c r="B33" s="2" t="n"/>
-      <c r="C33" s="2" t="n"/>
-      <c r="D33" s="2" t="n"/>
-      <c r="E33" s="2" t="n"/>
-      <c r="F33" s="2" t="n"/>
-      <c r="G33" s="2" t="n"/>
-      <c r="H33" s="2" t="n"/>
-      <c r="I33" s="2" t="n"/>
-      <c r="J33" s="2" t="n"/>
+      <c r="A33" s="2" t="inlineStr">
+        <is>
+          <t>TC-032</t>
+        </is>
+      </c>
+      <c r="B33" s="2" t="inlineStr">
+        <is>
+          <t>S-20</t>
+        </is>
+      </c>
+      <c r="C33" s="2" t="inlineStr">
+        <is>
+          <t>Неавторизований відвідувач не потрапляє в кабінет і на кроки 3–4 оформлення замовлення</t>
+        </is>
+      </c>
+      <c r="D33" s="2" t="inlineStr">
+        <is>
+          <t>Chrome 120 або новіший, вікно 1280×800; demo доступне (збірка v2.5 від 2026-10-11 за написом у підвалі сторінки; стан звірено 28.10.2026); нова сесія (вікно інкогніто), без входу. Кошик порожній. Товар «Combination Pliers» є на першій сторінці каталогу і в наявності.</t>
+        </is>
+      </c>
+      <c r="E33" s="2" t="inlineStr">
+        <is>
+          <t>1. Відкрити https://practicesoftwaretesting.com у Chrome (нова сесія).
+2. В адресному рядку відкрити https://practicesoftwaretesting.com/account.
+3. В адресному рядку відкрити https://practicesoftwaretesting.com/account/favorites.
+4. В адресному рядку відкрити https://practicesoftwaretesting.com.
+5. Натиснути на картку товару «Combination Pliers».
+6. Натиснути кнопку «Add to cart».
+7. Натиснути піктограму кошика у верхньому меню.
+8. Натиснути кнопку «Proceed to checkout».
+9. Закрити вкладку.</t>
+        </is>
+      </c>
+      <c r="F33" s="2" t="inlineStr">
+        <is>
+          <t>Після кроку 1: головна сторінка з каталогом; у меню — «Sign in».
+Після кроку 2: відкрито сторінку входу (адреса містить /auth/login); особистий кабінет не відкрито; у меню — «Sign in» (S-20).
+Після кроку 3: відкрито сторінку входу (адреса містить /auth/login); розділ «My favorites» не показано (S-20).
+Після кроку 4: головна сторінка з каталогом; є картка «Combination Pliers».
+Після кроку 5: сторінка товару «Combination Pliers» з кнопкою «Add to cart».
+Після кроку 6: не пізніше ніж за 2 с — повідомлення «Product added to shopping cart.»; на піктограмі кошика в меню — 1.
+Після кроку 7: крок «Cart»: один рядок «Combination Pliers», кнопка «Proceed to checkout».
+Після кроку 8: відкрито крок «Sign in» (2) з формою входу («Email address», «Password», «Login»); кроки «Billing Address» (3) і «Payment» (4) для неавторизованого користувача недоступні (S-20, SRS 1.1). На demo 28.10.2026 крок 2 містить ще вкладку «Continue as Guest» («Checkout without creating an account») з полями email, ім'я, прізвище, яка веде до кроку 3; це розбіжність із S-20 — записати в журнал як спостереження (кандидат у дефект).
+Після кроку 9: вкладку закрито.</t>
+        </is>
+      </c>
+      <c r="G33" s="2" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="H33" s="2" t="inlineStr">
+        <is>
+          <t>негативний</t>
+        </is>
+      </c>
+      <c r="I33" s="2" t="inlineStr">
+        <is>
+          <t>Клас «неавторизований відвідувач»: прямий перехід за адресами кабінету (/account, /account/favorites) і спроба пройти кроки 3–4 оформлення без входу (S-20). Вхід не виконується, паролі не вводяться. Маскування пароля (S-20) перевіряють TC-004, TC-005–TC-008, TC-015, TC-026; перенаправлення після «Sign out» окремо не перевіряється, бо потребує входу спільним обліковим записом (S-20 покрито частково). Дані вигадані, одна додана в кошик позиція не змінює дані demo (п. 1.7).</t>
+        </is>
+      </c>
+      <c r="J33" s="2" t="inlineStr">
+        <is>
+          <t>Горбонос О. (КТ)</t>
+        </is>
+      </c>
       <c r="K33" s="2" t="n"/>
       <c r="L33" s="2" t="n"/>
-      <c r="M33" s="2" t="n"/>
+      <c r="M33" s="2" t="inlineStr">
+        <is>
+          <t>draft</t>
+        </is>
+      </c>
       <c r="N33" s="2" t="n"/>
     </row>
     <row r="34">
-      <c r="A34" s="2" t="n"/>
-      <c r="B34" s="2" t="n"/>
-      <c r="C34" s="2" t="n"/>
-      <c r="D34" s="2" t="n"/>
-      <c r="E34" s="2" t="n"/>
-      <c r="F34" s="2" t="n"/>
-      <c r="G34" s="2" t="n"/>
-      <c r="H34" s="2" t="n"/>
-      <c r="I34" s="2" t="n"/>
-      <c r="J34" s="2" t="n"/>
+      <c r="A34" s="2" t="inlineStr">
+        <is>
+          <t>TC-033</t>
+        </is>
+      </c>
+      <c r="B34" s="2" t="inlineStr">
+        <is>
+          <t>F-60</t>
+        </is>
+      </c>
+      <c r="C34" s="2" t="inlineStr">
+        <is>
+          <t>Пошук за запитом без збігів «xyzabc»: карток немає, «X» повертає повний каталог</t>
+        </is>
+      </c>
+      <c r="D34" s="2" t="inlineStr">
+        <is>
+          <t>Chrome 120 або новіший, вікно 1280×800; demo доступне (збірка v2.5 від 2026-10-11 за написом у підвалі сторінки, стан звірено 28.10.2026); нова сесія, без входу. Активних фільтрів і сортування немає; у каталозі немає товарів, назва яких містить «xyzabc».</t>
+        </is>
+      </c>
+      <c r="E34" s="2" t="inlineStr">
+        <is>
+          <t>1. Відкрити https://practicesoftwaretesting.com у Chrome (нова сесія).
+2. У поле пошуку «Search» ввести: xyzabc
+3. Натиснути кнопку «Search».
+4. Натиснути кнопку «X» біля поля пошуку.
+5. Закрити вкладку.</t>
+        </is>
+      </c>
+      <c r="F34" s="2" t="inlineStr">
+        <is>
+          <t>Після кроку 1: головна сторінка з каталогом, полем «Search» і кнопками «X» та «Search».
+Після кроку 2: у полі «Search» — xyzabc.
+Після кроку 3: заголовок «Searched for: xyzabc»; карток товарів немає (F-60); замість списку — текстове повідомлення про відсутність товарів (SRS 1.1 тексту не задає; на demo 28.10.2026 — «There are no products found.»).
+Після кроку 4: поле «Search» порожнє; заголовка «Searched for:» немає; показано повний каталог із 9 картками і посторінковою навігацією (F-60, F-40).
+Після кроку 5: вкладку закрито.</t>
+        </is>
+      </c>
+      <c r="G34" s="2" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="H34" s="2" t="inlineStr">
+        <is>
+          <t>негативний</t>
+        </is>
+      </c>
+      <c r="I34" s="2" t="inlineStr">
+        <is>
+          <t>Клас «запит, якого немає в жодній назві» для F-60. xyzabc — довільний набір латинських літер, без спецсимволів і атакувальних рядків (етика demo, п. 1.7). Позитивна пара — TC-022. Номер — наступний вільний після TC-032 [ЗАПОВНИТИ: підтвердити з ТА].</t>
+        </is>
+      </c>
+      <c r="J34" s="2" t="inlineStr">
+        <is>
+          <t>Дрєпіна А. (СМ)</t>
+        </is>
+      </c>
       <c r="K34" s="2" t="n"/>
       <c r="L34" s="2" t="n"/>
-      <c r="M34" s="2" t="n"/>
+      <c r="M34" s="2" t="inlineStr">
+        <is>
+          <t>draft</t>
+        </is>
+      </c>
       <c r="N34" s="2" t="n"/>
     </row>
     <row r="35">
@@ -4379,7 +4750,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N29"/>
+  <dimension ref="A1:N36"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -4791,9 +5162,9 @@
           <t>так</t>
         </is>
       </c>
-      <c r="F6" s="6" t="inlineStr">
-        <is>
-          <t>ні</t>
+      <c r="F6" s="2" t="inlineStr">
+        <is>
+          <t>так</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr">
@@ -4801,9 +5172,9 @@
           <t>так</t>
         </is>
       </c>
-      <c r="H6" s="6" t="inlineStr">
-        <is>
-          <t>ні</t>
+      <c r="H6" s="2" t="inlineStr">
+        <is>
+          <t>так</t>
         </is>
       </c>
       <c r="I6" s="2" t="inlineStr">
@@ -4824,11 +5195,20 @@
       <c r="L6" s="2" t="inlineStr">
         <is>
           <t>П3: адреса shopline.ta005@example.com фіксована — після першого виконання вона зареєстрована, тож повторне виконання (ІТ повторює кожен failed; спринти 4–5) впаде на кроці 16. Додати дату виконання, як у TC-019: shopline.ta005.ДДММРРРР@example.com.
-П5: крок 20 «У меню користувача натиснути Sign out» — дві дії; розбити: натиснути ім'я користувача / натиснути «Sign out».</t>
-        </is>
-      </c>
-      <c r="M6" s="2" t="n"/>
-      <c r="N6" s="2" t="n"/>
+П5: крок 20 «У меню користувача натиснути Sign out» — дві дії; розбити: натиснути ім'я користувача / натиснути «Sign out».
+Фаза 2 (28.10.2026, коміт 3a520b0): П3 виправлено (адреса з датою виконання), П5 виправлено (вихід двома кроками). Рекомендація: при повторному виконанні того самого дня (повтор failed) додати до адреси суфікс, напр. .28102026b.</t>
+        </is>
+      </c>
+      <c r="M6" s="2" t="inlineStr">
+        <is>
+          <t>так</t>
+        </is>
+      </c>
+      <c r="N6" s="2" t="inlineStr">
+        <is>
+          <t>28.10.2026</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
@@ -4856,9 +5236,9 @@
           <t>так</t>
         </is>
       </c>
-      <c r="F7" s="6" t="inlineStr">
-        <is>
-          <t>ні</t>
+      <c r="F7" s="2" t="inlineStr">
+        <is>
+          <t>так</t>
         </is>
       </c>
       <c r="G7" s="2" t="inlineStr">
@@ -4888,11 +5268,20 @@
       </c>
       <c r="L7" s="2" t="inlineStr">
         <is>
-          <t>П3: адреса shopline.ta006@example.com фіксована — після першого виконання вона зареєстрована, тож повторне виконання (ІТ повторює кожен failed; спринти 4–5) впаде на кроці 16. Додати дату виконання, як у TC-019: shopline.ta006.ДДММРРРР@example.com. Межа a−1 (7 символів) і склад пароля перевірено.</t>
-        </is>
-      </c>
-      <c r="M7" s="2" t="n"/>
-      <c r="N7" s="2" t="n"/>
+          <t>П3: адреса shopline.ta006@example.com фіксована — після першого виконання вона зареєстрована, тож повторне виконання (ІТ повторює кожен failed; спринти 4–5) впаде на кроці 16. Додати дату виконання, як у TC-019: shopline.ta006.ДДММРРРР@example.com. Межа a−1 (7 символів) і склад пароля перевірено.
+Фаза 2 (28.10.2026, коміт 3a520b0): П3 виправлено (адреса з датою виконання).</t>
+        </is>
+      </c>
+      <c r="M7" s="2" t="inlineStr">
+        <is>
+          <t>так</t>
+        </is>
+      </c>
+      <c r="N7" s="2" t="inlineStr">
+        <is>
+          <t>28.10.2026</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
@@ -4920,9 +5309,9 @@
           <t>так</t>
         </is>
       </c>
-      <c r="F8" s="6" t="inlineStr">
-        <is>
-          <t>ні</t>
+      <c r="F8" s="2" t="inlineStr">
+        <is>
+          <t>так</t>
         </is>
       </c>
       <c r="G8" s="2" t="inlineStr">
@@ -4930,9 +5319,9 @@
           <t>так</t>
         </is>
       </c>
-      <c r="H8" s="6" t="inlineStr">
-        <is>
-          <t>ні</t>
+      <c r="H8" s="2" t="inlineStr">
+        <is>
+          <t>так</t>
         </is>
       </c>
       <c r="I8" s="2" t="inlineStr">
@@ -4953,11 +5342,20 @@
       <c r="L8" s="2" t="inlineStr">
         <is>
           <t>П3: адреса shopline.ta007@example.com фіксована — після першого виконання вона зареєстрована, тож повторне виконання (ІТ повторює кожен failed; спринти 4–5) впаде на кроці 16. Додати дату виконання, як у TC-019: shopline.ta007.ДДММРРРР@example.com.
-П5: крок 20 «У меню користувача натиснути Sign out» — дві дії; розбити: натиснути ім'я користувача / натиснути «Sign out». Межа a = 8 перевірено.</t>
-        </is>
-      </c>
-      <c r="M8" s="2" t="n"/>
-      <c r="N8" s="2" t="n"/>
+П5: крок 20 «У меню користувача натиснути Sign out» — дві дії; розбити: натиснути ім'я користувача / натиснути «Sign out». Межа a = 8 перевірено.
+Фаза 2 (28.10.2026, коміт 3a520b0): П3, П5 виправлено. Рекомендація щодо повтору того самого дня — як у TC-005.</t>
+        </is>
+      </c>
+      <c r="M8" s="2" t="inlineStr">
+        <is>
+          <t>так</t>
+        </is>
+      </c>
+      <c r="N8" s="2" t="inlineStr">
+        <is>
+          <t>28.10.2026</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
@@ -5072,9 +5470,9 @@
           <t>так</t>
         </is>
       </c>
-      <c r="I10" s="6" t="inlineStr">
-        <is>
-          <t>ні</t>
+      <c r="I10" s="2" t="inlineStr">
+        <is>
+          <t>так</t>
         </is>
       </c>
       <c r="J10" s="2" t="inlineStr">
@@ -5089,11 +5487,20 @@
       </c>
       <c r="L10" s="2" t="inlineStr">
         <is>
-          <t>П6: «повідомлення, яке називає межу в 50 символів» — SRS 1.1 (F-140, GUI-50) цього не вимагає; через це кейс може дати хибний failed. Залишити: текстове повідомлення про помилку безпосередньо під полем «Message»; форму не надіслано. Довжину рядка перевірено: 49 символів.</t>
-        </is>
-      </c>
-      <c r="M10" s="2" t="n"/>
-      <c r="N10" s="2" t="n"/>
+          <t>П6: «повідомлення, яке називає межу в 50 символів» — SRS 1.1 (F-140, GUI-50) цього не вимагає; через це кейс може дати хибний failed. Залишити: текстове повідомлення про помилку безпосередньо під полем «Message»; форму не надіслано. Довжину рядка перевірено: 49 символів.
+Фаза 2 (28.10.2026, коміт c47dce6): П6 виправлено — критерій «текстове повідомлення під полем «Message»» без вимоги називати межу.</t>
+        </is>
+      </c>
+      <c r="M10" s="2" t="inlineStr">
+        <is>
+          <t>так</t>
+        </is>
+      </c>
+      <c r="N10" s="2" t="inlineStr">
+        <is>
+          <t>28.10.2026</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
@@ -5280,9 +5687,9 @@
           <t>так</t>
         </is>
       </c>
-      <c r="I13" s="6" t="inlineStr">
-        <is>
-          <t>ні</t>
+      <c r="I13" s="2" t="inlineStr">
+        <is>
+          <t>так</t>
         </is>
       </c>
       <c r="J13" s="2" t="inlineStr">
@@ -5297,11 +5704,20 @@
       </c>
       <c r="L13" s="2" t="inlineStr">
         <is>
-          <t>П6: «повідомлення, яке називає межу в 250 символів» — SRS 1.1 (F-140, GUI-50) цього не вимагає; через це кейс може дати хибний failed. Залишити: текстове повідомлення про помилку безпосередньо під полем «Message»; форму не надіслано. Довжину рядка перевірено: 251 символ.</t>
-        </is>
-      </c>
-      <c r="M13" s="2" t="n"/>
-      <c r="N13" s="2" t="n"/>
+          <t>П6: «повідомлення, яке називає межу в 250 символів» — SRS 1.1 (F-140, GUI-50) цього не вимагає; через це кейс може дати хибний failed. Залишити: текстове повідомлення про помилку безпосередньо під полем «Message»; форму не надіслано. Довжину рядка перевірено: 251 символ.
+Фаза 2 (28.10.2026, коміт c47dce6): П6 виправлено — як у TC-009.</t>
+        </is>
+      </c>
+      <c r="M13" s="2" t="inlineStr">
+        <is>
+          <t>так</t>
+        </is>
+      </c>
+      <c r="N13" s="2" t="inlineStr">
+        <is>
+          <t>28.10.2026</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
@@ -5818,17 +6234,61 @@
           <t>Горбонос О. (КТ)</t>
         </is>
       </c>
-      <c r="C21" s="2" t="n"/>
-      <c r="D21" s="2" t="n"/>
-      <c r="E21" s="2" t="n"/>
-      <c r="F21" s="2" t="n"/>
-      <c r="G21" s="2" t="n"/>
-      <c r="H21" s="2" t="n"/>
-      <c r="I21" s="2" t="n"/>
-      <c r="J21" s="2" t="n"/>
-      <c r="K21" s="2" t="n"/>
-      <c r="L21" s="2" t="n"/>
-      <c r="M21" s="2" t="n"/>
+      <c r="C21" s="2" t="inlineStr">
+        <is>
+          <t>28.10.2026</t>
+        </is>
+      </c>
+      <c r="D21" s="2" t="inlineStr">
+        <is>
+          <t>так</t>
+        </is>
+      </c>
+      <c r="E21" s="2" t="inlineStr">
+        <is>
+          <t>так</t>
+        </is>
+      </c>
+      <c r="F21" s="2" t="inlineStr">
+        <is>
+          <t>так</t>
+        </is>
+      </c>
+      <c r="G21" s="2" t="inlineStr">
+        <is>
+          <t>так</t>
+        </is>
+      </c>
+      <c r="H21" s="6" t="inlineStr">
+        <is>
+          <t>ні</t>
+        </is>
+      </c>
+      <c r="I21" s="2" t="inlineStr">
+        <is>
+          <t>так</t>
+        </is>
+      </c>
+      <c r="J21" s="2" t="inlineStr">
+        <is>
+          <t>так</t>
+        </is>
+      </c>
+      <c r="K21" s="2" t="inlineStr">
+        <is>
+          <t>так</t>
+        </is>
+      </c>
+      <c r="L21" s="2" t="inlineStr">
+        <is>
+          <t>П5: крок 2 містить дві дії — «порахувати картки» і «записати назви першої та останньої». Розділити на два кроки. Крок 4: запис «кнопку ««»» читається важко через вкладені лапки — написати «кнопку «Previous» (знак «)». Перевірено на demo 28.10.2026: на сторінці 1 дев'ять карток у три колонки (3 ряди по 3), на картці зображення, назва, шкала CO2 і ціна; сторінка 2 містить інші товари; «Previous» повертає на сторінку 1 з тими самими першою й останньою картками.</t>
+        </is>
+      </c>
+      <c r="M21" s="2" t="inlineStr">
+        <is>
+          <t>так</t>
+        </is>
+      </c>
       <c r="N21" s="2" t="n"/>
     </row>
     <row r="22">
@@ -5842,17 +6302,61 @@
           <t>Горбонос О. (КТ)</t>
         </is>
       </c>
-      <c r="C22" s="2" t="n"/>
-      <c r="D22" s="2" t="n"/>
-      <c r="E22" s="2" t="n"/>
-      <c r="F22" s="2" t="n"/>
-      <c r="G22" s="2" t="n"/>
-      <c r="H22" s="2" t="n"/>
-      <c r="I22" s="2" t="n"/>
-      <c r="J22" s="2" t="n"/>
-      <c r="K22" s="2" t="n"/>
-      <c r="L22" s="2" t="n"/>
-      <c r="M22" s="2" t="n"/>
+      <c r="C22" s="2" t="inlineStr">
+        <is>
+          <t>28.10.2026</t>
+        </is>
+      </c>
+      <c r="D22" s="2" t="inlineStr">
+        <is>
+          <t>так</t>
+        </is>
+      </c>
+      <c r="E22" s="2" t="inlineStr">
+        <is>
+          <t>так</t>
+        </is>
+      </c>
+      <c r="F22" s="2" t="inlineStr">
+        <is>
+          <t>так</t>
+        </is>
+      </c>
+      <c r="G22" s="2" t="inlineStr">
+        <is>
+          <t>так</t>
+        </is>
+      </c>
+      <c r="H22" s="2" t="inlineStr">
+        <is>
+          <t>так</t>
+        </is>
+      </c>
+      <c r="I22" s="6" t="inlineStr">
+        <is>
+          <t>ні</t>
+        </is>
+      </c>
+      <c r="J22" s="2" t="inlineStr">
+        <is>
+          <t>так</t>
+        </is>
+      </c>
+      <c r="K22" s="2" t="inlineStr">
+        <is>
+          <t>так</t>
+        </is>
+      </c>
+      <c r="L22" s="2" t="inlineStr">
+        <is>
+          <t>П6: «Після кроку 4: на сторінці від 1 до 9 карток» не перевіряє фільтрацію — цю умову виконує й незафільтрований список (9 карток). Указати критерій: кількість карток змінилась порівняно з початковою (на demo 28.10.2026 — 5 карток, без пагінації) і назви належать товарам Power Tools (Sheet Sander, Belt Sander, Circular Saw, Cordless Drill 24V, Cordless Drill 12V). «Без перезавантаження сторінки», «прокрутка зберігаються» вручну надійно не перевіряються — сформулювати через F-50 («список оновлюється після вибору прапорця»). Список на demo оновлюється із затримкою близько 3 с — додати «дочекатися оновлення списку», інакше можливий хибний failed. Крок 5 перевірено: на сторінці товару Sheet Sander категорія — Sander (підкатегорія Power Tools).</t>
+        </is>
+      </c>
+      <c r="M22" s="2" t="inlineStr">
+        <is>
+          <t>так</t>
+        </is>
+      </c>
       <c r="N22" s="2" t="n"/>
     </row>
     <row r="23">
@@ -5866,17 +6370,61 @@
           <t>Горбонос О. (КТ)</t>
         </is>
       </c>
-      <c r="C23" s="2" t="n"/>
-      <c r="D23" s="2" t="n"/>
-      <c r="E23" s="2" t="n"/>
-      <c r="F23" s="2" t="n"/>
-      <c r="G23" s="2" t="n"/>
-      <c r="H23" s="2" t="n"/>
-      <c r="I23" s="2" t="n"/>
-      <c r="J23" s="2" t="n"/>
-      <c r="K23" s="2" t="n"/>
-      <c r="L23" s="2" t="n"/>
-      <c r="M23" s="2" t="n"/>
+      <c r="C23" s="2" t="inlineStr">
+        <is>
+          <t>28.10.2026</t>
+        </is>
+      </c>
+      <c r="D23" s="2" t="inlineStr">
+        <is>
+          <t>так</t>
+        </is>
+      </c>
+      <c r="E23" s="2" t="inlineStr">
+        <is>
+          <t>так</t>
+        </is>
+      </c>
+      <c r="F23" s="2" t="inlineStr">
+        <is>
+          <t>так</t>
+        </is>
+      </c>
+      <c r="G23" s="2" t="inlineStr">
+        <is>
+          <t>так</t>
+        </is>
+      </c>
+      <c r="H23" s="2" t="inlineStr">
+        <is>
+          <t>так</t>
+        </is>
+      </c>
+      <c r="I23" s="2" t="inlineStr">
+        <is>
+          <t>так</t>
+        </is>
+      </c>
+      <c r="J23" s="2" t="inlineStr">
+        <is>
+          <t>так</t>
+        </is>
+      </c>
+      <c r="K23" s="6" t="inlineStr">
+        <is>
+          <t>ні</t>
+        </is>
+      </c>
+      <c r="L23" s="2" t="inlineStr">
+        <is>
+          <t>П8: для поля пошуку немає негативної пари. Вона заплановена як резервний кейс (task-board.md, розд. 3), але ще не написана — додати кейс із запитом без результатів. Приклад на demo 28.10.2026 для запиту xyzabc: заголовок «Searched for: xyzabc», карток немає, повідомлення «There are no products found.» (SRS 1.1 тексту не задає). Номер видає ТА. Позитивний кейс перевірено: запит Hammer дає 6 карток, усі містять hammer, кнопка «X» повертає повний каталог з тією самою першою карткою.</t>
+        </is>
+      </c>
+      <c r="M23" s="2" t="inlineStr">
+        <is>
+          <t>так</t>
+        </is>
+      </c>
       <c r="N23" s="2" t="n"/>
     </row>
     <row r="24">
@@ -5890,17 +6438,61 @@
           <t>Горбонос О. (КТ)</t>
         </is>
       </c>
-      <c r="C24" s="2" t="n"/>
-      <c r="D24" s="2" t="n"/>
-      <c r="E24" s="2" t="n"/>
-      <c r="F24" s="2" t="n"/>
-      <c r="G24" s="2" t="n"/>
-      <c r="H24" s="2" t="n"/>
-      <c r="I24" s="2" t="n"/>
-      <c r="J24" s="2" t="n"/>
-      <c r="K24" s="2" t="n"/>
-      <c r="L24" s="2" t="n"/>
-      <c r="M24" s="2" t="n"/>
+      <c r="C24" s="2" t="inlineStr">
+        <is>
+          <t>28.10.2026</t>
+        </is>
+      </c>
+      <c r="D24" s="2" t="inlineStr">
+        <is>
+          <t>так</t>
+        </is>
+      </c>
+      <c r="E24" s="2" t="inlineStr">
+        <is>
+          <t>так</t>
+        </is>
+      </c>
+      <c r="F24" s="2" t="inlineStr">
+        <is>
+          <t>так</t>
+        </is>
+      </c>
+      <c r="G24" s="2" t="inlineStr">
+        <is>
+          <t>так</t>
+        </is>
+      </c>
+      <c r="H24" s="2" t="inlineStr">
+        <is>
+          <t>так</t>
+        </is>
+      </c>
+      <c r="I24" s="6" t="inlineStr">
+        <is>
+          <t>ні</t>
+        </is>
+      </c>
+      <c r="J24" s="2" t="inlineStr">
+        <is>
+          <t>так</t>
+        </is>
+      </c>
+      <c r="K24" s="2" t="inlineStr">
+        <is>
+          <t>так</t>
+        </is>
+      </c>
+      <c r="L24" s="2" t="inlineStr">
+        <is>
+          <t>П6: назви варіантів у списку «Sort» (Price (Low–High), Name (A–Z), CO2 Rating (A–E)) взято зі SRS 1.1, а на demo 28.10.2026 вони подані як «Price (Low - High)», «Name (A - Z)», «CO₂ Rating (A - E)» (дефіс з пробілами, «CO₂»). Тестувальниця може поставити failed лише через пунктуацію. Указати: назви за SRS, а критерій — шість варіантів, що збігаються за змістом; розбіжність тире записати окремо (кандидат у дефект рівня Trivial для ІТ). Функціонально перевірено: Price (Low - High) сортує сторінки 1 і 2 за зростанням, перша ціна сторінки 2 (10.07) не менша за останню сторінки 1 (9.17), вибраний порядок на сторінці 2 зберігається.</t>
+        </is>
+      </c>
+      <c r="M24" s="2" t="inlineStr">
+        <is>
+          <t>так</t>
+        </is>
+      </c>
       <c r="N24" s="2" t="n"/>
     </row>
     <row r="25">
@@ -5914,17 +6506,61 @@
           <t>Горбонос О. (КТ)</t>
         </is>
       </c>
-      <c r="C25" s="2" t="n"/>
-      <c r="D25" s="2" t="n"/>
-      <c r="E25" s="2" t="n"/>
-      <c r="F25" s="2" t="n"/>
-      <c r="G25" s="2" t="n"/>
-      <c r="H25" s="2" t="n"/>
-      <c r="I25" s="2" t="n"/>
-      <c r="J25" s="2" t="n"/>
-      <c r="K25" s="2" t="n"/>
-      <c r="L25" s="2" t="n"/>
-      <c r="M25" s="2" t="n"/>
+      <c r="C25" s="2" t="inlineStr">
+        <is>
+          <t>28.10.2026</t>
+        </is>
+      </c>
+      <c r="D25" s="2" t="inlineStr">
+        <is>
+          <t>так</t>
+        </is>
+      </c>
+      <c r="E25" s="2" t="inlineStr">
+        <is>
+          <t>так</t>
+        </is>
+      </c>
+      <c r="F25" s="2" t="inlineStr">
+        <is>
+          <t>так</t>
+        </is>
+      </c>
+      <c r="G25" s="2" t="inlineStr">
+        <is>
+          <t>так</t>
+        </is>
+      </c>
+      <c r="H25" s="2" t="inlineStr">
+        <is>
+          <t>так</t>
+        </is>
+      </c>
+      <c r="I25" s="2" t="inlineStr">
+        <is>
+          <t>так</t>
+        </is>
+      </c>
+      <c r="J25" s="2" t="inlineStr">
+        <is>
+          <t>так</t>
+        </is>
+      </c>
+      <c r="K25" s="2" t="inlineStr">
+        <is>
+          <t>так</t>
+        </is>
+      </c>
+      <c r="L25" s="2" t="inlineStr">
+        <is>
+          <t>Зауважень за чек-листом немає. Перевірено на demo 28.10.2026: склад сторінки «Combination Pliers» (категорія, бренд, ціна, шкала CO2, опис, таблиця характеристик, «Related products»), поле «Quantity» = 1 з кнопками «−» і «+», кнопки «Add to cart», «Add to favourites», «Compare»; повідомлення «Product added to shopping cart.» з'явилося за ≈1,4 с; на піктограмі кошика 1; у кошику один рядок з кількістю 1. Рекомендація, що не блокує: «клас CO2 (одна з літер A–E)» на сторінці подано як шкалу A–E з виділеним класом — уточнити формулювання.</t>
+        </is>
+      </c>
+      <c r="M25" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
       <c r="N25" s="2" t="n"/>
     </row>
     <row r="26">
@@ -6064,8 +6700,448 @@
       <c r="M27" s="2" t="n"/>
       <c r="N27" s="2" t="n"/>
     </row>
+    <row r="28">
+      <c r="A28" s="2" t="inlineStr">
+        <is>
+          <t>TC-027</t>
+        </is>
+      </c>
+      <c r="B28" s="2" t="inlineStr">
+        <is>
+          <t>Дрєпіна А. (СМ)</t>
+        </is>
+      </c>
+      <c r="C28" s="2" t="inlineStr">
+        <is>
+          <t>28.10.2026</t>
+        </is>
+      </c>
+      <c r="D28" s="2" t="inlineStr">
+        <is>
+          <t>так</t>
+        </is>
+      </c>
+      <c r="E28" s="2" t="inlineStr">
+        <is>
+          <t>так</t>
+        </is>
+      </c>
+      <c r="F28" s="2" t="inlineStr">
+        <is>
+          <t>так</t>
+        </is>
+      </c>
+      <c r="G28" s="2" t="inlineStr">
+        <is>
+          <t>так</t>
+        </is>
+      </c>
+      <c r="H28" s="2" t="inlineStr">
+        <is>
+          <t>так</t>
+        </is>
+      </c>
+      <c r="I28" s="6" t="inlineStr">
+        <is>
+          <t>ні</t>
+        </is>
+      </c>
+      <c r="J28" s="2" t="inlineStr">
+        <is>
+          <t>так</t>
+        </is>
+      </c>
+      <c r="K28" s="2" t="inlineStr">
+        <is>
+          <t>так</t>
+        </is>
+      </c>
+      <c r="L28" s="2" t="inlineStr">
+        <is>
+          <t>П6: у кроці 3 поведінку demo («поле одразу замінює 0 на 1 без повідомлення») подано як допустиму. За GUI-50 помилка валідації виводиться текстом під полем, а в TC-003 (100) Ксенія очікує саме повідомлення під полем — для меж 0 і 100 критерій має бути однаковий. Записати: «значення не 0; під полем — текстове повідомлення про помилку (GUI-30, GUI-50)»; якщо demo мовчки замінює 0 на 1 — це failed і звіт про дефект, а не запис у журналі.</t>
+        </is>
+      </c>
+      <c r="M28" s="2" t="n"/>
+      <c r="N28" s="2" t="n"/>
+    </row>
     <row r="29">
-      <c r="A29" t="inlineStr">
+      <c r="A29" s="2" t="inlineStr">
+        <is>
+          <t>TC-028</t>
+        </is>
+      </c>
+      <c r="B29" s="2" t="inlineStr">
+        <is>
+          <t>Дрєпіна А. (СМ)</t>
+        </is>
+      </c>
+      <c r="C29" s="2" t="inlineStr">
+        <is>
+          <t>28.10.2026</t>
+        </is>
+      </c>
+      <c r="D29" s="2" t="inlineStr">
+        <is>
+          <t>так</t>
+        </is>
+      </c>
+      <c r="E29" s="2" t="inlineStr">
+        <is>
+          <t>так</t>
+        </is>
+      </c>
+      <c r="F29" s="2" t="inlineStr">
+        <is>
+          <t>так</t>
+        </is>
+      </c>
+      <c r="G29" s="2" t="inlineStr">
+        <is>
+          <t>так</t>
+        </is>
+      </c>
+      <c r="H29" s="2" t="inlineStr">
+        <is>
+          <t>так</t>
+        </is>
+      </c>
+      <c r="I29" s="2" t="inlineStr">
+        <is>
+          <t>так</t>
+        </is>
+      </c>
+      <c r="J29" s="2" t="inlineStr">
+        <is>
+          <t>так</t>
+        </is>
+      </c>
+      <c r="K29" s="2" t="inlineStr">
+        <is>
+          <t>так</t>
+        </is>
+      </c>
+      <c r="L29" s="2" t="inlineStr">
+        <is>
+          <t>Зауважень немає. Межа a = 1 (GUI-30), пара — TC-027.</t>
+        </is>
+      </c>
+      <c r="M29" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="N29" s="2" t="inlineStr">
+        <is>
+          <t>28.10.2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="2" t="inlineStr">
+        <is>
+          <t>TC-029</t>
+        </is>
+      </c>
+      <c r="B30" s="2" t="inlineStr">
+        <is>
+          <t>Дрєпіна А. (СМ)</t>
+        </is>
+      </c>
+      <c r="C30" s="2" t="inlineStr">
+        <is>
+          <t>28.10.2026</t>
+        </is>
+      </c>
+      <c r="D30" s="2" t="inlineStr">
+        <is>
+          <t>так</t>
+        </is>
+      </c>
+      <c r="E30" s="2" t="inlineStr">
+        <is>
+          <t>так</t>
+        </is>
+      </c>
+      <c r="F30" s="2" t="inlineStr">
+        <is>
+          <t>так</t>
+        </is>
+      </c>
+      <c r="G30" s="2" t="inlineStr">
+        <is>
+          <t>так</t>
+        </is>
+      </c>
+      <c r="H30" s="2" t="inlineStr">
+        <is>
+          <t>так</t>
+        </is>
+      </c>
+      <c r="I30" s="2" t="inlineStr">
+        <is>
+          <t>так</t>
+        </is>
+      </c>
+      <c r="J30" s="2" t="inlineStr">
+        <is>
+          <t>так</t>
+        </is>
+      </c>
+      <c r="K30" s="2" t="inlineStr">
+        <is>
+          <t>так</t>
+        </is>
+      </c>
+      <c r="L30" s="2" t="inlineStr">
+        <is>
+          <t>Зауважень немає. Рекомендація: налаштування DevTools (Disable cache, профіль «10 Mbit») зберігаються між сесіями — у передумовах уточнити, що їх зроблено заздалегідь, до кроку 1.</t>
+        </is>
+      </c>
+      <c r="M30" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="N30" s="2" t="inlineStr">
+        <is>
+          <t>28.10.2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="2" t="inlineStr">
+        <is>
+          <t>TC-030</t>
+        </is>
+      </c>
+      <c r="B31" s="2" t="inlineStr">
+        <is>
+          <t>Дрєпіна А. (СМ)</t>
+        </is>
+      </c>
+      <c r="C31" s="2" t="inlineStr">
+        <is>
+          <t>28.10.2026</t>
+        </is>
+      </c>
+      <c r="D31" s="2" t="inlineStr">
+        <is>
+          <t>так</t>
+        </is>
+      </c>
+      <c r="E31" s="2" t="inlineStr">
+        <is>
+          <t>так</t>
+        </is>
+      </c>
+      <c r="F31" s="2" t="inlineStr">
+        <is>
+          <t>так</t>
+        </is>
+      </c>
+      <c r="G31" s="2" t="inlineStr">
+        <is>
+          <t>так</t>
+        </is>
+      </c>
+      <c r="H31" s="2" t="inlineStr">
+        <is>
+          <t>так</t>
+        </is>
+      </c>
+      <c r="I31" s="2" t="inlineStr">
+        <is>
+          <t>так</t>
+        </is>
+      </c>
+      <c r="J31" s="2" t="inlineStr">
+        <is>
+          <t>так</t>
+        </is>
+      </c>
+      <c r="K31" s="2" t="inlineStr">
+        <is>
+          <t>так</t>
+        </is>
+      </c>
+      <c r="L31" s="2" t="inlineStr">
+        <is>
+          <t>Зауважень немає. Один запуск Lighthouse — не масові запити (п. 1.7), ок.</t>
+        </is>
+      </c>
+      <c r="M31" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="N31" s="2" t="inlineStr">
+        <is>
+          <t>28.10.2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="2" t="inlineStr">
+        <is>
+          <t>TC-031</t>
+        </is>
+      </c>
+      <c r="B32" s="2" t="inlineStr">
+        <is>
+          <t>Дрєпіна А. (СМ)</t>
+        </is>
+      </c>
+      <c r="C32" s="2" t="inlineStr">
+        <is>
+          <t>28.10.2026</t>
+        </is>
+      </c>
+      <c r="D32" s="2" t="inlineStr">
+        <is>
+          <t>так</t>
+        </is>
+      </c>
+      <c r="E32" s="2" t="inlineStr">
+        <is>
+          <t>так</t>
+        </is>
+      </c>
+      <c r="F32" s="2" t="inlineStr">
+        <is>
+          <t>так</t>
+        </is>
+      </c>
+      <c r="G32" s="2" t="inlineStr">
+        <is>
+          <t>так</t>
+        </is>
+      </c>
+      <c r="H32" s="2" t="inlineStr">
+        <is>
+          <t>так</t>
+        </is>
+      </c>
+      <c r="I32" s="2" t="inlineStr">
+        <is>
+          <t>так</t>
+        </is>
+      </c>
+      <c r="J32" s="2" t="inlineStr">
+        <is>
+          <t>так</t>
+        </is>
+      </c>
+      <c r="K32" s="2" t="inlineStr">
+        <is>
+          <t>так</t>
+        </is>
+      </c>
+      <c r="L32" s="2" t="inlineStr">
+        <is>
+          <t>Зауважень немає. Перегляд розділів без зміни даних спільного запису — відповідає п. 1.7. Кроки після входу звірити на пробному прогоні (як зазначено в передумовах).</t>
+        </is>
+      </c>
+      <c r="M32" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="N32" s="2" t="inlineStr">
+        <is>
+          <t>28.10.2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="2" t="inlineStr">
+        <is>
+          <t>TC-032</t>
+        </is>
+      </c>
+      <c r="B33" s="2" t="inlineStr">
+        <is>
+          <t>Дрєпіна А. (СМ)</t>
+        </is>
+      </c>
+      <c r="C33" s="2" t="inlineStr">
+        <is>
+          <t>28.10.2026</t>
+        </is>
+      </c>
+      <c r="D33" s="2" t="inlineStr">
+        <is>
+          <t>так</t>
+        </is>
+      </c>
+      <c r="E33" s="2" t="inlineStr">
+        <is>
+          <t>так</t>
+        </is>
+      </c>
+      <c r="F33" s="2" t="inlineStr">
+        <is>
+          <t>так</t>
+        </is>
+      </c>
+      <c r="G33" s="2" t="inlineStr">
+        <is>
+          <t>так</t>
+        </is>
+      </c>
+      <c r="H33" s="2" t="inlineStr">
+        <is>
+          <t>так</t>
+        </is>
+      </c>
+      <c r="I33" s="6" t="inlineStr">
+        <is>
+          <t>ні</t>
+        </is>
+      </c>
+      <c r="J33" s="2" t="inlineStr">
+        <is>
+          <t>так</t>
+        </is>
+      </c>
+      <c r="K33" s="2" t="inlineStr">
+        <is>
+          <t>так</t>
+        </is>
+      </c>
+      <c r="L33" s="2" t="inlineStr">
+        <is>
+          <t>П6: «кроки «Billing Address» (3) і «Payment» (4) недоступні» після кроку 8 не перевіряється — у кейсі немає дії, що пробує туди перейти. А вкладку «Continue as Guest», яка веде до кроку 3 без входу, подано як «спостереження в журнал». За S-20 це розбіжність, тобто failed і звіт про дефект (як і в TC-027: поведінку demo не записуємо як допустиму). Додати крок-спробу (напр., вкладка «Continue as Guest» → заповнити вигаданими даними → «Continue»), очікування — крок 3 не відкривається (S-20). Кроки 2–3 (/account, /account/favorites → /auth/login) перевірювані, ок.</t>
+        </is>
+      </c>
+      <c r="M33" s="2" t="n"/>
+      <c r="N33" s="2" t="n"/>
+    </row>
+    <row r="34">
+      <c r="A34" s="2" t="inlineStr">
+        <is>
+          <t>TC-033</t>
+        </is>
+      </c>
+      <c r="B34" s="2" t="inlineStr">
+        <is>
+          <t>Горбонос О. (КТ)</t>
+        </is>
+      </c>
+      <c r="C34" s="2" t="n"/>
+      <c r="D34" s="2" t="n"/>
+      <c r="E34" s="2" t="n"/>
+      <c r="F34" s="2" t="n"/>
+      <c r="G34" s="2" t="n"/>
+      <c r="H34" s="2" t="n"/>
+      <c r="I34" s="2" t="n"/>
+      <c r="J34" s="2" t="n"/>
+      <c r="K34" s="2" t="n"/>
+      <c r="L34" s="2" t="n"/>
+      <c r="M34" s="2" t="n"/>
+      <c r="N34" s="2" t="n"/>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
         <is>
           <t>П1 шість полів, унікальний TC-NNN · П2 вимога з SRS 1.1, кейс перевіряє саме її · П3 незалежний (відкриття → вихід/закриття) · П4 передумови повні · П5 одна дія на крок, конкретні дані · П6 перевірювані очікувані результати · П7 заголовок і тип · П8 граничні значення / негативна пара</t>
         </is>
@@ -6073,10 +7149,10 @@
     </row>
   </sheetData>
   <dataValidations count="2">
-    <dataValidation sqref="D2:K27" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="D2:K34" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"так,ні"</formula1>
     </dataValidation>
-    <dataValidation sqref="M2:M27" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="M2:M34" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"так,ні,—"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
SCRUM-110: TC-034 (U-30, ширина 375 px) і TC-035 (U-20, мітки, зірочки, Tab/Enter), draft; Coverage — F-60 +TC-033, GUI-30 TC-027/028, F-130 TC-031 з приміткою, S-20 TC-032 частково, U-30 TC-034, U-20 TC-035; звірено з demo 28.10.2026
</commit_message>
<xml_diff>
--- a/docs/sprint3/test-cases.xlsx
+++ b/docs/sprint3/test-cases.xlsx
@@ -3228,35 +3228,165 @@
       <c r="N34" s="2" t="n"/>
     </row>
     <row r="35">
-      <c r="A35" s="2" t="n"/>
-      <c r="B35" s="2" t="n"/>
-      <c r="C35" s="2" t="n"/>
-      <c r="D35" s="2" t="n"/>
-      <c r="E35" s="2" t="n"/>
-      <c r="F35" s="2" t="n"/>
-      <c r="G35" s="2" t="n"/>
-      <c r="H35" s="2" t="n"/>
-      <c r="I35" s="2" t="n"/>
-      <c r="J35" s="2" t="n"/>
+      <c r="A35" s="2" t="inlineStr">
+        <is>
+          <t>TC-034</t>
+        </is>
+      </c>
+      <c r="B35" s="2" t="inlineStr">
+        <is>
+          <t>U-30</t>
+        </is>
+      </c>
+      <c r="C35" s="2" t="inlineStr">
+        <is>
+          <t>Головна сторінка за ширини вікна 375 px: без горизонтального прокручування, меню доступне, кнопки не менше 44×44 px</t>
+        </is>
+      </c>
+      <c r="D35" s="2" t="inlineStr">
+        <is>
+          <t>Chrome 120 або новіший; demo доступне (збірка v2.5 від 2026-10-11 за написом у підвалі сторінки; стан звірено 28.10.2026); нова сесія (вікно інкогніто), без входу. Інструменти розробника Chrome (DevTools) відкриваються клавішею F12; режим пристрою вмикається клавішами Ctrl+Shift+M.</t>
+        </is>
+      </c>
+      <c r="E35" s="2" t="inlineStr">
+        <is>
+          <t>1. Відкрити https://practicesoftwaretesting.com у Chrome (нова сесія).
+2. Натиснути F12.
+3. Натиснути Ctrl+Shift+M.
+4. На панелі режиму пристрою у списку пристроїв вибрати «Responsive».
+5. У полі ширини на панелі режиму пристрою ввести 375.
+6. Натиснути Enter.
+7. Натиснути F5 (перезавантажити сторінку).
+8. У DevTools відкрити вкладку «Console».
+9. У консолі ввести: document.documentElement.scrollWidth + ' / ' + document.documentElement.clientWidth
+10. Натиснути Enter.
+11. На сторінці натиснути кнопку меню (☰) у шапці.
+12. У консолі ввести: (b =&gt; Math.round(b.width) + '×' + Math.round(b.height))(document.querySelector('[aria-label="Toggle navigation"]').getBoundingClientRect())
+13. Натиснути Enter.
+14. У консолі ввести: (b =&gt; Math.round(b.width) + '×' + Math.round(b.height))(document.querySelector('[data-test=search-submit]').getBoundingClientRect())
+15. Натиснути Enter.
+16. Закрити вкладку.</t>
+        </is>
+      </c>
+      <c r="F35" s="2" t="inlineStr">
+        <is>
+          <t>Після кроку 1: головна сторінка з каталогом.
+Після кроку 2: відкрито DevTools.
+Після кроку 3: увімкнено режим пристрою; над сторінкою — панель з розмірами вікна.
+Після кроку 4: вибрано «Responsive»; поля ширини і висоти доступні для введення.
+Після кроку 5: у полі ширини — 375.
+Після кроку 6: ширина області сторінки — 375 px.
+Після кроку 7: сторінку перезавантажено за ширини 375 px; замість пунктів меню в шапці — кнопка меню (☰).
+Після кроку 8: вкладка «Console».
+Після кроку 9: вираз введено.
+Після кроку 10: консоль показує два числа «A / B»; A не більше за B — горизонтального прокручування немає (U-30).
+Після кроку 11: розгорнуто меню навігації з пунктами «Home», «Categories», «Contact», «Sign in» (U-30, GUI-10).
+Після кроку 12: вираз введено.
+Після кроку 13: консоль показує розмір кнопки меню «ширина×висота»; обидва числа не менші за 44 (U-30).
+Після кроку 14: вираз введено.
+Після кроку 15: консоль показує розмір кнопки «Search»; обидва числа не менші за 44 (U-30).
+Після кроку 16: вкладку закрито.</t>
+        </is>
+      </c>
+      <c r="G35" s="2" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="H35" s="2" t="inlineStr">
+        <is>
+          <t>позитивний</t>
+        </is>
+      </c>
+      <c r="I35" s="2" t="inlineStr">
+        <is>
+          <t>Межі з U-30: ширина вікна 375 px (найменша підтримувана, SRS 1.1, розд. 2.2), кнопки не менше 44×44 px. Відсутність горизонтального прокручування — scrollWidth не більше clientWidth. Кнопки обрано як основні елементи керування головної сторінки на мобільній ширині: меню (☰) і «Search». Розмір — фактичний на екрані (getBoundingClientRect).</t>
+        </is>
+      </c>
+      <c r="J35" s="2" t="inlineStr">
+        <is>
+          <t>Коротка К. (ТА)</t>
+        </is>
+      </c>
       <c r="K35" s="2" t="n"/>
       <c r="L35" s="2" t="n"/>
-      <c r="M35" s="2" t="n"/>
+      <c r="M35" s="2" t="inlineStr">
+        <is>
+          <t>draft</t>
+        </is>
+      </c>
       <c r="N35" s="2" t="n"/>
     </row>
     <row r="36">
-      <c r="A36" s="2" t="n"/>
-      <c r="B36" s="2" t="n"/>
-      <c r="C36" s="2" t="n"/>
-      <c r="D36" s="2" t="n"/>
-      <c r="E36" s="2" t="n"/>
-      <c r="F36" s="2" t="n"/>
-      <c r="G36" s="2" t="n"/>
-      <c r="H36" s="2" t="n"/>
-      <c r="I36" s="2" t="n"/>
-      <c r="J36" s="2" t="n"/>
+      <c r="A36" s="2" t="inlineStr">
+        <is>
+          <t>TC-035</t>
+        </is>
+      </c>
+      <c r="B36" s="2" t="inlineStr">
+        <is>
+          <t>U-20</t>
+        </is>
+      </c>
+      <c r="C36" s="2" t="inlineStr">
+        <is>
+          <t>Форма входу: мітки полів, зірочки обов'язкових полів, повідомлення про помилку текстом; керування клавішами Tab і Enter</t>
+        </is>
+      </c>
+      <c r="D36" s="2" t="inlineStr">
+        <is>
+          <t>Chrome 120 або новіший, вікно 1280×800; demo доступне (збірка v2.5 від 2026-10-11 за написом у підвалі сторінки; стан звірено 28.10.2026); нова сесія (вікно інкогніто), без входу. Поля форми входу порожні.</t>
+        </is>
+      </c>
+      <c r="E36" s="2" t="inlineStr">
+        <is>
+          <t>1. Відкрити https://practicesoftwaretesting.com/auth/login у Chrome (нова сесія).
+2. Натиснути на поле «Email address».
+3. Натиснути клавішу Tab.
+4. Натиснути клавішу Tab.
+5. Натиснути клавішу Tab.
+6. Натиснути клавішу Enter.
+7. Закрити вкладку.</t>
+        </is>
+      </c>
+      <c r="F36" s="2" t="inlineStr">
+        <is>
+          <t>Після кроку 1: сторінка входу; над полями — текстові мітки «Email address *» і «Password *»; обов'язкові поля позначено зірочкою (U-20).
+Після кроку 2: курсор у полі «Email address»; поле виділено рамкою фокуса.
+Після кроку 3: фокус перейшов на поле «Password» (U-20).
+Після кроку 4: фокус на кнопці «показати / приховати пароль» (U-20).
+Після кроку 5: фокус на кнопці «Login» (U-20).
+Після кроку 6: форму не надіслано; під полями «Email address» і «Password» — текстові повідомлення про помилку, а не лише зміна кольору (U-20, GUI-50); адреса сторінки не змінилася (/auth/login).
+Після кроку 7: вкладку закрито.</t>
+        </is>
+      </c>
+      <c r="G36" s="2" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="H36" s="2" t="inlineStr">
+        <is>
+          <t>негативний</t>
+        </is>
+      </c>
+      <c r="I36" s="2" t="inlineStr">
+        <is>
+          <t>Клас «обов'язкові поля порожні» — негативна перевірка: відправлення з клавіатури має дати текстові повідомлення під полями. Порядок фокуса — порядок елементів форми входу на demo (поле Email, поле Password, кнопка показу пароля, «Login»; звірено 28.10.2026). Форма входу — найкоротша форма з двома обов'язковими полями; дані не вводяться, обліковий запис не потрібен.</t>
+        </is>
+      </c>
+      <c r="J36" s="2" t="inlineStr">
+        <is>
+          <t>Коротка К. (ТА)</t>
+        </is>
+      </c>
       <c r="K36" s="2" t="n"/>
       <c r="L36" s="2" t="n"/>
-      <c r="M36" s="2" t="n"/>
+      <c r="M36" s="2" t="inlineStr">
+        <is>
+          <t>draft</t>
+        </is>
+      </c>
       <c r="N36" s="2" t="n"/>
     </row>
     <row r="37">
@@ -3644,7 +3774,7 @@
       </c>
       <c r="E7" s="2" t="inlineStr">
         <is>
-          <t>TC-001, TC-022</t>
+          <t>TC-001, TC-022, TC-033</t>
         </is>
       </c>
       <c r="F7" s="2" t="inlineStr"/>
@@ -3852,12 +3982,12 @@
       </c>
       <c r="E14" s="2" t="inlineStr">
         <is>
-          <t>TC-031 (КТ, у роботі)</t>
+          <t>TC-031</t>
         </is>
       </c>
       <c r="F14" s="2" t="inlineStr">
         <is>
-          <t>Етика demo (методичка, п. 5.4): пароль спільного тестового облікового запису не змінювати — зміну пароля перевіряти лише на власному зареєстрованому обліковому записі.</t>
+          <t>Кейс TC-031 перевіряє лише перегляд розділів кабінету («My profile», «My favorites», «My invoices», «My messages»). Зміну пароля й редагування профілю на спільному обліковому записі не виконуємо (етика demo, п. 1.7); деталі замовлення і завантаження PDF у кейс не входять.</t>
         </is>
       </c>
     </row>
@@ -3972,7 +4102,7 @@
       </c>
       <c r="E18" s="2" t="inlineStr">
         <is>
-          <t>TC-002, TC-003; TC-027, TC-028 (КТ, draft)</t>
+          <t>TC-002, TC-003, TC-027, TC-028</t>
         </is>
       </c>
       <c r="F18" s="2" t="inlineStr">
@@ -4576,12 +4706,12 @@
       </c>
       <c r="E38" s="2" t="inlineStr">
         <is>
-          <t>TC-025+ (КТ)</t>
+          <t>TC-032; покрито частково</t>
         </is>
       </c>
       <c r="F38" s="2" t="inlineStr">
         <is>
-          <t>Перевіряється спостереженням.</t>
+          <t>Маскування пароля перевіряють TC-004, TC-005–008, TC-015, TC-026; TC-032 — недоступність кабінету і кроків 3–4 оформлення без входу. Перенаправлення на сторінку входу після «Sign out» окремим кейсом не перевіряється.</t>
         </is>
       </c>
     </row>
@@ -4636,7 +4766,7 @@
       </c>
       <c r="E40" s="2" t="inlineStr">
         <is>
-          <t>TC-025+ (ТА)</t>
+          <t>TC-035</t>
         </is>
       </c>
       <c r="F40" s="2" t="inlineStr">
@@ -4668,7 +4798,7 @@
       </c>
       <c r="E41" s="2" t="inlineStr">
         <is>
-          <t>TC-025+ (ТА)</t>
+          <t>TC-034</t>
         </is>
       </c>
       <c r="F41" s="2" t="inlineStr">

</xml_diff>

<commit_message>
SCRUM-119, SCRUM-118: TC-036 (S-10, HTTP → HTTPS),
draft; Review фаза 1 TC-034, TC-035
</commit_message>
<xml_diff>
--- a/docs/sprint3/test-cases.xlsx
+++ b/docs/sprint3/test-cases.xlsx
@@ -3308,11 +3308,19 @@
           <t>Коротка К. (ТА)</t>
         </is>
       </c>
-      <c r="K35" s="2" t="n"/>
-      <c r="L35" s="2" t="n"/>
+      <c r="K35" s="2" t="inlineStr">
+        <is>
+          <t>Дрєпіна А. (СМ)</t>
+        </is>
+      </c>
+      <c r="L35" s="2" t="inlineStr">
+        <is>
+          <t>28.10.2026</t>
+        </is>
+      </c>
       <c r="M35" s="2" t="inlineStr">
         <is>
-          <t>draft</t>
+          <t>reviewed</t>
         </is>
       </c>
       <c r="N35" s="2" t="n"/>
@@ -3380,29 +3388,97 @@
           <t>Коротка К. (ТА)</t>
         </is>
       </c>
-      <c r="K36" s="2" t="n"/>
-      <c r="L36" s="2" t="n"/>
+      <c r="K36" s="2" t="inlineStr">
+        <is>
+          <t>Дрєпіна А. (СМ)</t>
+        </is>
+      </c>
+      <c r="L36" s="2" t="inlineStr">
+        <is>
+          <t>28.10.2026</t>
+        </is>
+      </c>
       <c r="M36" s="2" t="inlineStr">
         <is>
-          <t>draft</t>
+          <t>reviewed</t>
         </is>
       </c>
       <c r="N36" s="2" t="n"/>
     </row>
     <row r="37">
-      <c r="A37" s="2" t="n"/>
-      <c r="B37" s="2" t="n"/>
-      <c r="C37" s="2" t="n"/>
-      <c r="D37" s="2" t="n"/>
-      <c r="E37" s="2" t="n"/>
-      <c r="F37" s="2" t="n"/>
-      <c r="G37" s="2" t="n"/>
-      <c r="H37" s="2" t="n"/>
-      <c r="I37" s="2" t="n"/>
-      <c r="J37" s="2" t="n"/>
+      <c r="A37" s="2" t="inlineStr">
+        <is>
+          <t>TC-036</t>
+        </is>
+      </c>
+      <c r="B37" s="2" t="inlineStr">
+        <is>
+          <t>S-10</t>
+        </is>
+      </c>
+      <c r="C37" s="2" t="inlineStr">
+        <is>
+          <t>Відкриття demo за адресою http://: сервер перенаправляє на https://, з'єднання TLS 1.3</t>
+        </is>
+      </c>
+      <c r="D37" s="2" t="inlineStr">
+        <is>
+          <t>Chrome 120 або новіший, вікно 1280×800; demo доступне (збірка v2.5 від 2026-10-11 за написом у підвалі сторінки); нова сесія (вікно інкогніто), без входу. У налаштуваннях Chrome (chrome://settings/security) вимкнено «Always use secure connections», щоб перехід на HTTPS не виконав сам браузер. Обліковий запис не потрібен, дані не вводяться. Назви вкладок DevTools і текст на вкладці «Security» звірити на пробному прогоні.</t>
+        </is>
+      </c>
+      <c r="E37" s="2" t="inlineStr">
+        <is>
+          <t>1. Відкрити http://practicesoftwaretesting.com у Chrome (нова сесія).
+2. Натиснути F12.
+3. У DevTools відкрити вкладку «Network».
+4. Позначити прапорець «Preserve log».
+5. В адресний рядок ввести: http://practicesoftwaretesting.com
+6. Натиснути Enter.
+7. У списку «Network» натиснути перший рядок (запит до practicesoftwaretesting.com).
+8. У DevTools відкрити вкладку «Security».
+9. Закрити вкладку.</t>
+        </is>
+      </c>
+      <c r="F37" s="2" t="inlineStr">
+        <is>
+          <t>Після кроку 1: відкрито головну сторінку з каталогом; адреса в адресному рядку починається з https:// (S-10).
+Після кроку 2: відкрито DevTools.
+Після кроку 3: вкладка «Network».
+Після кроку 4: прапорець «Preserve log» позначено.
+Після кроку 5: в адресному рядку — http://practicesoftwaretesting.com.
+Після кроку 6: відкрито головну сторінку з каталогом; адреса знову починається з https:// (S-10).
+Після кроку 7: у деталях запиту на вкладці «Headers»: Request URL — http://practicesoftwaretesting.com/; Status Code — 301, 302, 307 або 308; заголовок відповіді Location починається з https://practicesoftwaretesting.com (перенаправлення виконав сервер, S-10). Якщо статус «307 Internal Redirect» — перехід зробив браузер, а не сервер: кейс blocked, повідомити КТ.
+Після кроку 8: на вкладці «Security» — з'єднання захищене, у розділі «Connection» вказано протокол TLS 1.3 (S-10).
+Після кроку 9: вкладку закрито.</t>
+        </is>
+      </c>
+      <c r="G37" s="2" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="H37" s="2" t="inlineStr">
+        <is>
+          <t>позитивний</t>
+        </is>
+      </c>
+      <c r="I37" s="2" t="inlineStr">
+        <is>
+          <t>S-10 покривається частково — лише те, що можна спостерегти на публічному demo: перенаправлення HTTP → HTTPS і версія TLS сторінки. Хеш bcrypt, код 403 на чужі дані і сканування вразливостей на demo не перевіряються (інструкція, п. 1.7; S-10 — сканування лише на локальному стенді). API не перевіряється в цьому кейсі (один кейс — один набір даних). Один запит до головної сторінки — не навантаження. Стовпець «Status Code» і заголовок Location відрізняють перенаправлення сервера від автоматичного переходу браузера на HTTPS. Номер TC-036 — наступний вільний після TC-035 [ЗАПОВНИТИ: підтвердити з ТА].</t>
+        </is>
+      </c>
+      <c r="J37" s="2" t="inlineStr">
+        <is>
+          <t>Дрєпіна А. (СМ)</t>
+        </is>
+      </c>
       <c r="K37" s="2" t="n"/>
       <c r="L37" s="2" t="n"/>
-      <c r="M37" s="2" t="n"/>
+      <c r="M37" s="2" t="inlineStr">
+        <is>
+          <t>draft</t>
+        </is>
+      </c>
       <c r="N37" s="2" t="n"/>
     </row>
     <row r="38">
@@ -4880,7 +4956,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N36"/>
+  <dimension ref="A1:N39"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -7270,8 +7346,176 @@
       <c r="M34" s="2" t="n"/>
       <c r="N34" s="2" t="n"/>
     </row>
+    <row r="35">
+      <c r="A35" s="2" t="inlineStr">
+        <is>
+          <t>TC-034</t>
+        </is>
+      </c>
+      <c r="B35" s="2" t="inlineStr">
+        <is>
+          <t>Дрєпіна А. (СМ)</t>
+        </is>
+      </c>
+      <c r="C35" s="2" t="inlineStr">
+        <is>
+          <t>28.10.2026</t>
+        </is>
+      </c>
+      <c r="D35" s="2" t="inlineStr">
+        <is>
+          <t>так</t>
+        </is>
+      </c>
+      <c r="E35" s="2" t="inlineStr">
+        <is>
+          <t>так</t>
+        </is>
+      </c>
+      <c r="F35" s="2" t="inlineStr">
+        <is>
+          <t>так</t>
+        </is>
+      </c>
+      <c r="G35" s="2" t="inlineStr">
+        <is>
+          <t>так</t>
+        </is>
+      </c>
+      <c r="H35" s="2" t="inlineStr">
+        <is>
+          <t>так</t>
+        </is>
+      </c>
+      <c r="I35" s="2" t="inlineStr">
+        <is>
+          <t>так</t>
+        </is>
+      </c>
+      <c r="J35" s="2" t="inlineStr">
+        <is>
+          <t>так</t>
+        </is>
+      </c>
+      <c r="K35" s="2" t="inlineStr">
+        <is>
+          <t>так</t>
+        </is>
+      </c>
+      <c r="L35" s="2" t="inlineStr">
+        <is>
+          <t>Зауважень немає. Ширина 375 px, scrollWidth ≤ clientWidth і 44×44 px — з U-30. Рекомендація: U-30 вимагає придатних для пальця «кнопок» загалом, а міряються дві (☰ і «Search») — у README зазначити, що покриття вибіркове.</t>
+        </is>
+      </c>
+      <c r="M35" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="N35" s="2" t="inlineStr">
+        <is>
+          <t>28.10.2026</t>
+        </is>
+      </c>
+    </row>
     <row r="36">
-      <c r="A36" t="inlineStr">
+      <c r="A36" s="2" t="inlineStr">
+        <is>
+          <t>TC-035</t>
+        </is>
+      </c>
+      <c r="B36" s="2" t="inlineStr">
+        <is>
+          <t>Дрєпіна А. (СМ)</t>
+        </is>
+      </c>
+      <c r="C36" s="2" t="inlineStr">
+        <is>
+          <t>28.10.2026</t>
+        </is>
+      </c>
+      <c r="D36" s="2" t="inlineStr">
+        <is>
+          <t>так</t>
+        </is>
+      </c>
+      <c r="E36" s="2" t="inlineStr">
+        <is>
+          <t>так</t>
+        </is>
+      </c>
+      <c r="F36" s="2" t="inlineStr">
+        <is>
+          <t>так</t>
+        </is>
+      </c>
+      <c r="G36" s="2" t="inlineStr">
+        <is>
+          <t>так</t>
+        </is>
+      </c>
+      <c r="H36" s="2" t="inlineStr">
+        <is>
+          <t>так</t>
+        </is>
+      </c>
+      <c r="I36" s="2" t="inlineStr">
+        <is>
+          <t>так</t>
+        </is>
+      </c>
+      <c r="J36" s="2" t="inlineStr">
+        <is>
+          <t>так</t>
+        </is>
+      </c>
+      <c r="K36" s="2" t="inlineStr">
+        <is>
+          <t>так</t>
+        </is>
+      </c>
+      <c r="L36" s="2" t="inlineStr">
+        <is>
+          <t>Зауважень немає. Мітки, зірочки, помилка текстом під полем, Tab/Enter — усі чотири умови U-20 мають перевірюваний результат; порядок фокуса звірено з demo 28.10.2026.</t>
+        </is>
+      </c>
+      <c r="M36" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="N36" s="2" t="inlineStr">
+        <is>
+          <t>28.10.2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="2" t="inlineStr">
+        <is>
+          <t>TC-036</t>
+        </is>
+      </c>
+      <c r="B37" s="2" t="inlineStr">
+        <is>
+          <t>Горбонос О. (КТ)</t>
+        </is>
+      </c>
+      <c r="C37" s="2" t="n"/>
+      <c r="D37" s="2" t="n"/>
+      <c r="E37" s="2" t="n"/>
+      <c r="F37" s="2" t="n"/>
+      <c r="G37" s="2" t="n"/>
+      <c r="H37" s="2" t="n"/>
+      <c r="I37" s="2" t="n"/>
+      <c r="J37" s="2" t="n"/>
+      <c r="K37" s="2" t="n"/>
+      <c r="L37" s="2" t="n"/>
+      <c r="M37" s="2" t="n"/>
+      <c r="N37" s="2" t="n"/>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
         <is>
           <t>П1 шість полів, унікальний TC-NNN · П2 вимога з SRS 1.1, кейс перевіряє саме її · П3 незалежний (відкриття → вихід/закриття) · П4 передумови повні · П5 одна дія на крок, конкретні дані · П6 перевірювані очікувані результати · П7 заголовок і тип · П8 граничні значення / негативна пара</t>
         </is>
@@ -7279,10 +7523,10 @@
     </row>
   </sheetData>
   <dataValidations count="2">
-    <dataValidation sqref="D2:K34" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="D2:K37" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"так,ні"</formula1>
     </dataValidation>
-    <dataValidation sqref="M2:M34" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="M2:M37" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"так,ні,—"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
SCRUM-118, SCRUM-119: фаза 2 TC-019,
TC-026 (reviewed); TC-036 — перенаправлення через curl (зауваження ІТ), draft
</commit_message>
<xml_diff>
--- a/docs/sprint3/test-cases.xlsx
+++ b/docs/sprint3/test-cases.xlsx
@@ -2134,11 +2134,19 @@
           <t>Тимчак А. (ІТ)</t>
         </is>
       </c>
-      <c r="K20" s="2" t="n"/>
-      <c r="L20" s="2" t="n"/>
+      <c r="K20" s="2" t="inlineStr">
+        <is>
+          <t>Дрєпіна А. (СМ)</t>
+        </is>
+      </c>
+      <c r="L20" s="2" t="inlineStr">
+        <is>
+          <t>28.10.2026</t>
+        </is>
+      </c>
       <c r="M20" s="2" t="inlineStr">
         <is>
-          <t>draft</t>
+          <t>reviewed</t>
         </is>
       </c>
       <c r="N20" s="2" t="n"/>
@@ -2691,11 +2699,19 @@
           <t>Тимчак А. (ІТ)</t>
         </is>
       </c>
-      <c r="K27" s="2" t="n"/>
-      <c r="L27" s="2" t="n"/>
+      <c r="K27" s="2" t="inlineStr">
+        <is>
+          <t>Дрєпіна А. (СМ)</t>
+        </is>
+      </c>
+      <c r="L27" s="2" t="inlineStr">
+        <is>
+          <t>28.10.2026</t>
+        </is>
+      </c>
       <c r="M27" s="2" t="inlineStr">
         <is>
-          <t>draft</t>
+          <t>reviewed</t>
         </is>
       </c>
       <c r="N27" s="2" t="n"/>
@@ -3503,33 +3519,31 @@
       </c>
       <c r="D37" s="2" t="inlineStr">
         <is>
-          <t>Chrome 120 або новіший, вікно 1280×800; demo доступне (збірка v2.5 від 2026-10-11 за написом у підвалі сторінки); нова сесія (вікно інкогніто), без входу. У налаштуваннях Chrome (chrome://settings/security) вимкнено «Always use secure connections», щоб перехід на HTTPS не виконав сам браузер. Обліковий запис не потрібен, дані не вводяться. Назви вкладок DevTools і текст на вкладці «Security» звірити на пробному прогоні.</t>
+          <t>Chrome 120 або новіший, вікно 1280×800; demo доступне (збірка v2.5 від 2026-10-11 за написом у підвалі сторінки); нова сесія (вікно інкогніто), без входу. На комп'ютері є термінал із командою curl (Windows 10+ — PowerShell або cmd, macOS/Linux — Terminal). Chrome сам переводить http:// на https:// незалежно від налаштування «Always use secure connections» (Chrome 156, звірено ІТ 28.10.2026), тому перенаправлення сервера перевіряється через curl, а не в браузері. Обліковий запис не потрібен, дані не вводяться.</t>
         </is>
       </c>
       <c r="E37" s="2" t="inlineStr">
         <is>
           <t>1. Відкрити http://practicesoftwaretesting.com у Chrome (нова сесія).
 2. Натиснути F12.
-3. У DevTools відкрити вкладку «Network».
-4. Позначити прапорець «Preserve log».
-5. В адресний рядок ввести: http://practicesoftwaretesting.com
-6. Натиснути Enter.
-7. У списку «Network» натиснути перший рядок (запит до practicesoftwaretesting.com).
-8. У DevTools відкрити вкладку «Security».
-9. Закрити вкладку.</t>
+3. У DevTools відкрити вкладку «Security».
+4. Закрити вкладку.
+5. Відкрити термінал.
+6. Ввести команду: curl -sI http://practicesoftwaretesting.com/
+7. Натиснути Enter.
+8. Закрити термінал.</t>
         </is>
       </c>
       <c r="F37" s="2" t="inlineStr">
         <is>
-          <t>Після кроку 1: відкрито головну сторінку з каталогом; адреса в адресному рядку починається з https:// (S-10).
+          <t>Після кроку 1: відкрито головну сторінку з каталогом; адреса в адресному рядку починається з https://.
 Після кроку 2: відкрито DevTools.
-Після кроку 3: вкладка «Network».
-Після кроку 4: прапорець «Preserve log» позначено.
-Після кроку 5: в адресному рядку — http://practicesoftwaretesting.com.
-Після кроку 6: відкрито головну сторінку з каталогом; адреса знову починається з https:// (S-10).
-Після кроку 7: у деталях запиту на вкладці «Headers»: Request URL — http://practicesoftwaretesting.com/; Status Code — 301, 302, 307 або 308; заголовок відповіді Location починається з https://practicesoftwaretesting.com (перенаправлення виконав сервер, S-10). Якщо статус «307 Internal Redirect» — перехід зробив браузер, а не сервер: кейс blocked, повідомити КТ.
-Після кроку 8: на вкладці «Security» — з'єднання захищене, у розділі «Connection» вказано протокол TLS 1.3 (S-10).
-Після кроку 9: вкладку закрито.</t>
+Після кроку 3: на вкладці «Security» — з'єднання захищене, у розділі «Connection» вказано протокол TLS 1.3 (S-10).
+Після кроку 4: вкладку закрито.
+Після кроку 5: відкрито вікно термінала.
+Після кроку 6: команду введено.
+Після кроку 7: перший рядок відповіді — HTTP/1.1 з кодом 301, 302, 307 або 308; є заголовок Location, що починається з https://practicesoftwaretesting.com (сервер перенаправляє HTTP на HTTPS, S-10).
+Після кроку 8: термінал закрито.</t>
         </is>
       </c>
       <c r="G37" s="2" t="inlineStr">
@@ -3544,7 +3558,7 @@
       </c>
       <c r="I37" s="2" t="inlineStr">
         <is>
-          <t>S-10 покривається частково — лише те, що можна спостерегти на публічному demo: перенаправлення HTTP → HTTPS і версія TLS сторінки. Хеш bcrypt, код 403 на чужі дані і сканування вразливостей на demo не перевіряються (інструкція, п. 1.7; S-10 — сканування лише на локальному стенді). API не перевіряється в цьому кейсі (один кейс — один набір даних). Один запит до головної сторінки — не навантаження. Стовпець «Status Code» і заголовок Location відрізняють перенаправлення сервера від автоматичного переходу браузера на HTTPS.</t>
+          <t>S-10 покривається частково — лише те, що можна спостерегти на публічному demo: перенаправлення HTTP → HTTPS і версія TLS. Хеш bcrypt, код 403 на чужі дані і сканування вразливостей на demo не перевіряються (інструкція, п. 1.7; S-10 — сканування лише на локальному стенді). Перенаправлення перевіряється curl, бо браузер сам переходить на https:// і не показує відповідь сервера (зауваження ІТ, 28.10.2026). Один запит curl і одне відкриття сторінки — не навантаження. API не перевіряється (один кейс — один набір даних).</t>
         </is>
       </c>
       <c r="J37" s="2" t="inlineStr">
@@ -3552,19 +3566,11 @@
           <t>Дрєпіна А. (СМ)</t>
         </is>
       </c>
-      <c r="K37" s="2" t="inlineStr">
-        <is>
-          <t>Горбонос О. (КТ)</t>
-        </is>
-      </c>
-      <c r="L37" s="2" t="inlineStr">
-        <is>
-          <t>28.10.2026</t>
-        </is>
-      </c>
+      <c r="K37" s="2" t="n"/>
+      <c r="L37" s="2" t="n"/>
       <c r="M37" s="2" t="inlineStr">
         <is>
-          <t>reviewed</t>
+          <t>draft</t>
         </is>
       </c>
       <c r="N37" s="2" t="n"/>
@@ -6482,9 +6488,9 @@
           <t>так</t>
         </is>
       </c>
-      <c r="H20" s="6" t="inlineStr">
-        <is>
-          <t>ні</t>
+      <c r="H20" s="2" t="inlineStr">
+        <is>
+          <t>так</t>
         </is>
       </c>
       <c r="I20" s="2" t="inlineStr">
@@ -6507,15 +6513,20 @@
           <t>П3, П4: кейс спирається на обліковий запис, «зареєстрований заздалегідь»; дані demo скидаються (SRS 1.1, розд. 2.3), тож кейс залежить від стану з попереднього сеансу. Додати реєстрацію в кроки кейсу або вказати, хто і коли створює запис перед виконанням.
 П8: для форми відновлення пароля немає негативної пари (напр., порожнє поле «Email address» → помилка під полем, GUI-50) — додати як TC-025+.
 Фаза 2 (28.10.2026, коміт 61bd56d): П3, П4 виправлено (реєстрація в кроках, адреса з датою); П8 виправлено (TC-025).
-Нове П5: крок 15 «ввести пароль і натиснути Register» — дві дії; розбити на два кроки.</t>
+Нове П5: крок 15 «ввести пароль і натиснути Register» — дві дії; розбити на два кроки.
+Фаза 2 (28.10.2026, коміт 1c0dcd7): П5 виправлено: крок 15 розбито на «ввести пароль» (15) і «натиснути Register» (16); передумови й очікувані результати перенумеровано.</t>
         </is>
       </c>
       <c r="M20" s="6" t="inlineStr">
         <is>
-          <t>ні</t>
-        </is>
-      </c>
-      <c r="N20" s="2" t="n"/>
+          <t>так</t>
+        </is>
+      </c>
+      <c r="N20" s="2" t="inlineStr">
+        <is>
+          <t>28.10.2026</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
@@ -6985,14 +6996,14 @@
           <t>так</t>
         </is>
       </c>
-      <c r="G27" s="6" t="inlineStr">
-        <is>
-          <t>ні</t>
-        </is>
-      </c>
-      <c r="H27" s="6" t="inlineStr">
-        <is>
-          <t>ні</t>
+      <c r="G27" s="2" t="inlineStr">
+        <is>
+          <t>так</t>
+        </is>
+      </c>
+      <c r="H27" s="2" t="inlineStr">
+        <is>
+          <t>так</t>
         </is>
       </c>
       <c r="I27" s="2" t="inlineStr">
@@ -7013,11 +7024,20 @@
       <c r="L27" s="2" t="inlineStr">
         <is>
           <t>П5: кроки 6, 10, 12 — по дві дії (ім'я користувача в меню + пункт меню); розбити.
-П4: у передумовах «у кроці 13 повертає список до початкового стану», а видалення — крок 11; виправити номер.</t>
-        </is>
-      </c>
-      <c r="M27" s="2" t="n"/>
-      <c r="N27" s="2" t="n"/>
+П4: у передумовах «у кроці 13 повертає список до початкового стану», а видалення — крок 11; виправити номер.
+Фаза 2 (28.10.2026, коміт 1c0dcd7): П5 виправлено: кроки 6, 10, 12 розбито по одній дії. П4: після перенумерації видалення — крок 13, тож «крок 13» у передумовах тепер правильний (пояснення ІТ в описі PR SCRUM-113).</t>
+        </is>
+      </c>
+      <c r="M27" s="2" t="inlineStr">
+        <is>
+          <t>так</t>
+        </is>
+      </c>
+      <c r="N27" s="2" t="inlineStr">
+        <is>
+          <t>28.10.2026</t>
+        </is>
+      </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
@@ -7743,6 +7763,7 @@
         </is>
       </c>
     </row>
+    <row r="38"/>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
SCRUM-114: test-cases.xlsx — «Issue #» для failed-кейсів: TC-003 #54, 005 #55, 010 #57, 011 #57, 012 #53, 027 #52, 029 #56, 032 #50, 034 #63 (TC-013, TC-023 без номера: дефекти поза кроками)
</commit_message>
<xml_diff>
--- a/docs/sprint3/test-cases.xlsx
+++ b/docs/sprint3/test-cases.xlsx
@@ -790,7 +790,11 @@
           <t>reviewed</t>
         </is>
       </c>
-      <c r="N4" s="2" t="n"/>
+      <c r="N4" s="2" t="inlineStr">
+        <is>
+          <t>#54</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
@@ -966,7 +970,11 @@
           <t>reviewed</t>
         </is>
       </c>
-      <c r="N6" s="2" t="n"/>
+      <c r="N6" s="2" t="inlineStr">
+        <is>
+          <t>#55</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
@@ -1400,7 +1408,11 @@
           <t>reviewed</t>
         </is>
       </c>
-      <c r="N11" s="2" t="n"/>
+      <c r="N11" s="2" t="inlineStr">
+        <is>
+          <t>#57</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
@@ -1479,7 +1491,11 @@
           <t>reviewed</t>
         </is>
       </c>
-      <c r="N12" s="2" t="n"/>
+      <c r="N12" s="2" t="inlineStr">
+        <is>
+          <t>#57</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
@@ -1558,7 +1574,11 @@
           <t>reviewed</t>
         </is>
       </c>
-      <c r="N13" s="2" t="n"/>
+      <c r="N13" s="2" t="inlineStr">
+        <is>
+          <t>#53</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
@@ -2808,7 +2828,11 @@
           <t>reviewed</t>
         </is>
       </c>
-      <c r="N28" s="2" t="n"/>
+      <c r="N28" s="2" t="inlineStr">
+        <is>
+          <t>#56</t>
+        </is>
+      </c>
     </row>
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
@@ -2976,7 +3000,11 @@
           <t>reviewed</t>
         </is>
       </c>
-      <c r="N30" s="2" t="n"/>
+      <c r="N30" s="2" t="inlineStr">
+        <is>
+          <t>#52</t>
+        </is>
+      </c>
     </row>
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
@@ -3245,7 +3273,11 @@
           <t>reviewed</t>
         </is>
       </c>
-      <c r="N33" s="2" t="n"/>
+      <c r="N33" s="2" t="inlineStr">
+        <is>
+          <t>#50</t>
+        </is>
+      </c>
     </row>
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
@@ -3419,7 +3451,11 @@
           <t>reviewed</t>
         </is>
       </c>
-      <c r="N35" s="2" t="n"/>
+      <c r="N35" s="2" t="inlineStr">
+        <is>
+          <t>#63</t>
+        </is>
+      </c>
     </row>
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
@@ -3590,27 +3626,27 @@
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">TC-037</t>
+          <t>TC-037</t>
         </is>
       </c>
       <c r="B38" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">F-140</t>
+          <t>F-140</t>
         </is>
       </c>
       <c r="C38" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Контактна форма: допустиме вкладення .txt (1 КБ) приймається, звернення надсилається</t>
+          <t>Контактна форма: допустиме вкладення .txt (1 КБ) приймається, звернення надсилається</t>
         </is>
       </c>
       <c r="D38" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Chrome 120 або новіший, вікно 1280×800; demo доступне (збірка v2.5 від 2026-10-11 за написом у підвалі сторінки; стан звірено 28.10.2026); обліковий запис не потрібен (звернення від анонімного відвідувача); дані лише вигадані. На комп'ютері є текстовий файл note.txt розміром 1 КБ (близько 1000 символів) з вигаданим текстом без особистих даних.</t>
+          <t>Chrome 120 або новіший, вікно 1280×800; demo доступне (збірка v2.5 від 2026-10-11 за написом у підвалі сторінки; стан звірено 28.10.2026); обліковий запис не потрібен (звернення від анонімного відвідувача); дані лише вигадані. На комп'ютері є текстовий файл note.txt розміром 1 КБ (близько 1000 символів) з вигаданим текстом без особистих даних.</t>
         </is>
       </c>
       <c r="E38" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">1. Відкрити https://practicesoftwaretesting.com/contact у Chrome (нова сесія).
+          <t>1. Відкрити https://practicesoftwaretesting.com/contact у Chrome (нова сесія).
 2. У поле «Your first name» ввести: Test
 3. У поле «Your last name» ввести: Tester
 4. У поле «Your email» ввести: tester.tc037@example.com
@@ -3624,7 +3660,7 @@
       </c>
       <c r="F38" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Після кроку 1: відкрито сторінку «Contact», усі поля порожні.
+          <t>Після кроку 1: відкрито сторінку «Contact», усі поля порожні.
 Після кроків 2–5: у полях відображено введені значення: Test, Tester, tester.tc037@example.com, Customer service.
 Після кроку 6: у полі «Message» 50 символів (допустима довжина).
 Після кроку 7: відкрито вікно вибору файла.
@@ -3635,29 +3671,29 @@
       </c>
       <c r="G38" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">High</t>
+          <t>High</t>
         </is>
       </c>
       <c r="H38" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">позитивний</t>
+          <t>позитивний</t>
         </is>
       </c>
       <c r="I38" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Клас «допустимий файл»: один файл .txt розміром до 500 КБ (F-140); 1 КБ — типовий представник класу, значно нижче межі 500 КБ. Позитивна пара до TC-013 (недопустимий формат .png). Довжина повідомлення 50 і решта полів валідні, тож результат залежить лише від вкладення. Межі 500 і 501 КБ у цьому кейсі не перевіряються (один кейс — один набір даних). Це одне допустиме надсилання вигаданого звернення, не навантаження (етика demo, п. 1.7).</t>
+          <t>Клас «допустимий файл»: один файл .txt розміром до 500 КБ (F-140); 1 КБ — типовий представник класу, значно нижче межі 500 КБ. Позитивна пара до TC-013 (недопустимий формат .png). Довжина повідомлення 50 і решта полів валідні, тож результат залежить лише від вкладення. Межі 500 і 501 КБ у цьому кейсі не перевіряються (один кейс — один набір даних). Це одне допустиме надсилання вигаданого звернення, не навантаження (етика demo, п. 1.7).</t>
         </is>
       </c>
       <c r="J38" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Горбонос О. (КТ)</t>
+          <t>Горбонос О. (КТ)</t>
         </is>
       </c>
       <c r="K38" s="2" t="n"/>
       <c r="L38" s="2" t="n"/>
       <c r="M38" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">draft</t>
+          <t>draft</t>
         </is>
       </c>
       <c r="N38" s="2" t="n"/>

</xml_diff>

<commit_message>
SCRUM-118, SCRUM-119: Review TC-037 (reviewed);
TC-036 крок 3 — «TLS 1.3 або QUIC», draft
</commit_message>
<xml_diff>
--- a/docs/sprint3/test-cases.xlsx
+++ b/docs/sprint3/test-cases.xlsx
@@ -1,15 +1,15 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Test cases" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Coverage" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Review" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test cases" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Coverage" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Review" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Test cases'!$A$1:$N$45</definedName>
@@ -3574,7 +3574,7 @@
         <is>
           <t>Після кроку 1: відкрито головну сторінку з каталогом; адреса в адресному рядку починається з https://.
 Після кроку 2: відкрито DevTools.
-Після кроку 3: на вкладці «Security» — з'єднання захищене, у розділі «Connection» вказано протокол TLS 1.3 (S-10).
+Після кроку 3: на вкладці «Security» — з'єднання захищене; у розділі «Connection» вказано протокол TLS 1.3 або QUIC (QUIC працює лише поверх TLS 1.3, тож обидва значення відповідають S-10). Інша версія TLS (1.2 і нижче) — failed.
 Після кроку 4: вкладку закрито.
 Після кроку 5: відкрито вікно термінала.
 Після кроку 6: команду введено.
@@ -3594,7 +3594,7 @@
       </c>
       <c r="I37" s="2" t="inlineStr">
         <is>
-          <t>S-10 покривається частково — лише те, що можна спостерегти на публічному demo: перенаправлення HTTP → HTTPS і версія TLS. Хеш bcrypt, код 403 на чужі дані і сканування вразливостей на demo не перевіряються (інструкція, п. 1.7; S-10 — сканування лише на локальному стенді). Перенаправлення перевіряється curl, бо браузер сам переходить на https:// і не показує відповідь сервера (зауваження ІТ, 28.10.2026). Один запит curl і одне відкриття сторінки — не навантаження. API не перевіряється (один кейс — один набір даних).</t>
+          <t>S-10 покривається частково — лише те, що можна спостерегти на публічному demo: перенаправлення HTTP → HTTPS і версія TLS. Хеш bcrypt, код 403 на чужі дані і сканування вразливостей на demo не перевіряються (інструкція, п. 1.7; S-10 — сканування лише на локальному стенді). Перенаправлення перевіряється curl, бо браузер сам переходить на https:// і не показує відповідь сервера (зауваження ІТ, 28.10.2026). Один запит curl і одне відкриття сторінки — не навантаження. API не перевіряється (один кейс — один набір даних). Крок 3: Chrome 156 для з'єднання HTTP/3 показує в «Connection» протокол QUIC замість назви TLS 1.3; QUIC (RFC 9001) використовує лише TLS 1.3, тому QUIC приймається як TLS 1.3 (зауваження ІТ, 28.10.2026).</t>
         </is>
       </c>
       <c r="J37" s="2" t="inlineStr">
@@ -3602,19 +3602,11 @@
           <t>Дрєпіна А. (СМ)</t>
         </is>
       </c>
-      <c r="K37" s="2" t="inlineStr">
-        <is>
-          <t>Горбонос О. (КТ)</t>
-        </is>
-      </c>
-      <c r="L37" s="2" t="inlineStr">
-        <is>
-          <t>28.10.2026</t>
-        </is>
-      </c>
+      <c r="K37" s="2" t="n"/>
+      <c r="L37" s="2" t="n"/>
       <c r="M37" s="2" t="inlineStr">
         <is>
-          <t>reviewed</t>
+          <t>draft</t>
         </is>
       </c>
       <c r="N37" s="2" t="inlineStr">
@@ -3689,11 +3681,19 @@
           <t>Горбонос О. (КТ)</t>
         </is>
       </c>
-      <c r="K38" s="2" t="n"/>
-      <c r="L38" s="2" t="n"/>
+      <c r="K38" s="2" t="inlineStr">
+        <is>
+          <t>Дрєпіна А. (СМ)</t>
+        </is>
+      </c>
+      <c r="L38" s="2" t="inlineStr">
+        <is>
+          <t>28.10.2026</t>
+        </is>
+      </c>
       <c r="M38" s="2" t="inlineStr">
         <is>
-          <t>draft</t>
+          <t>reviewed</t>
         </is>
       </c>
       <c r="N38" s="2" t="n"/>
@@ -5157,7 +5157,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N39"/>
+  <dimension ref="A1:N40"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -7871,8 +7871,80 @@
         </is>
       </c>
     </row>
-    <row r="39">
-      <c r="A39" t="inlineStr">
+    <row r="38">
+      <c r="A38" s="2" t="inlineStr">
+        <is>
+          <t>TC-037</t>
+        </is>
+      </c>
+      <c r="B38" s="2" t="inlineStr">
+        <is>
+          <t>Дрєпіна А. (СМ)</t>
+        </is>
+      </c>
+      <c r="C38" s="2" t="inlineStr">
+        <is>
+          <t>28.10.2026</t>
+        </is>
+      </c>
+      <c r="D38" s="2" t="inlineStr">
+        <is>
+          <t>так</t>
+        </is>
+      </c>
+      <c r="E38" s="2" t="inlineStr">
+        <is>
+          <t>так</t>
+        </is>
+      </c>
+      <c r="F38" s="2" t="inlineStr">
+        <is>
+          <t>так</t>
+        </is>
+      </c>
+      <c r="G38" s="2" t="inlineStr">
+        <is>
+          <t>так</t>
+        </is>
+      </c>
+      <c r="H38" s="2" t="inlineStr">
+        <is>
+          <t>так</t>
+        </is>
+      </c>
+      <c r="I38" s="2" t="inlineStr">
+        <is>
+          <t>так</t>
+        </is>
+      </c>
+      <c r="J38" s="2" t="inlineStr">
+        <is>
+          <t>так</t>
+        </is>
+      </c>
+      <c r="K38" s="2" t="inlineStr">
+        <is>
+          <t>так</t>
+        </is>
+      </c>
+      <c r="L38" s="2" t="inlineStr">
+        <is>
+          <t>Зауважень немає: шість полів, вимога F-140, незалежний (відкрити → закрити вкладку), одна дія на крок, очікування перевірювані; позитивна пара до TC-013. Рекомендація, що не блокує: у передумовах указати точний розмір файла, як у #51 (1 020 байт), замість «близько 1000 символів».</t>
+        </is>
+      </c>
+      <c r="M38" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="N38" s="2" t="inlineStr">
+        <is>
+          <t>28.10.2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
         <is>
           <t>П1 шість полів, унікальний TC-NNN · П2 вимога з SRS 1.1, кейс перевіряє саме її · П3 незалежний (відкриття → вихід/закриття) · П4 передумови повні · П5 одна дія на крок, конкретні дані · П6 перевірювані очікувані результати · П7 заголовок і тип · П8 граничні значення / негативна пара</t>
         </is>
@@ -7880,10 +7952,10 @@
     </row>
   </sheetData>
   <dataValidations count="2">
-    <dataValidation sqref="D2:K37" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="D2:K38" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"так,ні"</formula1>
     </dataValidation>
-    <dataValidation sqref="M2:M37" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="M2:M38" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"так,ні,—"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
SCRUM-114: test-cases.xlsx — «Issue #»: TC-007 #65, TC-034 #63, #66
</commit_message>
<xml_diff>
--- a/docs/sprint3/test-cases.xlsx
+++ b/docs/sprint3/test-cases.xlsx
@@ -1,15 +1,15 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test cases" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Coverage" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Review" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Test cases" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Coverage" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Review" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Test cases'!$A$1:$N$45</definedName>
@@ -1161,7 +1161,11 @@
           <t>reviewed</t>
         </is>
       </c>
-      <c r="N8" s="2" t="n"/>
+      <c r="N8" s="2" t="inlineStr">
+        <is>
+          <t>#65</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
@@ -3453,7 +3457,7 @@
       </c>
       <c r="N35" s="2" t="inlineStr">
         <is>
-          <t>#63</t>
+          <t>#63, #66</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
SCRUM-114: test-cases.xlsx — «Issue #»: TC-019 #68, TC-031 #67, TC-037 #51
</commit_message>
<xml_diff>
--- a/docs/sprint3/test-cases.xlsx
+++ b/docs/sprint3/test-cases.xlsx
@@ -1,15 +1,15 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test cases" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Coverage" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Review" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Test cases" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Coverage" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Review" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Test cases'!$A$1:$N$45</definedName>
@@ -2173,7 +2173,11 @@
           <t>reviewed</t>
         </is>
       </c>
-      <c r="N20" s="2" t="n"/>
+      <c r="N20" s="2" t="inlineStr">
+        <is>
+          <t>#68</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
@@ -3185,7 +3189,11 @@
           <t>reviewed</t>
         </is>
       </c>
-      <c r="N32" s="2" t="n"/>
+      <c r="N32" s="2" t="inlineStr">
+        <is>
+          <t>#67</t>
+        </is>
+      </c>
     </row>
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
@@ -3700,7 +3708,11 @@
           <t>reviewed</t>
         </is>
       </c>
-      <c r="N38" s="2" t="n"/>
+      <c r="N38" s="2" t="inlineStr">
+        <is>
+          <t>#51</t>
+        </is>
+      </c>
     </row>
     <row r="39">
       <c r="A39" s="2" t="n"/>

</xml_diff>